<commit_message>
[feat/HD-15447] fix: fixed the formulation part
</commit_message>
<xml_diff>
--- a/api/templates/results_ntp_use/en.xlsx
+++ b/api/templates/results_ntp_use/en.xlsx
@@ -632,9 +632,6 @@
     <t>&lt;cnt_TypeOfPatient_Column_8_all_stool&gt;</t>
   </si>
   <si>
-    <t>#REF!&lt;cnt_TypeOfPatient_Column_8_Mtb_stool&gt;</t>
-  </si>
-  <si>
     <t>&lt;cnt_TypeOfPatient_Column_8_MtbRif_stool&gt;</t>
   </si>
   <si>
@@ -879,6 +876,9 @@
   </si>
   <si>
     <t>&lt;cnt_Xdr_Total_Tests_stool&gt;</t>
+  </si>
+  <si>
+    <t>&lt;cnt_TypeOfPatient_Column_8_Mtb_stool&gt;</t>
   </si>
 </sst>
 </file>
@@ -1258,47 +1258,43 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1307,40 +1303,44 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1686,7 +1686,7 @@
     </row>
     <row r="6" spans="1:150" s="4" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1705,7 +1705,7 @@
     </row>
     <row r="7" spans="1:150" s="4" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -1761,22 +1761,22 @@
       <c r="O9" s="5"/>
     </row>
     <row r="10" spans="1:150" s="8" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="49" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="50"/>
-      <c r="E10" s="48" t="s">
+      <c r="E10" s="51" t="s">
         <v>9</v>
       </c>
       <c r="F10" s="29"/>
       <c r="G10" s="30"/>
-      <c r="H10" s="42" t="s">
+      <c r="H10" s="52" t="s">
         <v>10</v>
       </c>
       <c r="I10" s="29"/>
@@ -1803,80 +1803,80 @@
       <c r="AD10" s="29"/>
       <c r="AE10" s="29"/>
       <c r="AF10" s="30"/>
-      <c r="AG10" s="42" t="s">
+      <c r="AG10" s="52" t="s">
         <v>11</v>
       </c>
       <c r="AH10" s="29"/>
       <c r="AI10" s="29"/>
       <c r="AJ10" s="30"/>
-      <c r="AK10" s="39" t="s">
+      <c r="AK10" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="AL10" s="39" t="s">
+      <c r="AL10" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="AM10" s="39" t="s">
+      <c r="AM10" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="AN10" s="28" t="s">
+      <c r="AN10" s="41" t="s">
         <v>15</v>
       </c>
       <c r="AO10" s="29"/>
       <c r="AP10" s="29"/>
       <c r="AQ10" s="30"/>
-      <c r="AR10" s="39" t="s">
+      <c r="AR10" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="AS10" s="28" t="s">
+      <c r="AS10" s="41" t="s">
         <v>17</v>
       </c>
       <c r="AT10" s="29"/>
       <c r="AU10" s="29"/>
       <c r="AV10" s="30"/>
-      <c r="AW10" s="25" t="s">
+      <c r="AW10" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="AX10" s="28" t="s">
+      <c r="AX10" s="41" t="s">
         <v>19</v>
       </c>
       <c r="AY10" s="29"/>
       <c r="AZ10" s="29"/>
       <c r="BA10" s="30"/>
-      <c r="BB10" s="25" t="s">
+      <c r="BB10" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="BC10" s="33" t="s">
+      <c r="BC10" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="BD10" s="34" t="s">
+      <c r="BD10" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="BE10" s="35"/>
-      <c r="BF10" s="36"/>
-      <c r="BG10" s="34" t="s">
+      <c r="BE10" s="32"/>
+      <c r="BF10" s="33"/>
+      <c r="BG10" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="BH10" s="35"/>
-      <c r="BI10" s="36"/>
-      <c r="BJ10" s="49" t="s">
+      <c r="BH10" s="32"/>
+      <c r="BI10" s="33"/>
+      <c r="BJ10" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="BK10" s="39" t="s">
+      <c r="BK10" s="42" t="s">
         <v>158</v>
       </c>
-      <c r="BL10" s="39" t="s">
+      <c r="BL10" s="42" t="s">
         <v>159</v>
       </c>
-      <c r="BM10" s="39" t="s">
+      <c r="BM10" s="42" t="s">
         <v>160</v>
       </c>
-      <c r="BN10" s="33" t="s">
+      <c r="BN10" s="40" t="s">
         <v>161</v>
       </c>
-      <c r="BO10" s="33" t="s">
+      <c r="BO10" s="40" t="s">
         <v>162</v>
       </c>
-      <c r="BP10" s="45" t="s">
+      <c r="BP10" s="48" t="s">
         <v>163</v>
       </c>
       <c r="BQ10" s="29"/>
@@ -1884,7 +1884,7 @@
       <c r="BS10" s="29"/>
       <c r="BT10" s="29"/>
       <c r="BU10" s="30"/>
-      <c r="BV10" s="45" t="s">
+      <c r="BV10" s="48" t="s">
         <v>167</v>
       </c>
       <c r="BW10" s="29"/>
@@ -1892,17 +1892,17 @@
       <c r="BY10" s="29"/>
       <c r="BZ10" s="29"/>
       <c r="CA10" s="30"/>
-      <c r="CB10" s="53" t="s">
+      <c r="CB10" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="CC10" s="35"/>
-      <c r="CD10" s="36"/>
-      <c r="CE10" s="45" t="s">
+      <c r="CC10" s="32"/>
+      <c r="CD10" s="33"/>
+      <c r="CE10" s="48" t="s">
         <v>168</v>
       </c>
       <c r="CF10" s="29"/>
       <c r="CG10" s="30"/>
-      <c r="CH10" s="45" t="s">
+      <c r="CH10" s="48" t="s">
         <v>172</v>
       </c>
       <c r="CI10" s="29"/>
@@ -1913,16 +1913,16 @@
       <c r="CN10" s="29"/>
       <c r="CO10" s="29"/>
       <c r="CP10" s="30"/>
-      <c r="CQ10" s="45" t="s">
+      <c r="CQ10" s="48" t="s">
         <v>26</v>
       </c>
       <c r="CR10" s="30"/>
-      <c r="CS10" s="48" t="s">
+      <c r="CS10" s="51" t="s">
         <v>9</v>
       </c>
       <c r="CT10" s="29"/>
       <c r="CU10" s="30"/>
-      <c r="CV10" s="42" t="s">
+      <c r="CV10" s="52" t="s">
         <v>10</v>
       </c>
       <c r="CW10" s="29"/>
@@ -1949,49 +1949,49 @@
       <c r="DR10" s="29"/>
       <c r="DS10" s="29"/>
       <c r="DT10" s="30"/>
-      <c r="DU10" s="42" t="s">
+      <c r="DU10" s="52" t="s">
         <v>11</v>
       </c>
       <c r="DV10" s="29"/>
       <c r="DW10" s="29"/>
       <c r="DX10" s="30"/>
-      <c r="DY10" s="39" t="s">
+      <c r="DY10" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="DZ10" s="39" t="s">
+      <c r="DZ10" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="EA10" s="39" t="s">
+      <c r="EA10" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="EB10" s="28" t="s">
+      <c r="EB10" s="41" t="s">
         <v>15</v>
       </c>
       <c r="EC10" s="29"/>
       <c r="ED10" s="29"/>
       <c r="EE10" s="30"/>
-      <c r="EF10" s="39" t="s">
+      <c r="EF10" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="EG10" s="28" t="s">
+      <c r="EG10" s="41" t="s">
         <v>17</v>
       </c>
       <c r="EH10" s="29"/>
       <c r="EI10" s="29"/>
       <c r="EJ10" s="30"/>
-      <c r="EK10" s="25" t="s">
+      <c r="EK10" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="EL10" s="28" t="s">
+      <c r="EL10" s="41" t="s">
         <v>19</v>
       </c>
       <c r="EM10" s="29"/>
       <c r="EN10" s="29"/>
       <c r="EO10" s="30"/>
-      <c r="EP10" s="25" t="s">
+      <c r="EP10" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="EQ10" s="28" t="s">
+      <c r="EQ10" s="41" t="s">
         <v>26</v>
       </c>
       <c r="ER10" s="29"/>
@@ -2011,71 +2011,71 @@
       <c r="F11" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="41" t="s">
+      <c r="G11" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="47" t="s">
+      <c r="H11" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="I11" s="41" t="s">
+      <c r="I11" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="J11" s="41" t="s">
+      <c r="J11" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="41" t="s">
+      <c r="K11" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="41" t="s">
+      <c r="L11" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="M11" s="41" t="s">
+      <c r="M11" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="N11" s="41" t="s">
+      <c r="N11" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="O11" s="41" t="s">
+      <c r="O11" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="P11" s="40" t="s">
+      <c r="P11" s="28" t="s">
         <v>39</v>
       </c>
       <c r="Q11" s="29"/>
       <c r="R11" s="30"/>
-      <c r="S11" s="40" t="s">
+      <c r="S11" s="28" t="s">
         <v>40</v>
       </c>
       <c r="T11" s="29"/>
       <c r="U11" s="30"/>
-      <c r="V11" s="40" t="s">
+      <c r="V11" s="28" t="s">
         <v>41</v>
       </c>
       <c r="W11" s="29"/>
       <c r="X11" s="30"/>
-      <c r="Y11" s="40" t="s">
+      <c r="Y11" s="28" t="s">
         <v>42</v>
       </c>
       <c r="Z11" s="29"/>
       <c r="AA11" s="30"/>
-      <c r="AB11" s="40" t="s">
+      <c r="AB11" s="28" t="s">
         <v>43</v>
       </c>
       <c r="AC11" s="29"/>
       <c r="AD11" s="30"/>
-      <c r="AE11" s="41" t="s">
+      <c r="AE11" s="45" t="s">
         <v>44</v>
       </c>
       <c r="AF11" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="AG11" s="41" t="s">
+      <c r="AG11" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="AH11" s="41" t="s">
+      <c r="AH11" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="AI11" s="41" t="s">
+      <c r="AI11" s="45" t="s">
         <v>45</v>
       </c>
       <c r="AJ11" s="46" t="s">
@@ -2084,125 +2084,125 @@
       <c r="AK11" s="23"/>
       <c r="AL11" s="23"/>
       <c r="AM11" s="23"/>
-      <c r="AN11" s="39" t="s">
+      <c r="AN11" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="AO11" s="39" t="s">
+      <c r="AO11" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="AP11" s="39" t="s">
+      <c r="AP11" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="AQ11" s="32" t="s">
+      <c r="AQ11" s="55" t="s">
         <v>49</v>
       </c>
       <c r="AR11" s="23"/>
-      <c r="AS11" s="39" t="s">
+      <c r="AS11" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="AT11" s="39" t="s">
+      <c r="AT11" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="AU11" s="39" t="s">
+      <c r="AU11" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="AV11" s="32" t="s">
+      <c r="AV11" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="AW11" s="26"/>
-      <c r="AX11" s="31" t="s">
+      <c r="AW11" s="36"/>
+      <c r="AX11" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="AY11" s="31" t="s">
+      <c r="AY11" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="AZ11" s="31" t="s">
+      <c r="AZ11" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="BA11" s="32" t="s">
+      <c r="BA11" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="BB11" s="26"/>
+      <c r="BB11" s="36"/>
       <c r="BC11" s="23"/>
       <c r="BD11" s="37"/>
       <c r="BE11" s="38"/>
-      <c r="BF11" s="27"/>
+      <c r="BF11" s="39"/>
       <c r="BG11" s="37"/>
       <c r="BH11" s="38"/>
-      <c r="BI11" s="27"/>
+      <c r="BI11" s="39"/>
       <c r="BJ11" s="23"/>
       <c r="BK11" s="23"/>
       <c r="BL11" s="23"/>
       <c r="BM11" s="23"/>
       <c r="BN11" s="23"/>
       <c r="BO11" s="23"/>
-      <c r="BP11" s="45" t="s">
+      <c r="BP11" s="48" t="s">
         <v>164</v>
       </c>
       <c r="BQ11" s="30"/>
-      <c r="BR11" s="45" t="s">
+      <c r="BR11" s="48" t="s">
         <v>165</v>
       </c>
       <c r="BS11" s="30"/>
-      <c r="BT11" s="45" t="s">
+      <c r="BT11" s="48" t="s">
         <v>166</v>
       </c>
       <c r="BU11" s="30"/>
-      <c r="BV11" s="45" t="s">
+      <c r="BV11" s="48" t="s">
         <v>164</v>
       </c>
       <c r="BW11" s="30"/>
-      <c r="BX11" s="45" t="s">
+      <c r="BX11" s="48" t="s">
         <v>165</v>
       </c>
       <c r="BY11" s="30"/>
-      <c r="BZ11" s="45" t="s">
+      <c r="BZ11" s="48" t="s">
         <v>166</v>
       </c>
       <c r="CA11" s="30"/>
-      <c r="CB11" s="54"/>
-      <c r="CC11" s="55"/>
-      <c r="CD11" s="26"/>
-      <c r="CE11" s="33" t="s">
+      <c r="CB11" s="34"/>
+      <c r="CC11" s="35"/>
+      <c r="CD11" s="36"/>
+      <c r="CE11" s="40" t="s">
         <v>169</v>
       </c>
-      <c r="CF11" s="33" t="s">
+      <c r="CF11" s="40" t="s">
         <v>170</v>
       </c>
-      <c r="CG11" s="33" t="s">
+      <c r="CG11" s="40" t="s">
         <v>171</v>
       </c>
-      <c r="CH11" s="33" t="s">
+      <c r="CH11" s="40" t="s">
         <v>173</v>
       </c>
-      <c r="CI11" s="33" t="s">
+      <c r="CI11" s="40" t="s">
         <v>174</v>
       </c>
-      <c r="CJ11" s="33" t="s">
+      <c r="CJ11" s="40" t="s">
         <v>175</v>
       </c>
-      <c r="CK11" s="33" t="s">
+      <c r="CK11" s="40" t="s">
         <v>176</v>
       </c>
-      <c r="CL11" s="33" t="s">
+      <c r="CL11" s="40" t="s">
         <v>177</v>
       </c>
-      <c r="CM11" s="33" t="s">
+      <c r="CM11" s="40" t="s">
         <v>178</v>
       </c>
-      <c r="CN11" s="33" t="s">
+      <c r="CN11" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="CO11" s="33" t="s">
+      <c r="CO11" s="40" t="s">
         <v>180</v>
       </c>
-      <c r="CP11" s="33" t="s">
+      <c r="CP11" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="CQ11" s="33" t="s">
+      <c r="CQ11" s="40" t="s">
         <v>50</v>
       </c>
-      <c r="CR11" s="33" t="s">
+      <c r="CR11" s="40" t="s">
         <v>51</v>
       </c>
       <c r="CS11" s="43" t="s">
@@ -2211,71 +2211,71 @@
       <c r="CT11" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="CU11" s="41" t="s">
+      <c r="CU11" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="CV11" s="47" t="s">
+      <c r="CV11" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="CW11" s="41" t="s">
+      <c r="CW11" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="CX11" s="41" t="s">
+      <c r="CX11" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="CY11" s="41" t="s">
+      <c r="CY11" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="CZ11" s="41" t="s">
+      <c r="CZ11" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="DA11" s="41" t="s">
+      <c r="DA11" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="DB11" s="41" t="s">
+      <c r="DB11" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="DC11" s="41" t="s">
+      <c r="DC11" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="DD11" s="40" t="s">
+      <c r="DD11" s="28" t="s">
         <v>39</v>
       </c>
       <c r="DE11" s="29"/>
       <c r="DF11" s="30"/>
-      <c r="DG11" s="40" t="s">
+      <c r="DG11" s="28" t="s">
         <v>40</v>
       </c>
       <c r="DH11" s="29"/>
       <c r="DI11" s="30"/>
-      <c r="DJ11" s="40" t="s">
+      <c r="DJ11" s="28" t="s">
         <v>41</v>
       </c>
       <c r="DK11" s="29"/>
       <c r="DL11" s="30"/>
-      <c r="DM11" s="40" t="s">
+      <c r="DM11" s="28" t="s">
         <v>42</v>
       </c>
       <c r="DN11" s="29"/>
       <c r="DO11" s="30"/>
-      <c r="DP11" s="40" t="s">
+      <c r="DP11" s="28" t="s">
         <v>43</v>
       </c>
       <c r="DQ11" s="29"/>
       <c r="DR11" s="30"/>
-      <c r="DS11" s="41" t="s">
+      <c r="DS11" s="45" t="s">
         <v>44</v>
       </c>
       <c r="DT11" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="DU11" s="41" t="s">
+      <c r="DU11" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="DV11" s="41" t="s">
+      <c r="DV11" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="DW11" s="41" t="s">
+      <c r="DW11" s="45" t="s">
         <v>45</v>
       </c>
       <c r="DX11" s="46" t="s">
@@ -2284,55 +2284,55 @@
       <c r="DY11" s="23"/>
       <c r="DZ11" s="23"/>
       <c r="EA11" s="23"/>
-      <c r="EB11" s="39" t="s">
+      <c r="EB11" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="EC11" s="39" t="s">
+      <c r="EC11" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="ED11" s="39" t="s">
+      <c r="ED11" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="EE11" s="32" t="s">
+      <c r="EE11" s="55" t="s">
         <v>49</v>
       </c>
       <c r="EF11" s="23"/>
-      <c r="EG11" s="39" t="s">
+      <c r="EG11" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="EH11" s="39" t="s">
+      <c r="EH11" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="EI11" s="39" t="s">
+      <c r="EI11" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="EJ11" s="32" t="s">
+      <c r="EJ11" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="EK11" s="26"/>
-      <c r="EL11" s="31" t="s">
+      <c r="EK11" s="36"/>
+      <c r="EL11" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="EM11" s="31" t="s">
+      <c r="EM11" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="EN11" s="31" t="s">
+      <c r="EN11" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="EO11" s="32" t="s">
+      <c r="EO11" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="EP11" s="26"/>
-      <c r="EQ11" s="39" t="s">
+      <c r="EP11" s="36"/>
+      <c r="EQ11" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="ER11" s="39" t="s">
+      <c r="ER11" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="ES11" s="39" t="s">
+      <c r="ES11" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="ET11" s="33" t="s">
+      <c r="ET11" s="40" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2415,12 +2415,12 @@
       <c r="AT12" s="24"/>
       <c r="AU12" s="24"/>
       <c r="AV12" s="24"/>
-      <c r="AW12" s="27"/>
+      <c r="AW12" s="39"/>
       <c r="AX12" s="24"/>
       <c r="AY12" s="24"/>
       <c r="AZ12" s="24"/>
       <c r="BA12" s="24"/>
-      <c r="BB12" s="27"/>
+      <c r="BB12" s="39"/>
       <c r="BC12" s="24"/>
       <c r="BD12" s="12" t="s">
         <v>55</v>
@@ -2484,7 +2484,7 @@
       </c>
       <c r="CB12" s="37"/>
       <c r="CC12" s="38"/>
-      <c r="CD12" s="27"/>
+      <c r="CD12" s="39"/>
       <c r="CE12" s="24"/>
       <c r="CF12" s="24"/>
       <c r="CG12" s="24"/>
@@ -2573,25 +2573,25 @@
       <c r="EH12" s="24"/>
       <c r="EI12" s="24"/>
       <c r="EJ12" s="24"/>
-      <c r="EK12" s="27"/>
+      <c r="EK12" s="39"/>
       <c r="EL12" s="24"/>
       <c r="EM12" s="24"/>
       <c r="EN12" s="24"/>
       <c r="EO12" s="24"/>
-      <c r="EP12" s="27"/>
+      <c r="EP12" s="39"/>
       <c r="EQ12" s="24"/>
       <c r="ER12" s="24"/>
       <c r="ES12" s="24"/>
       <c r="ET12" s="24"/>
     </row>
     <row r="13" spans="1:150" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="56" t="s">
+      <c r="A13" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="56" t="s">
-        <v>263</v>
-      </c>
-      <c r="C13" s="56" t="s">
+      <c r="B13" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="C13" s="22" t="s">
         <v>60</v>
       </c>
       <c r="D13" s="16" t="s">
@@ -2653,7 +2653,7 @@
         <v>112</v>
       </c>
       <c r="W13" s="18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="X13" s="18" t="s">
         <v>117</v>
@@ -2695,73 +2695,73 @@
         <f>SUM(AG13:AI13)</f>
         <v>0</v>
       </c>
-      <c r="AK13" s="51">
+      <c r="AK13" s="25">
         <f>G13+AJ13</f>
         <v>0</v>
       </c>
-      <c r="AL13" s="51">
+      <c r="AL13" s="25">
         <f>AF13</f>
         <v>0</v>
       </c>
-      <c r="AM13" s="51">
+      <c r="AM13" s="25">
         <f>AK13+AL13</f>
         <v>0</v>
       </c>
-      <c r="AN13" s="51">
+      <c r="AN13" s="25">
         <f>G14+AJ14-G15-AJ15</f>
         <v>0</v>
       </c>
-      <c r="AO13" s="51">
+      <c r="AO13" s="25">
         <f>G15+AJ15</f>
         <v>0</v>
       </c>
-      <c r="AP13" s="51" t="s">
+      <c r="AP13" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="AQ13" s="51">
+      <c r="AQ13" s="25">
         <f>AE15</f>
         <v>0</v>
       </c>
-      <c r="AR13" s="51">
+      <c r="AR13" s="25">
         <f>AK13-G14-AJ14</f>
         <v>0</v>
       </c>
-      <c r="AS13" s="51">
+      <c r="AS13" s="25">
         <f>+AF14-AF15</f>
         <v>0</v>
       </c>
-      <c r="AT13" s="51">
+      <c r="AT13" s="25">
         <f>AF15</f>
         <v>0</v>
       </c>
-      <c r="AU13" s="51" t="s">
+      <c r="AU13" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="AV13" s="51">
+      <c r="AV13" s="25">
         <f>AF15</f>
         <v>0</v>
       </c>
-      <c r="AW13" s="51">
+      <c r="AW13" s="25">
         <f>AL13-AF14</f>
         <v>0</v>
       </c>
-      <c r="AX13" s="51">
+      <c r="AX13" s="25">
         <f>AN13+AS13</f>
         <v>0</v>
       </c>
-      <c r="AY13" s="51">
+      <c r="AY13" s="25">
         <f>AO13+AT13</f>
         <v>0</v>
       </c>
-      <c r="AZ13" s="51" t="e">
+      <c r="AZ13" s="25" t="e">
         <f>AP13+AU13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA13" s="51">
+      <c r="BA13" s="25">
         <f>AQ13+AV13</f>
         <v>0</v>
       </c>
-      <c r="BB13" s="51">
+      <c r="BB13" s="25">
         <f>AR13+AW13</f>
         <v>0</v>
       </c>
@@ -2789,82 +2789,82 @@
       <c r="BJ13" s="15" t="e">
         <v>#REF!</v>
       </c>
-      <c r="BK13" s="52" t="e">
+      <c r="BK13" s="27" t="e">
         <v>#REF!</v>
       </c>
-      <c r="BL13" s="52" t="e">
+      <c r="BL13" s="27" t="e">
         <v>#REF!</v>
       </c>
-      <c r="BM13" s="57" t="e">
+      <c r="BM13" s="26" t="e">
         <v>#REF!</v>
       </c>
-      <c r="BN13" s="51"/>
-      <c r="BO13" s="51"/>
-      <c r="BP13" s="51" t="s">
+      <c r="BN13" s="25"/>
+      <c r="BO13" s="25"/>
+      <c r="BP13" s="25" t="s">
+        <v>266</v>
+      </c>
+      <c r="BQ13" s="25" t="s">
         <v>267</v>
       </c>
-      <c r="BQ13" s="51" t="s">
+      <c r="BR13" s="25" t="s">
         <v>268</v>
       </c>
-      <c r="BR13" s="51" t="s">
+      <c r="BS13" s="25" t="s">
         <v>269</v>
       </c>
-      <c r="BS13" s="51" t="s">
+      <c r="BT13" s="25" t="s">
         <v>270</v>
       </c>
-      <c r="BT13" s="51" t="s">
+      <c r="BU13" s="25" t="s">
         <v>271</v>
       </c>
-      <c r="BU13" s="51" t="s">
+      <c r="BV13" s="25" t="s">
         <v>272</v>
       </c>
-      <c r="BV13" s="51" t="s">
+      <c r="BW13" s="25" t="s">
         <v>273</v>
       </c>
-      <c r="BW13" s="51" t="s">
+      <c r="BX13" s="25" t="s">
         <v>274</v>
       </c>
-      <c r="BX13" s="51" t="s">
+      <c r="BY13" s="25" t="s">
         <v>275</v>
       </c>
-      <c r="BY13" s="51" t="s">
+      <c r="BZ13" s="25" t="s">
         <v>276</v>
       </c>
-      <c r="BZ13" s="51" t="s">
+      <c r="CA13" s="25" t="s">
         <v>277</v>
       </c>
-      <c r="CA13" s="51" t="s">
+      <c r="CB13" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="CB13" s="51" t="s">
+      <c r="CC13" s="25" t="s">
         <v>279</v>
       </c>
-      <c r="CC13" s="51" t="s">
+      <c r="CD13" s="25" t="s">
         <v>280</v>
       </c>
-      <c r="CD13" s="51" t="s">
+      <c r="CE13" s="25" t="s">
         <v>281</v>
       </c>
-      <c r="CE13" s="51" t="s">
+      <c r="CF13" s="25" t="s">
         <v>282</v>
       </c>
-      <c r="CF13" s="51" t="s">
+      <c r="CG13" s="25" t="s">
         <v>283</v>
       </c>
-      <c r="CG13" s="51" t="s">
-        <v>284</v>
-      </c>
-      <c r="CH13" s="51"/>
-      <c r="CI13" s="51"/>
-      <c r="CJ13" s="51"/>
-      <c r="CK13" s="51"/>
-      <c r="CL13" s="51"/>
-      <c r="CM13" s="51"/>
-      <c r="CN13" s="51"/>
-      <c r="CO13" s="51"/>
-      <c r="CP13" s="51"/>
-      <c r="CQ13" s="52"/>
-      <c r="CR13" s="52"/>
+      <c r="CH13" s="25"/>
+      <c r="CI13" s="25"/>
+      <c r="CJ13" s="25"/>
+      <c r="CK13" s="25"/>
+      <c r="CL13" s="25"/>
+      <c r="CM13" s="25"/>
+      <c r="CN13" s="25"/>
+      <c r="CO13" s="25"/>
+      <c r="CP13" s="25"/>
+      <c r="CQ13" s="27"/>
+      <c r="CR13" s="27"/>
       <c r="CS13" s="17" t="s">
         <v>182</v>
       </c>
@@ -2894,52 +2894,52 @@
         <v>204</v>
       </c>
       <c r="DB13" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="DC13" s="17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="DD13" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="DE13" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="DE13" s="18" t="s">
-        <v>214</v>
-      </c>
       <c r="DF13" s="18" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="DG13" s="18" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="DH13" s="18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="DI13" s="18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="DJ13" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="DK13" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="DL13" s="18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="DM13" s="18" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="DN13" s="18" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="DO13" s="18" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="DP13" s="18" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="DQ13" s="18" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="DR13" s="18"/>
       <c r="DS13" s="19">
@@ -2951,97 +2951,97 @@
         <v>0</v>
       </c>
       <c r="DU13" s="19" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="DV13" s="19" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="DW13" s="19" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="DX13" s="19">
         <f>SUM(DU13:DW13)</f>
         <v>0</v>
       </c>
-      <c r="DY13" s="51">
+      <c r="DY13" s="25">
         <f>SUM(CU13:DX13)</f>
         <v>0</v>
       </c>
-      <c r="DZ13" s="51">
+      <c r="DZ13" s="25">
         <f>DT13</f>
         <v>0</v>
       </c>
-      <c r="EA13" s="51">
+      <c r="EA13" s="25">
         <f>DY13+DZ13</f>
         <v>0</v>
       </c>
-      <c r="EB13" s="51">
+      <c r="EB13" s="25">
         <f>CU14+DT14-CU15-DT15</f>
         <v>0</v>
       </c>
-      <c r="EC13" s="51">
+      <c r="EC13" s="25">
         <f>CU15+DT15</f>
         <v>0</v>
       </c>
-      <c r="ED13" s="51" t="s">
+      <c r="ED13" s="25" t="s">
+        <v>284</v>
+      </c>
+      <c r="EE13" s="25">
+        <f>DS15</f>
+        <v>0</v>
+      </c>
+      <c r="EF13" s="25">
+        <f>DY13-DX14-CU14</f>
+        <v>0</v>
+      </c>
+      <c r="EG13" s="25">
+        <f>+DT14-DT15</f>
+        <v>0</v>
+      </c>
+      <c r="EH13" s="25">
+        <f>DT15</f>
+        <v>0</v>
+      </c>
+      <c r="EI13" s="25" t="s">
         <v>285</v>
       </c>
-      <c r="EE13" s="51">
-        <f>DS15</f>
-        <v>0</v>
-      </c>
-      <c r="EF13" s="51">
-        <f>DY13-DX14-CU14</f>
-        <v>0</v>
-      </c>
-      <c r="EG13" s="51">
-        <f>+DT14-DT15</f>
-        <v>0</v>
-      </c>
-      <c r="EH13" s="51">
+      <c r="EJ13" s="25">
         <f>DT15</f>
         <v>0</v>
       </c>
-      <c r="EI13" s="51" t="s">
-        <v>286</v>
-      </c>
-      <c r="EJ13" s="51">
-        <f>DT15</f>
-        <v>0</v>
-      </c>
-      <c r="EK13" s="51">
+      <c r="EK13" s="25">
         <f>DZ13-DT14</f>
         <v>0</v>
       </c>
-      <c r="EL13" s="51">
+      <c r="EL13" s="25">
         <f>EB13+EG13</f>
         <v>0</v>
       </c>
-      <c r="EM13" s="51">
+      <c r="EM13" s="25">
         <f>EC13-EH13</f>
         <v>0</v>
       </c>
-      <c r="EN13" s="51" t="e">
+      <c r="EN13" s="25" t="e">
         <f>ED13+EI13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="EO13" s="51">
+      <c r="EO13" s="25">
         <f>EE13+EJ13</f>
         <v>0</v>
       </c>
-      <c r="EP13" s="51">
+      <c r="EP13" s="25">
         <f>EF13+EK13</f>
         <v>0</v>
       </c>
-      <c r="EQ13" s="52">
+      <c r="EQ13" s="27">
         <f>EG13+EM13</f>
         <v>0</v>
       </c>
-      <c r="ER13" s="52"/>
-      <c r="ES13" s="52" t="s">
-        <v>287</v>
-      </c>
-      <c r="ET13" s="51" t="str">
+      <c r="ER13" s="27"/>
+      <c r="ES13" s="27" t="s">
+        <v>286</v>
+      </c>
+      <c r="ET13" s="25" t="str">
         <f>ES13</f>
         <v>&lt;cnt_Xdr_Total_Tests_stool&gt;</v>
       </c>
@@ -3070,7 +3070,7 @@
         <v>76</v>
       </c>
       <c r="J14" s="21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="K14" s="21" t="s">
         <v>81</v>
@@ -3253,55 +3253,55 @@
         <v>202</v>
       </c>
       <c r="DA14" s="16" t="s">
-        <v>205</v>
+        <v>287</v>
       </c>
       <c r="DB14" s="16" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="DC14" s="16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="DD14" s="18" t="s">
         <v>183</v>
       </c>
       <c r="DE14" s="18" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="DF14" s="18" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="DG14" s="18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="DH14" s="18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="DI14" s="18" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="DJ14" s="18" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="DK14" s="18" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="DL14" s="18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="DM14" s="18" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="DN14" s="18" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="DO14" s="18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="DP14" s="18" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="DQ14" s="18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="DR14" s="18"/>
       <c r="DS14" s="19">
@@ -3313,13 +3313,13 @@
         <v>0</v>
       </c>
       <c r="DU14" s="19" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="DV14" s="19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="DW14" s="19" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="DX14" s="19">
         <f>SUM(DU14:DW14)</f>
@@ -3539,55 +3539,55 @@
         <v>203</v>
       </c>
       <c r="DA15" s="16" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="DB15" s="16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="DC15" s="16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="DD15" s="18" t="s">
         <v>183</v>
       </c>
       <c r="DE15" s="18" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="DF15" s="18" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="DG15" s="18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="DH15" s="18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="DI15" s="18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="DJ15" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="DK15" s="18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="DL15" s="18" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="DM15" s="18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="DN15" s="18" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="DO15" s="18" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="DP15" s="18" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="DQ15" s="18" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="DR15" s="18"/>
       <c r="DS15" s="19">
@@ -3599,13 +3599,13 @@
         <v>0</v>
       </c>
       <c r="DU15" s="19" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="DV15" s="19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="DW15" s="19" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="DX15" s="19">
         <f>SUM(DU15:DW15)</f>
@@ -3640,6 +3640,195 @@
     </row>
   </sheetData>
   <mergeCells count="213">
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="EP10:EP12"/>
+    <mergeCell ref="EL10:EO10"/>
+    <mergeCell ref="EL11:EL12"/>
+    <mergeCell ref="EM11:EM12"/>
+    <mergeCell ref="EN11:EN12"/>
+    <mergeCell ref="EO11:EO12"/>
+    <mergeCell ref="AW10:AW12"/>
+    <mergeCell ref="AZ11:AZ12"/>
+    <mergeCell ref="BA11:BA12"/>
+    <mergeCell ref="AX10:BA10"/>
+    <mergeCell ref="BB10:BB12"/>
+    <mergeCell ref="BC10:BC12"/>
+    <mergeCell ref="BD10:BF11"/>
+    <mergeCell ref="BG10:BI11"/>
+    <mergeCell ref="EJ11:EJ12"/>
+    <mergeCell ref="DZ10:DZ12"/>
+    <mergeCell ref="EA10:EA12"/>
+    <mergeCell ref="EB10:EE10"/>
+    <mergeCell ref="EF10:EF12"/>
+    <mergeCell ref="EG10:EJ10"/>
+    <mergeCell ref="EK10:EK12"/>
+    <mergeCell ref="DP11:DR11"/>
+    <mergeCell ref="DS11:DS12"/>
+    <mergeCell ref="CL11:CL12"/>
+    <mergeCell ref="CM11:CM12"/>
+    <mergeCell ref="CN11:CN12"/>
+    <mergeCell ref="DY10:DY12"/>
+    <mergeCell ref="ED11:ED12"/>
+    <mergeCell ref="EE11:EE12"/>
+    <mergeCell ref="EG11:EG12"/>
+    <mergeCell ref="EH11:EH12"/>
+    <mergeCell ref="DU10:DX10"/>
+    <mergeCell ref="CO11:CO12"/>
+    <mergeCell ref="CP11:CP12"/>
+    <mergeCell ref="CQ11:CQ12"/>
+    <mergeCell ref="CR11:CR12"/>
+    <mergeCell ref="CS11:CS12"/>
+    <mergeCell ref="CT11:CT12"/>
+    <mergeCell ref="DB11:DB12"/>
+    <mergeCell ref="DC11:DC12"/>
+    <mergeCell ref="DD11:DF11"/>
+    <mergeCell ref="DG11:DI11"/>
+    <mergeCell ref="DJ11:DL11"/>
+    <mergeCell ref="EI11:EI12"/>
+    <mergeCell ref="BK10:BK12"/>
+    <mergeCell ref="BT11:BU11"/>
+    <mergeCell ref="BV11:BW11"/>
+    <mergeCell ref="BX11:BY11"/>
+    <mergeCell ref="BZ11:CA11"/>
+    <mergeCell ref="BL10:BL12"/>
+    <mergeCell ref="BM10:BM12"/>
+    <mergeCell ref="BN10:BN12"/>
+    <mergeCell ref="BO10:BO12"/>
+    <mergeCell ref="BP10:BU10"/>
+    <mergeCell ref="BV10:CA10"/>
+    <mergeCell ref="DT11:DT12"/>
+    <mergeCell ref="CU11:CU12"/>
+    <mergeCell ref="CV11:CV12"/>
+    <mergeCell ref="DU11:DU12"/>
+    <mergeCell ref="DV11:DV12"/>
+    <mergeCell ref="DW11:DW12"/>
+    <mergeCell ref="DX11:DX12"/>
+    <mergeCell ref="CE10:CG10"/>
+    <mergeCell ref="CH10:CP10"/>
+    <mergeCell ref="CQ10:CR10"/>
+    <mergeCell ref="CS10:CU10"/>
+    <mergeCell ref="CV10:DT10"/>
+    <mergeCell ref="BJ10:BJ12"/>
+    <mergeCell ref="AP11:AP12"/>
+    <mergeCell ref="AQ11:AQ12"/>
+    <mergeCell ref="AS11:AS12"/>
+    <mergeCell ref="AT11:AT12"/>
+    <mergeCell ref="AU11:AU12"/>
+    <mergeCell ref="AV11:AV12"/>
+    <mergeCell ref="AK10:AK12"/>
+    <mergeCell ref="AL10:AL12"/>
+    <mergeCell ref="AM10:AM12"/>
+    <mergeCell ref="AN10:AQ10"/>
+    <mergeCell ref="AR10:AR12"/>
+    <mergeCell ref="AS10:AV10"/>
+    <mergeCell ref="AO11:AO12"/>
+    <mergeCell ref="AF11:AF12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:AF10"/>
+    <mergeCell ref="AG10:AJ10"/>
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="V11:X11"/>
+    <mergeCell ref="Y11:AA11"/>
+    <mergeCell ref="AB11:AD11"/>
+    <mergeCell ref="AE11:AE12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="EQ10:ES10"/>
+    <mergeCell ref="EQ11:EQ12"/>
+    <mergeCell ref="ER11:ER12"/>
+    <mergeCell ref="ES11:ES12"/>
+    <mergeCell ref="ET11:ET12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="AH11:AH12"/>
+    <mergeCell ref="AI11:AI12"/>
+    <mergeCell ref="AJ11:AJ12"/>
+    <mergeCell ref="AX11:AX12"/>
+    <mergeCell ref="AY11:AY12"/>
+    <mergeCell ref="BP11:BQ11"/>
+    <mergeCell ref="BR11:BS11"/>
+    <mergeCell ref="CE11:CE12"/>
+    <mergeCell ref="CF11:CF12"/>
+    <mergeCell ref="CW11:CW12"/>
+    <mergeCell ref="CX11:CX12"/>
+    <mergeCell ref="CY11:CY12"/>
+    <mergeCell ref="CZ11:CZ12"/>
+    <mergeCell ref="DA11:DA12"/>
+    <mergeCell ref="EB11:EB12"/>
+    <mergeCell ref="EC11:EC12"/>
+    <mergeCell ref="CB13:CB15"/>
+    <mergeCell ref="CC13:CC15"/>
+    <mergeCell ref="CD13:CD15"/>
+    <mergeCell ref="CE13:CE15"/>
+    <mergeCell ref="CF13:CF15"/>
+    <mergeCell ref="CN13:CN15"/>
+    <mergeCell ref="DM11:DO11"/>
+    <mergeCell ref="CO13:CO15"/>
+    <mergeCell ref="CP13:CP15"/>
+    <mergeCell ref="CQ13:CQ15"/>
+    <mergeCell ref="CR13:CR15"/>
+    <mergeCell ref="CG13:CG15"/>
+    <mergeCell ref="CH13:CH15"/>
+    <mergeCell ref="CI13:CI15"/>
+    <mergeCell ref="CJ13:CJ15"/>
+    <mergeCell ref="CK13:CK15"/>
+    <mergeCell ref="CL13:CL15"/>
+    <mergeCell ref="CM13:CM15"/>
+    <mergeCell ref="CB10:CD12"/>
+    <mergeCell ref="CG11:CG12"/>
+    <mergeCell ref="CH11:CH12"/>
+    <mergeCell ref="CI11:CI12"/>
+    <mergeCell ref="CJ11:CJ12"/>
+    <mergeCell ref="CK11:CK12"/>
+    <mergeCell ref="EI13:EI15"/>
+    <mergeCell ref="EJ13:EJ15"/>
+    <mergeCell ref="ER13:ER15"/>
+    <mergeCell ref="ES13:ES15"/>
+    <mergeCell ref="ET13:ET15"/>
+    <mergeCell ref="EK13:EK15"/>
+    <mergeCell ref="EL13:EL15"/>
+    <mergeCell ref="EM13:EM15"/>
+    <mergeCell ref="EN13:EN15"/>
+    <mergeCell ref="EO13:EO15"/>
+    <mergeCell ref="EP13:EP15"/>
+    <mergeCell ref="EQ13:EQ15"/>
+    <mergeCell ref="EE13:EE15"/>
+    <mergeCell ref="EF13:EF15"/>
+    <mergeCell ref="AK13:AK15"/>
+    <mergeCell ref="AL13:AL15"/>
+    <mergeCell ref="AM13:AM15"/>
+    <mergeCell ref="AN13:AN15"/>
+    <mergeCell ref="AO13:AO15"/>
+    <mergeCell ref="EG13:EG15"/>
+    <mergeCell ref="EH13:EH15"/>
+    <mergeCell ref="AP13:AP15"/>
+    <mergeCell ref="AQ13:AQ15"/>
+    <mergeCell ref="AR13:AR15"/>
+    <mergeCell ref="AS13:AS15"/>
+    <mergeCell ref="AT13:AT15"/>
+    <mergeCell ref="AU13:AU15"/>
+    <mergeCell ref="AV13:AV15"/>
+    <mergeCell ref="AW13:AW15"/>
+    <mergeCell ref="AX13:AX15"/>
+    <mergeCell ref="AY13:AY15"/>
+    <mergeCell ref="AZ13:AZ15"/>
+    <mergeCell ref="BA13:BA15"/>
+    <mergeCell ref="BB13:BB15"/>
+    <mergeCell ref="BK13:BK15"/>
+    <mergeCell ref="BL13:BL15"/>
     <mergeCell ref="A13:A15"/>
     <mergeCell ref="B13:B15"/>
     <mergeCell ref="C13:C15"/>
@@ -3664,195 +3853,6 @@
     <mergeCell ref="BY13:BY15"/>
     <mergeCell ref="BZ13:BZ15"/>
     <mergeCell ref="CA13:CA15"/>
-    <mergeCell ref="EE13:EE15"/>
-    <mergeCell ref="EF13:EF15"/>
-    <mergeCell ref="AK13:AK15"/>
-    <mergeCell ref="AL13:AL15"/>
-    <mergeCell ref="AM13:AM15"/>
-    <mergeCell ref="AN13:AN15"/>
-    <mergeCell ref="AO13:AO15"/>
-    <mergeCell ref="EG13:EG15"/>
-    <mergeCell ref="EH13:EH15"/>
-    <mergeCell ref="AP13:AP15"/>
-    <mergeCell ref="AQ13:AQ15"/>
-    <mergeCell ref="AR13:AR15"/>
-    <mergeCell ref="AS13:AS15"/>
-    <mergeCell ref="AT13:AT15"/>
-    <mergeCell ref="AU13:AU15"/>
-    <mergeCell ref="AV13:AV15"/>
-    <mergeCell ref="AW13:AW15"/>
-    <mergeCell ref="AX13:AX15"/>
-    <mergeCell ref="AY13:AY15"/>
-    <mergeCell ref="AZ13:AZ15"/>
-    <mergeCell ref="BA13:BA15"/>
-    <mergeCell ref="BB13:BB15"/>
-    <mergeCell ref="BK13:BK15"/>
-    <mergeCell ref="BL13:BL15"/>
-    <mergeCell ref="EI13:EI15"/>
-    <mergeCell ref="EJ13:EJ15"/>
-    <mergeCell ref="ER13:ER15"/>
-    <mergeCell ref="ES13:ES15"/>
-    <mergeCell ref="ET13:ET15"/>
-    <mergeCell ref="EK13:EK15"/>
-    <mergeCell ref="EL13:EL15"/>
-    <mergeCell ref="EM13:EM15"/>
-    <mergeCell ref="EN13:EN15"/>
-    <mergeCell ref="EO13:EO15"/>
-    <mergeCell ref="EP13:EP15"/>
-    <mergeCell ref="EQ13:EQ15"/>
-    <mergeCell ref="CB13:CB15"/>
-    <mergeCell ref="CC13:CC15"/>
-    <mergeCell ref="CD13:CD15"/>
-    <mergeCell ref="CE13:CE15"/>
-    <mergeCell ref="CF13:CF15"/>
-    <mergeCell ref="CN13:CN15"/>
-    <mergeCell ref="DM11:DO11"/>
-    <mergeCell ref="CO13:CO15"/>
-    <mergeCell ref="CP13:CP15"/>
-    <mergeCell ref="CQ13:CQ15"/>
-    <mergeCell ref="CR13:CR15"/>
-    <mergeCell ref="CG13:CG15"/>
-    <mergeCell ref="CH13:CH15"/>
-    <mergeCell ref="CI13:CI15"/>
-    <mergeCell ref="CJ13:CJ15"/>
-    <mergeCell ref="CK13:CK15"/>
-    <mergeCell ref="CL13:CL15"/>
-    <mergeCell ref="CM13:CM15"/>
-    <mergeCell ref="CB10:CD12"/>
-    <mergeCell ref="CG11:CG12"/>
-    <mergeCell ref="CH11:CH12"/>
-    <mergeCell ref="CI11:CI12"/>
-    <mergeCell ref="CJ11:CJ12"/>
-    <mergeCell ref="CK11:CK12"/>
-    <mergeCell ref="EQ10:ES10"/>
-    <mergeCell ref="EQ11:EQ12"/>
-    <mergeCell ref="ER11:ER12"/>
-    <mergeCell ref="ES11:ES12"/>
-    <mergeCell ref="ET11:ET12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="AG11:AG12"/>
-    <mergeCell ref="AH11:AH12"/>
-    <mergeCell ref="AI11:AI12"/>
-    <mergeCell ref="AJ11:AJ12"/>
-    <mergeCell ref="AX11:AX12"/>
-    <mergeCell ref="AY11:AY12"/>
-    <mergeCell ref="BP11:BQ11"/>
-    <mergeCell ref="BR11:BS11"/>
-    <mergeCell ref="CE11:CE12"/>
-    <mergeCell ref="CF11:CF12"/>
-    <mergeCell ref="CW11:CW12"/>
-    <mergeCell ref="CX11:CX12"/>
-    <mergeCell ref="CY11:CY12"/>
-    <mergeCell ref="CZ11:CZ12"/>
-    <mergeCell ref="DA11:DA12"/>
-    <mergeCell ref="EB11:EB12"/>
-    <mergeCell ref="EC11:EC12"/>
-    <mergeCell ref="AF11:AF12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:AF10"/>
-    <mergeCell ref="AG10:AJ10"/>
-    <mergeCell ref="AN11:AN12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="S11:U11"/>
-    <mergeCell ref="V11:X11"/>
-    <mergeCell ref="Y11:AA11"/>
-    <mergeCell ref="AB11:AD11"/>
-    <mergeCell ref="AE11:AE12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="BJ10:BJ12"/>
-    <mergeCell ref="AP11:AP12"/>
-    <mergeCell ref="AQ11:AQ12"/>
-    <mergeCell ref="AS11:AS12"/>
-    <mergeCell ref="AT11:AT12"/>
-    <mergeCell ref="AU11:AU12"/>
-    <mergeCell ref="AV11:AV12"/>
-    <mergeCell ref="AK10:AK12"/>
-    <mergeCell ref="AL10:AL12"/>
-    <mergeCell ref="AM10:AM12"/>
-    <mergeCell ref="AN10:AQ10"/>
-    <mergeCell ref="AR10:AR12"/>
-    <mergeCell ref="AS10:AV10"/>
-    <mergeCell ref="AO11:AO12"/>
-    <mergeCell ref="EI11:EI12"/>
-    <mergeCell ref="BK10:BK12"/>
-    <mergeCell ref="BT11:BU11"/>
-    <mergeCell ref="BV11:BW11"/>
-    <mergeCell ref="BX11:BY11"/>
-    <mergeCell ref="BZ11:CA11"/>
-    <mergeCell ref="BL10:BL12"/>
-    <mergeCell ref="BM10:BM12"/>
-    <mergeCell ref="BN10:BN12"/>
-    <mergeCell ref="BO10:BO12"/>
-    <mergeCell ref="BP10:BU10"/>
-    <mergeCell ref="BV10:CA10"/>
-    <mergeCell ref="DT11:DT12"/>
-    <mergeCell ref="CU11:CU12"/>
-    <mergeCell ref="CV11:CV12"/>
-    <mergeCell ref="DU11:DU12"/>
-    <mergeCell ref="DV11:DV12"/>
-    <mergeCell ref="DW11:DW12"/>
-    <mergeCell ref="DX11:DX12"/>
-    <mergeCell ref="CE10:CG10"/>
-    <mergeCell ref="CH10:CP10"/>
-    <mergeCell ref="CQ10:CR10"/>
-    <mergeCell ref="CS10:CU10"/>
-    <mergeCell ref="CV10:DT10"/>
-    <mergeCell ref="DS11:DS12"/>
-    <mergeCell ref="CL11:CL12"/>
-    <mergeCell ref="CM11:CM12"/>
-    <mergeCell ref="CN11:CN12"/>
-    <mergeCell ref="DY10:DY12"/>
-    <mergeCell ref="ED11:ED12"/>
-    <mergeCell ref="EE11:EE12"/>
-    <mergeCell ref="EG11:EG12"/>
-    <mergeCell ref="EH11:EH12"/>
-    <mergeCell ref="DU10:DX10"/>
-    <mergeCell ref="CO11:CO12"/>
-    <mergeCell ref="CP11:CP12"/>
-    <mergeCell ref="CQ11:CQ12"/>
-    <mergeCell ref="CR11:CR12"/>
-    <mergeCell ref="CS11:CS12"/>
-    <mergeCell ref="CT11:CT12"/>
-    <mergeCell ref="DB11:DB12"/>
-    <mergeCell ref="DC11:DC12"/>
-    <mergeCell ref="DD11:DF11"/>
-    <mergeCell ref="DG11:DI11"/>
-    <mergeCell ref="DJ11:DL11"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="EP10:EP12"/>
-    <mergeCell ref="EL10:EO10"/>
-    <mergeCell ref="EL11:EL12"/>
-    <mergeCell ref="EM11:EM12"/>
-    <mergeCell ref="EN11:EN12"/>
-    <mergeCell ref="EO11:EO12"/>
-    <mergeCell ref="AW10:AW12"/>
-    <mergeCell ref="AZ11:AZ12"/>
-    <mergeCell ref="BA11:BA12"/>
-    <mergeCell ref="AX10:BA10"/>
-    <mergeCell ref="BB10:BB12"/>
-    <mergeCell ref="BC10:BC12"/>
-    <mergeCell ref="BD10:BF11"/>
-    <mergeCell ref="BG10:BI11"/>
-    <mergeCell ref="EJ11:EJ12"/>
-    <mergeCell ref="DZ10:DZ12"/>
-    <mergeCell ref="EA10:EA12"/>
-    <mergeCell ref="EB10:EE10"/>
-    <mergeCell ref="EF10:EF12"/>
-    <mergeCell ref="EG10:EJ10"/>
-    <mergeCell ref="EK10:EK12"/>
-    <mergeCell ref="DP11:DR11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
[feat/HD-15447] Fixed template title
</commit_message>
<xml_diff>
--- a/api/templates/results_ntp_use/en.xlsx
+++ b/api/templates/results_ntp_use/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/results_ntp_use/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615BDEEB-68BC-EB49-AC9A-EA92690AD30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13173D70-87E2-BD46-8559-5C9C12456BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="500" windowWidth="33720" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="286">
   <si>
     <t>Date Range: &lt;Dates&gt;</t>
   </si>
@@ -889,6 +889,9 @@
   </si>
   <si>
     <t>&lt;cnt_TypeOfPatient_Column_8_Mtb_stool&gt;</t>
+  </si>
+  <si>
+    <t>NTP Use</t>
   </si>
 </sst>
 </file>
@@ -1257,123 +1260,123 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1626,7 +1629,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:152" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
+      <c r="A1" s="2" t="s">
+        <v>285</v>
+      </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -1794,232 +1799,232 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10" spans="1:152" s="6" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="42" t="s">
+      <c r="A10" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="55"/>
-      <c r="E10" s="44" t="s">
+      <c r="D10" s="46"/>
+      <c r="E10" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="22" t="s">
+      <c r="F10" s="25"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="23"/>
-      <c r="Q10" s="23"/>
-      <c r="R10" s="23"/>
-      <c r="S10" s="23"/>
-      <c r="T10" s="23"/>
-      <c r="U10" s="23"/>
-      <c r="V10" s="23"/>
-      <c r="W10" s="23"/>
-      <c r="X10" s="23"/>
-      <c r="Y10" s="23"/>
-      <c r="Z10" s="23"/>
-      <c r="AA10" s="23"/>
-      <c r="AB10" s="23"/>
-      <c r="AC10" s="23"/>
-      <c r="AD10" s="23"/>
-      <c r="AE10" s="23"/>
-      <c r="AF10" s="24"/>
-      <c r="AG10" s="22" t="s">
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
+      <c r="M10" s="25"/>
+      <c r="N10" s="25"/>
+      <c r="O10" s="25"/>
+      <c r="P10" s="25"/>
+      <c r="Q10" s="25"/>
+      <c r="R10" s="25"/>
+      <c r="S10" s="25"/>
+      <c r="T10" s="25"/>
+      <c r="U10" s="25"/>
+      <c r="V10" s="25"/>
+      <c r="W10" s="25"/>
+      <c r="X10" s="25"/>
+      <c r="Y10" s="25"/>
+      <c r="Z10" s="25"/>
+      <c r="AA10" s="25"/>
+      <c r="AB10" s="25"/>
+      <c r="AC10" s="25"/>
+      <c r="AD10" s="25"/>
+      <c r="AE10" s="25"/>
+      <c r="AF10" s="26"/>
+      <c r="AG10" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="AH10" s="23"/>
-      <c r="AI10" s="23"/>
-      <c r="AJ10" s="24"/>
-      <c r="AK10" s="37" t="s">
+      <c r="AH10" s="25"/>
+      <c r="AI10" s="25"/>
+      <c r="AJ10" s="26"/>
+      <c r="AK10" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AL10" s="37" t="s">
+      <c r="AL10" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="AM10" s="37" t="s">
+      <c r="AM10" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="AN10" s="36" t="s">
+      <c r="AN10" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AO10" s="23"/>
-      <c r="AP10" s="23"/>
-      <c r="AQ10" s="24"/>
-      <c r="AR10" s="37" t="s">
+      <c r="AO10" s="25"/>
+      <c r="AP10" s="25"/>
+      <c r="AQ10" s="26"/>
+      <c r="AR10" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="AS10" s="36" t="s">
+      <c r="AS10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AT10" s="23"/>
-      <c r="AU10" s="23"/>
-      <c r="AV10" s="24"/>
-      <c r="AW10" s="47" t="s">
+      <c r="AT10" s="25"/>
+      <c r="AU10" s="25"/>
+      <c r="AV10" s="26"/>
+      <c r="AW10" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="AX10" s="36" t="s">
+      <c r="AX10" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="AY10" s="23"/>
-      <c r="AZ10" s="23"/>
-      <c r="BA10" s="24"/>
-      <c r="BB10" s="47" t="s">
+      <c r="AY10" s="25"/>
+      <c r="AZ10" s="25"/>
+      <c r="BA10" s="26"/>
+      <c r="BB10" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="BC10" s="34" t="s">
+      <c r="BC10" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="BD10" s="48" t="s">
+      <c r="BD10" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="BE10" s="49"/>
-      <c r="BF10" s="50"/>
-      <c r="BG10" s="54" t="s">
+      <c r="BE10" s="31"/>
+      <c r="BF10" s="32"/>
+      <c r="BG10" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="BH10" s="26"/>
-      <c r="BI10" s="27"/>
-      <c r="BJ10" s="46" t="s">
+      <c r="BH10" s="37"/>
+      <c r="BI10" s="38"/>
+      <c r="BJ10" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="BK10" s="34" t="s">
+      <c r="BK10" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="BL10" s="34" t="s">
+      <c r="BL10" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="BM10" s="41" t="s">
+      <c r="BM10" s="42" t="s">
         <v>160</v>
       </c>
-      <c r="BN10" s="23"/>
-      <c r="BO10" s="23"/>
-      <c r="BP10" s="23"/>
-      <c r="BQ10" s="23"/>
-      <c r="BR10" s="24"/>
-      <c r="BS10" s="41" t="s">
+      <c r="BN10" s="25"/>
+      <c r="BO10" s="25"/>
+      <c r="BP10" s="25"/>
+      <c r="BQ10" s="25"/>
+      <c r="BR10" s="26"/>
+      <c r="BS10" s="42" t="s">
         <v>164</v>
       </c>
-      <c r="BT10" s="23"/>
-      <c r="BU10" s="23"/>
-      <c r="BV10" s="23"/>
-      <c r="BW10" s="23"/>
-      <c r="BX10" s="24"/>
-      <c r="BY10" s="25" t="s">
+      <c r="BT10" s="25"/>
+      <c r="BU10" s="25"/>
+      <c r="BV10" s="25"/>
+      <c r="BW10" s="25"/>
+      <c r="BX10" s="26"/>
+      <c r="BY10" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="BZ10" s="26"/>
-      <c r="CA10" s="27"/>
-      <c r="CB10" s="41" t="s">
+      <c r="BZ10" s="37"/>
+      <c r="CA10" s="38"/>
+      <c r="CB10" s="42" t="s">
         <v>165</v>
       </c>
-      <c r="CC10" s="23"/>
-      <c r="CD10" s="24"/>
-      <c r="CE10" s="41" t="s">
+      <c r="CC10" s="25"/>
+      <c r="CD10" s="26"/>
+      <c r="CE10" s="42" t="s">
         <v>169</v>
       </c>
-      <c r="CF10" s="23"/>
-      <c r="CG10" s="23"/>
-      <c r="CH10" s="23"/>
-      <c r="CI10" s="23"/>
-      <c r="CJ10" s="23"/>
-      <c r="CK10" s="23"/>
-      <c r="CL10" s="23"/>
-      <c r="CM10" s="24"/>
-      <c r="CN10" s="41" t="s">
+      <c r="CF10" s="25"/>
+      <c r="CG10" s="25"/>
+      <c r="CH10" s="25"/>
+      <c r="CI10" s="25"/>
+      <c r="CJ10" s="25"/>
+      <c r="CK10" s="25"/>
+      <c r="CL10" s="25"/>
+      <c r="CM10" s="26"/>
+      <c r="CN10" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="CO10" s="24"/>
-      <c r="CP10" s="44" t="s">
+      <c r="CO10" s="26"/>
+      <c r="CP10" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="CQ10" s="23"/>
-      <c r="CR10" s="24"/>
-      <c r="CS10" s="22" t="s">
+      <c r="CQ10" s="25"/>
+      <c r="CR10" s="26"/>
+      <c r="CS10" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="CT10" s="23"/>
-      <c r="CU10" s="23"/>
-      <c r="CV10" s="23"/>
-      <c r="CW10" s="23"/>
-      <c r="CX10" s="23"/>
-      <c r="CY10" s="23"/>
-      <c r="CZ10" s="23"/>
-      <c r="DA10" s="23"/>
-      <c r="DB10" s="23"/>
-      <c r="DC10" s="23"/>
-      <c r="DD10" s="23"/>
-      <c r="DE10" s="23"/>
-      <c r="DF10" s="23"/>
-      <c r="DG10" s="23"/>
-      <c r="DH10" s="23"/>
-      <c r="DI10" s="23"/>
-      <c r="DJ10" s="23"/>
-      <c r="DK10" s="23"/>
-      <c r="DL10" s="23"/>
-      <c r="DM10" s="23"/>
-      <c r="DN10" s="23"/>
-      <c r="DO10" s="23"/>
-      <c r="DP10" s="23"/>
-      <c r="DQ10" s="24"/>
-      <c r="DR10" s="22" t="s">
+      <c r="CT10" s="25"/>
+      <c r="CU10" s="25"/>
+      <c r="CV10" s="25"/>
+      <c r="CW10" s="25"/>
+      <c r="CX10" s="25"/>
+      <c r="CY10" s="25"/>
+      <c r="CZ10" s="25"/>
+      <c r="DA10" s="25"/>
+      <c r="DB10" s="25"/>
+      <c r="DC10" s="25"/>
+      <c r="DD10" s="25"/>
+      <c r="DE10" s="25"/>
+      <c r="DF10" s="25"/>
+      <c r="DG10" s="25"/>
+      <c r="DH10" s="25"/>
+      <c r="DI10" s="25"/>
+      <c r="DJ10" s="25"/>
+      <c r="DK10" s="25"/>
+      <c r="DL10" s="25"/>
+      <c r="DM10" s="25"/>
+      <c r="DN10" s="25"/>
+      <c r="DO10" s="25"/>
+      <c r="DP10" s="25"/>
+      <c r="DQ10" s="26"/>
+      <c r="DR10" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="DS10" s="23"/>
-      <c r="DT10" s="23"/>
-      <c r="DU10" s="24"/>
-      <c r="DV10" s="37" t="s">
+      <c r="DS10" s="25"/>
+      <c r="DT10" s="25"/>
+      <c r="DU10" s="26"/>
+      <c r="DV10" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="DW10" s="37" t="s">
+      <c r="DW10" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="DX10" s="37" t="s">
+      <c r="DX10" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="DY10" s="36" t="s">
+      <c r="DY10" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="DZ10" s="23"/>
-      <c r="EA10" s="23"/>
-      <c r="EB10" s="24"/>
-      <c r="EC10" s="37" t="s">
+      <c r="DZ10" s="25"/>
+      <c r="EA10" s="25"/>
+      <c r="EB10" s="26"/>
+      <c r="EC10" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="ED10" s="36" t="s">
+      <c r="ED10" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="EE10" s="23"/>
-      <c r="EF10" s="23"/>
-      <c r="EG10" s="24"/>
-      <c r="EH10" s="47" t="s">
+      <c r="EE10" s="25"/>
+      <c r="EF10" s="25"/>
+      <c r="EG10" s="26"/>
+      <c r="EH10" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="EI10" s="36" t="s">
+      <c r="EI10" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="EJ10" s="23"/>
-      <c r="EK10" s="23"/>
-      <c r="EL10" s="24"/>
-      <c r="EM10" s="47" t="s">
+      <c r="EJ10" s="25"/>
+      <c r="EK10" s="25"/>
+      <c r="EL10" s="26"/>
+      <c r="EM10" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="EN10" s="36" t="s">
+      <c r="EN10" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="EO10" s="23"/>
-      <c r="EP10" s="24"/>
+      <c r="EO10" s="25"/>
+      <c r="EP10" s="26"/>
       <c r="EQ10" s="7" t="s">
         <v>27</v>
       </c>
@@ -2030,335 +2035,335 @@
       <c r="EV10"/>
     </row>
     <row r="11" spans="1:152" s="6" customFormat="1" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="43"/>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="56"/>
-      <c r="E11" s="38" t="s">
+      <c r="A11" s="19"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="39" t="s">
+      <c r="F11" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="39" t="s">
+      <c r="G11" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="45" t="s">
+      <c r="H11" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="I11" s="39" t="s">
+      <c r="I11" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="J11" s="39" t="s">
+      <c r="J11" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="39" t="s">
+      <c r="K11" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="39" t="s">
+      <c r="L11" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="M11" s="39" t="s">
+      <c r="M11" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="N11" s="39" t="s">
+      <c r="N11" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="O11" s="39" t="s">
+      <c r="O11" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="P11" s="22" t="s">
+      <c r="P11" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="Q11" s="23"/>
-      <c r="R11" s="24"/>
-      <c r="S11" s="22" t="s">
+      <c r="Q11" s="25"/>
+      <c r="R11" s="26"/>
+      <c r="S11" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="T11" s="23"/>
-      <c r="U11" s="24"/>
-      <c r="V11" s="22" t="s">
+      <c r="T11" s="25"/>
+      <c r="U11" s="26"/>
+      <c r="V11" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="W11" s="23"/>
-      <c r="X11" s="24"/>
-      <c r="Y11" s="22" t="s">
+      <c r="W11" s="25"/>
+      <c r="X11" s="26"/>
+      <c r="Y11" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="Z11" s="23"/>
-      <c r="AA11" s="24"/>
-      <c r="AB11" s="22" t="s">
+      <c r="Z11" s="25"/>
+      <c r="AA11" s="26"/>
+      <c r="AB11" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="AC11" s="23"/>
-      <c r="AD11" s="24"/>
-      <c r="AE11" s="39" t="s">
+      <c r="AC11" s="25"/>
+      <c r="AD11" s="26"/>
+      <c r="AE11" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="AF11" s="39" t="s">
+      <c r="AF11" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="AG11" s="39" t="s">
+      <c r="AG11" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="AH11" s="39" t="s">
+      <c r="AH11" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AI11" s="39" t="s">
+      <c r="AI11" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="AJ11" s="39" t="s">
+      <c r="AJ11" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="AK11" s="43"/>
-      <c r="AL11" s="43"/>
-      <c r="AM11" s="43"/>
-      <c r="AN11" s="37" t="s">
+      <c r="AK11" s="19"/>
+      <c r="AL11" s="19"/>
+      <c r="AM11" s="19"/>
+      <c r="AN11" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="AO11" s="37" t="s">
+      <c r="AO11" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="AP11" s="37" t="s">
+      <c r="AP11" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="AQ11" s="37" t="s">
+      <c r="AQ11" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="AR11" s="43"/>
-      <c r="AS11" s="37" t="s">
+      <c r="AR11" s="19"/>
+      <c r="AS11" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="AT11" s="37" t="s">
+      <c r="AT11" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="AU11" s="37" t="s">
+      <c r="AU11" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="AV11" s="37" t="s">
+      <c r="AV11" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="AW11" s="30"/>
-      <c r="AX11" s="40" t="s">
+      <c r="AW11" s="22"/>
+      <c r="AX11" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="AY11" s="40" t="s">
+      <c r="AY11" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="AZ11" s="40" t="s">
+      <c r="AZ11" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="BA11" s="37" t="s">
+      <c r="BA11" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="BB11" s="30"/>
-      <c r="BC11" s="43"/>
-      <c r="BD11" s="51"/>
-      <c r="BE11" s="52"/>
-      <c r="BF11" s="53"/>
-      <c r="BG11" s="31"/>
-      <c r="BH11" s="32"/>
-      <c r="BI11" s="33"/>
-      <c r="BJ11" s="43"/>
-      <c r="BK11" s="43"/>
-      <c r="BL11" s="43"/>
-      <c r="BM11" s="41" t="s">
+      <c r="BB11" s="22"/>
+      <c r="BC11" s="19"/>
+      <c r="BD11" s="33"/>
+      <c r="BE11" s="34"/>
+      <c r="BF11" s="35"/>
+      <c r="BG11" s="39"/>
+      <c r="BH11" s="40"/>
+      <c r="BI11" s="23"/>
+      <c r="BJ11" s="19"/>
+      <c r="BK11" s="19"/>
+      <c r="BL11" s="19"/>
+      <c r="BM11" s="42" t="s">
         <v>161</v>
       </c>
-      <c r="BN11" s="24"/>
-      <c r="BO11" s="41" t="s">
+      <c r="BN11" s="26"/>
+      <c r="BO11" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="BP11" s="24"/>
-      <c r="BQ11" s="41" t="s">
+      <c r="BP11" s="26"/>
+      <c r="BQ11" s="42" t="s">
         <v>163</v>
       </c>
-      <c r="BR11" s="24"/>
-      <c r="BS11" s="41" t="s">
+      <c r="BR11" s="26"/>
+      <c r="BS11" s="42" t="s">
         <v>161</v>
       </c>
-      <c r="BT11" s="24"/>
-      <c r="BU11" s="41" t="s">
+      <c r="BT11" s="26"/>
+      <c r="BU11" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="BV11" s="24"/>
-      <c r="BW11" s="41" t="s">
+      <c r="BV11" s="26"/>
+      <c r="BW11" s="42" t="s">
         <v>163</v>
       </c>
-      <c r="BX11" s="24"/>
-      <c r="BY11" s="28"/>
-      <c r="BZ11" s="29"/>
-      <c r="CA11" s="30"/>
-      <c r="CB11" s="34" t="s">
+      <c r="BX11" s="26"/>
+      <c r="BY11" s="52"/>
+      <c r="BZ11" s="53"/>
+      <c r="CA11" s="22"/>
+      <c r="CB11" s="29" t="s">
         <v>166</v>
       </c>
-      <c r="CC11" s="34" t="s">
+      <c r="CC11" s="29" t="s">
         <v>167</v>
       </c>
-      <c r="CD11" s="34" t="s">
+      <c r="CD11" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="CE11" s="34" t="s">
+      <c r="CE11" s="29" t="s">
         <v>170</v>
       </c>
-      <c r="CF11" s="34" t="s">
+      <c r="CF11" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="CG11" s="34" t="s">
+      <c r="CG11" s="29" t="s">
         <v>172</v>
       </c>
-      <c r="CH11" s="34" t="s">
+      <c r="CH11" s="29" t="s">
         <v>173</v>
       </c>
-      <c r="CI11" s="34" t="s">
+      <c r="CI11" s="29" t="s">
         <v>174</v>
       </c>
-      <c r="CJ11" s="34" t="s">
+      <c r="CJ11" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="CK11" s="34" t="s">
+      <c r="CK11" s="29" t="s">
         <v>176</v>
       </c>
-      <c r="CL11" s="34" t="s">
+      <c r="CL11" s="29" t="s">
         <v>177</v>
       </c>
-      <c r="CM11" s="34" t="s">
+      <c r="CM11" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="CN11" s="34" t="s">
+      <c r="CN11" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="CO11" s="34" t="s">
+      <c r="CO11" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="CP11" s="38" t="s">
+      <c r="CP11" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="CQ11" s="39" t="s">
+      <c r="CQ11" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="CR11" s="39" t="s">
+      <c r="CR11" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="CS11" s="45" t="s">
+      <c r="CS11" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="CT11" s="39" t="s">
+      <c r="CT11" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="CU11" s="39" t="s">
+      <c r="CU11" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="CV11" s="39" t="s">
+      <c r="CV11" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="CW11" s="39" t="s">
+      <c r="CW11" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="CX11" s="39" t="s">
+      <c r="CX11" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="CY11" s="39" t="s">
+      <c r="CY11" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="CZ11" s="39" t="s">
+      <c r="CZ11" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="DA11" s="22" t="s">
+      <c r="DA11" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="DB11" s="23"/>
-      <c r="DC11" s="24"/>
-      <c r="DD11" s="22" t="s">
+      <c r="DB11" s="25"/>
+      <c r="DC11" s="26"/>
+      <c r="DD11" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="DE11" s="23"/>
-      <c r="DF11" s="24"/>
-      <c r="DG11" s="22" t="s">
+      <c r="DE11" s="25"/>
+      <c r="DF11" s="26"/>
+      <c r="DG11" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="DH11" s="23"/>
-      <c r="DI11" s="24"/>
-      <c r="DJ11" s="22" t="s">
+      <c r="DH11" s="25"/>
+      <c r="DI11" s="26"/>
+      <c r="DJ11" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="DK11" s="23"/>
-      <c r="DL11" s="24"/>
-      <c r="DM11" s="22" t="s">
+      <c r="DK11" s="25"/>
+      <c r="DL11" s="26"/>
+      <c r="DM11" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="DN11" s="23"/>
-      <c r="DO11" s="24"/>
-      <c r="DP11" s="39" t="s">
+      <c r="DN11" s="25"/>
+      <c r="DO11" s="26"/>
+      <c r="DP11" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="DQ11" s="39" t="s">
+      <c r="DQ11" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="DR11" s="39" t="s">
+      <c r="DR11" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="DS11" s="39" t="s">
+      <c r="DS11" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="DT11" s="39" t="s">
+      <c r="DT11" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="DU11" s="39" t="s">
+      <c r="DU11" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="DV11" s="43"/>
-      <c r="DW11" s="43"/>
-      <c r="DX11" s="43"/>
-      <c r="DY11" s="37" t="s">
+      <c r="DV11" s="19"/>
+      <c r="DW11" s="19"/>
+      <c r="DX11" s="19"/>
+      <c r="DY11" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="DZ11" s="37" t="s">
+      <c r="DZ11" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="EA11" s="37" t="s">
+      <c r="EA11" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="EB11" s="37" t="s">
+      <c r="EB11" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="EC11" s="43"/>
-      <c r="ED11" s="37" t="s">
+      <c r="EC11" s="19"/>
+      <c r="ED11" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="EE11" s="37" t="s">
+      <c r="EE11" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="EF11" s="37" t="s">
+      <c r="EF11" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="EG11" s="37" t="s">
+      <c r="EG11" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="EH11" s="30"/>
-      <c r="EI11" s="40" t="s">
+      <c r="EH11" s="22"/>
+      <c r="EI11" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="EJ11" s="40" t="s">
+      <c r="EJ11" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="EK11" s="40" t="s">
+      <c r="EK11" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="EL11" s="37" t="s">
+      <c r="EL11" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="EM11" s="30"/>
-      <c r="EN11" s="37" t="s">
+      <c r="EM11" s="22"/>
+      <c r="EN11" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="EO11" s="37" t="s">
+      <c r="EO11" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="EP11" s="37" t="s">
+      <c r="EP11" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="EQ11" s="34" t="s">
+      <c r="EQ11" s="29" t="s">
         <v>52</v>
       </c>
       <c r="ER11"/>
@@ -2368,21 +2373,21 @@
       <c r="EV11"/>
     </row>
     <row r="12" spans="1:152" s="6" customFormat="1" ht="79.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="35"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="57"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
-      <c r="N12" s="35"/>
-      <c r="O12" s="35"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
+      <c r="M12" s="20"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="20"/>
       <c r="P12" s="13" t="s">
         <v>53</v>
       </c>
@@ -2428,31 +2433,31 @@
       <c r="AD12" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="AE12" s="35"/>
-      <c r="AF12" s="35"/>
-      <c r="AG12" s="35"/>
-      <c r="AH12" s="35"/>
-      <c r="AI12" s="35"/>
-      <c r="AJ12" s="35"/>
-      <c r="AK12" s="35"/>
-      <c r="AL12" s="35"/>
-      <c r="AM12" s="35"/>
-      <c r="AN12" s="35"/>
-      <c r="AO12" s="35"/>
-      <c r="AP12" s="35"/>
-      <c r="AQ12" s="35"/>
-      <c r="AR12" s="35"/>
-      <c r="AS12" s="35"/>
-      <c r="AT12" s="35"/>
-      <c r="AU12" s="35"/>
-      <c r="AV12" s="35"/>
-      <c r="AW12" s="33"/>
-      <c r="AX12" s="35"/>
-      <c r="AY12" s="35"/>
-      <c r="AZ12" s="35"/>
-      <c r="BA12" s="35"/>
-      <c r="BB12" s="33"/>
-      <c r="BC12" s="35"/>
+      <c r="AE12" s="20"/>
+      <c r="AF12" s="20"/>
+      <c r="AG12" s="20"/>
+      <c r="AH12" s="20"/>
+      <c r="AI12" s="20"/>
+      <c r="AJ12" s="20"/>
+      <c r="AK12" s="20"/>
+      <c r="AL12" s="20"/>
+      <c r="AM12" s="20"/>
+      <c r="AN12" s="20"/>
+      <c r="AO12" s="20"/>
+      <c r="AP12" s="20"/>
+      <c r="AQ12" s="20"/>
+      <c r="AR12" s="20"/>
+      <c r="AS12" s="20"/>
+      <c r="AT12" s="20"/>
+      <c r="AU12" s="20"/>
+      <c r="AV12" s="20"/>
+      <c r="AW12" s="23"/>
+      <c r="AX12" s="20"/>
+      <c r="AY12" s="20"/>
+      <c r="AZ12" s="20"/>
+      <c r="BA12" s="20"/>
+      <c r="BB12" s="23"/>
+      <c r="BC12" s="20"/>
       <c r="BD12" s="8" t="s">
         <v>55</v>
       </c>
@@ -2471,9 +2476,9 @@
       <c r="BI12" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="BJ12" s="35"/>
-      <c r="BK12" s="35"/>
-      <c r="BL12" s="35"/>
+      <c r="BJ12" s="20"/>
+      <c r="BK12" s="20"/>
+      <c r="BL12" s="20"/>
       <c r="BM12" s="8" t="s">
         <v>58</v>
       </c>
@@ -2510,34 +2515,34 @@
       <c r="BX12" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="BY12" s="31"/>
-      <c r="BZ12" s="32"/>
-      <c r="CA12" s="33"/>
-      <c r="CB12" s="35"/>
-      <c r="CC12" s="35"/>
-      <c r="CD12" s="35"/>
-      <c r="CE12" s="35"/>
-      <c r="CF12" s="35"/>
-      <c r="CG12" s="35"/>
-      <c r="CH12" s="35"/>
-      <c r="CI12" s="35"/>
-      <c r="CJ12" s="35"/>
-      <c r="CK12" s="35"/>
-      <c r="CL12" s="35"/>
-      <c r="CM12" s="35"/>
-      <c r="CN12" s="35"/>
-      <c r="CO12" s="35"/>
-      <c r="CP12" s="35"/>
-      <c r="CQ12" s="35"/>
-      <c r="CR12" s="35"/>
-      <c r="CS12" s="35"/>
-      <c r="CT12" s="35"/>
-      <c r="CU12" s="35"/>
-      <c r="CV12" s="35"/>
-      <c r="CW12" s="35"/>
-      <c r="CX12" s="35"/>
-      <c r="CY12" s="35"/>
-      <c r="CZ12" s="35"/>
+      <c r="BY12" s="39"/>
+      <c r="BZ12" s="40"/>
+      <c r="CA12" s="23"/>
+      <c r="CB12" s="20"/>
+      <c r="CC12" s="20"/>
+      <c r="CD12" s="20"/>
+      <c r="CE12" s="20"/>
+      <c r="CF12" s="20"/>
+      <c r="CG12" s="20"/>
+      <c r="CH12" s="20"/>
+      <c r="CI12" s="20"/>
+      <c r="CJ12" s="20"/>
+      <c r="CK12" s="20"/>
+      <c r="CL12" s="20"/>
+      <c r="CM12" s="20"/>
+      <c r="CN12" s="20"/>
+      <c r="CO12" s="20"/>
+      <c r="CP12" s="20"/>
+      <c r="CQ12" s="20"/>
+      <c r="CR12" s="20"/>
+      <c r="CS12" s="20"/>
+      <c r="CT12" s="20"/>
+      <c r="CU12" s="20"/>
+      <c r="CV12" s="20"/>
+      <c r="CW12" s="20"/>
+      <c r="CX12" s="20"/>
+      <c r="CY12" s="20"/>
+      <c r="CZ12" s="20"/>
       <c r="DA12" s="13" t="s">
         <v>53</v>
       </c>
@@ -2583,34 +2588,34 @@
       <c r="DO12" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="DP12" s="35"/>
-      <c r="DQ12" s="35"/>
-      <c r="DR12" s="35"/>
-      <c r="DS12" s="35"/>
-      <c r="DT12" s="35"/>
-      <c r="DU12" s="35"/>
-      <c r="DV12" s="35"/>
-      <c r="DW12" s="35"/>
-      <c r="DX12" s="35"/>
-      <c r="DY12" s="35"/>
-      <c r="DZ12" s="35"/>
-      <c r="EA12" s="35"/>
-      <c r="EB12" s="35"/>
-      <c r="EC12" s="35"/>
-      <c r="ED12" s="35"/>
-      <c r="EE12" s="35"/>
-      <c r="EF12" s="35"/>
-      <c r="EG12" s="35"/>
-      <c r="EH12" s="33"/>
-      <c r="EI12" s="35"/>
-      <c r="EJ12" s="35"/>
-      <c r="EK12" s="35"/>
-      <c r="EL12" s="35"/>
-      <c r="EM12" s="33"/>
-      <c r="EN12" s="35"/>
-      <c r="EO12" s="35"/>
-      <c r="EP12" s="35"/>
-      <c r="EQ12" s="35"/>
+      <c r="DP12" s="20"/>
+      <c r="DQ12" s="20"/>
+      <c r="DR12" s="20"/>
+      <c r="DS12" s="20"/>
+      <c r="DT12" s="20"/>
+      <c r="DU12" s="20"/>
+      <c r="DV12" s="20"/>
+      <c r="DW12" s="20"/>
+      <c r="DX12" s="20"/>
+      <c r="DY12" s="20"/>
+      <c r="DZ12" s="20"/>
+      <c r="EA12" s="20"/>
+      <c r="EB12" s="20"/>
+      <c r="EC12" s="20"/>
+      <c r="ED12" s="20"/>
+      <c r="EE12" s="20"/>
+      <c r="EF12" s="20"/>
+      <c r="EG12" s="20"/>
+      <c r="EH12" s="23"/>
+      <c r="EI12" s="20"/>
+      <c r="EJ12" s="20"/>
+      <c r="EK12" s="20"/>
+      <c r="EL12" s="20"/>
+      <c r="EM12" s="23"/>
+      <c r="EN12" s="20"/>
+      <c r="EO12" s="20"/>
+      <c r="EP12" s="20"/>
+      <c r="EQ12" s="20"/>
       <c r="ER12"/>
       <c r="ES12"/>
       <c r="ET12"/>
@@ -2618,13 +2623,13 @@
       <c r="EV12"/>
     </row>
     <row r="13" spans="1:152" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="57" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="57" t="s">
         <v>259</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="57" t="s">
         <v>60</v>
       </c>
       <c r="D13" s="10" t="s">
@@ -2728,73 +2733,73 @@
         <f>SUM(AG13:AI13)</f>
         <v>0</v>
       </c>
-      <c r="AK13" s="20">
+      <c r="AK13" s="54">
         <f>G13+AJ13</f>
         <v>0</v>
       </c>
-      <c r="AL13" s="20">
+      <c r="AL13" s="54">
         <f>AF13</f>
         <v>0</v>
       </c>
-      <c r="AM13" s="20">
+      <c r="AM13" s="54">
         <f>AK13+AL13</f>
         <v>0</v>
       </c>
-      <c r="AN13" s="20">
+      <c r="AN13" s="54">
         <f>G14+AJ14-G15-AJ15</f>
         <v>0</v>
       </c>
-      <c r="AO13" s="20">
+      <c r="AO13" s="54">
         <f>G15+AJ15</f>
         <v>0</v>
       </c>
-      <c r="AP13" s="20" t="s">
+      <c r="AP13" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="AQ13" s="20">
+      <c r="AQ13" s="54">
         <f>AE15</f>
         <v>0</v>
       </c>
-      <c r="AR13" s="20">
+      <c r="AR13" s="54">
         <f>AK13-G14-AJ14</f>
         <v>0</v>
       </c>
-      <c r="AS13" s="20">
+      <c r="AS13" s="54">
         <f>+AF14-AF15</f>
         <v>0</v>
       </c>
-      <c r="AT13" s="20">
+      <c r="AT13" s="54">
         <f>AF15</f>
         <v>0</v>
       </c>
-      <c r="AU13" s="20" t="s">
+      <c r="AU13" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="AV13" s="20">
+      <c r="AV13" s="54">
         <f>AF15</f>
         <v>0</v>
       </c>
-      <c r="AW13" s="20">
+      <c r="AW13" s="54">
         <f>AL13-AF14</f>
         <v>0</v>
       </c>
-      <c r="AX13" s="20">
+      <c r="AX13" s="54">
         <f>AN13+AS13</f>
         <v>0</v>
       </c>
-      <c r="AY13" s="20">
+      <c r="AY13" s="54">
         <f>AO13+AT13</f>
         <v>0</v>
       </c>
-      <c r="AZ13" s="20" t="e">
+      <c r="AZ13" s="54" t="e">
         <f>AP13+AU13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA13" s="20">
+      <c r="BA13" s="54">
         <f>AQ13+AV13</f>
         <v>0</v>
       </c>
-      <c r="BB13" s="20">
+      <c r="BB13" s="54">
         <f>AR13+AW13</f>
         <v>0</v>
       </c>
@@ -2823,73 +2828,73 @@
         <f>SUM(BD13:BI13)</f>
         <v>0</v>
       </c>
-      <c r="BK13" s="20"/>
-      <c r="BL13" s="20"/>
-      <c r="BM13" s="20" t="s">
+      <c r="BK13" s="54"/>
+      <c r="BL13" s="54"/>
+      <c r="BM13" s="54" t="s">
         <v>263</v>
       </c>
-      <c r="BN13" s="20" t="s">
+      <c r="BN13" s="54" t="s">
         <v>264</v>
       </c>
-      <c r="BO13" s="20" t="s">
+      <c r="BO13" s="54" t="s">
         <v>265</v>
       </c>
-      <c r="BP13" s="20" t="s">
+      <c r="BP13" s="54" t="s">
         <v>266</v>
       </c>
-      <c r="BQ13" s="20" t="s">
+      <c r="BQ13" s="54" t="s">
         <v>267</v>
       </c>
-      <c r="BR13" s="20" t="s">
+      <c r="BR13" s="54" t="s">
         <v>268</v>
       </c>
-      <c r="BS13" s="20" t="s">
+      <c r="BS13" s="54" t="s">
         <v>269</v>
       </c>
-      <c r="BT13" s="20" t="s">
+      <c r="BT13" s="54" t="s">
         <v>270</v>
       </c>
-      <c r="BU13" s="20" t="s">
+      <c r="BU13" s="54" t="s">
         <v>271</v>
       </c>
-      <c r="BV13" s="20" t="s">
+      <c r="BV13" s="54" t="s">
         <v>272</v>
       </c>
-      <c r="BW13" s="20" t="s">
+      <c r="BW13" s="54" t="s">
         <v>273</v>
       </c>
-      <c r="BX13" s="20" t="s">
+      <c r="BX13" s="54" t="s">
         <v>274</v>
       </c>
-      <c r="BY13" s="20" t="s">
+      <c r="BY13" s="54" t="s">
         <v>275</v>
       </c>
-      <c r="BZ13" s="20" t="s">
+      <c r="BZ13" s="54" t="s">
         <v>276</v>
       </c>
-      <c r="CA13" s="20" t="s">
+      <c r="CA13" s="54" t="s">
         <v>277</v>
       </c>
-      <c r="CB13" s="20" t="s">
+      <c r="CB13" s="54" t="s">
         <v>278</v>
       </c>
-      <c r="CC13" s="20" t="s">
+      <c r="CC13" s="54" t="s">
         <v>279</v>
       </c>
-      <c r="CD13" s="20" t="s">
+      <c r="CD13" s="54" t="s">
         <v>280</v>
       </c>
-      <c r="CE13" s="20"/>
-      <c r="CF13" s="20"/>
-      <c r="CG13" s="20"/>
-      <c r="CH13" s="20"/>
-      <c r="CI13" s="20"/>
-      <c r="CJ13" s="20"/>
-      <c r="CK13" s="20"/>
-      <c r="CL13" s="20"/>
-      <c r="CM13" s="20"/>
-      <c r="CN13" s="21"/>
-      <c r="CO13" s="21"/>
+      <c r="CE13" s="54"/>
+      <c r="CF13" s="54"/>
+      <c r="CG13" s="54"/>
+      <c r="CH13" s="54"/>
+      <c r="CI13" s="54"/>
+      <c r="CJ13" s="54"/>
+      <c r="CK13" s="54"/>
+      <c r="CL13" s="54"/>
+      <c r="CM13" s="54"/>
+      <c r="CN13" s="56"/>
+      <c r="CO13" s="56"/>
       <c r="CP13" s="10" t="s">
         <v>179</v>
       </c>
@@ -2988,93 +2993,93 @@
         <f>SUM(DR13:DT13)</f>
         <v>0</v>
       </c>
-      <c r="DV13" s="20">
+      <c r="DV13" s="54">
         <f>SUM(CR13:DU13)</f>
         <v>0</v>
       </c>
-      <c r="DW13" s="20">
+      <c r="DW13" s="54">
         <f>DQ13</f>
         <v>0</v>
       </c>
-      <c r="DX13" s="20">
+      <c r="DX13" s="54">
         <f>DV13+DW13</f>
         <v>0</v>
       </c>
-      <c r="DY13" s="20">
+      <c r="DY13" s="54">
         <f>CR14+DQ14-CR15-DQ15</f>
         <v>0</v>
       </c>
-      <c r="DZ13" s="20">
+      <c r="DZ13" s="54">
         <f>CR15+DQ15</f>
         <v>0</v>
       </c>
-      <c r="EA13" s="20" t="s">
+      <c r="EA13" s="54" t="s">
         <v>281</v>
       </c>
-      <c r="EB13" s="20">
+      <c r="EB13" s="54">
         <f>DP15</f>
         <v>0</v>
       </c>
-      <c r="EC13" s="20">
+      <c r="EC13" s="54">
         <f>DV13-DU14-CR14</f>
         <v>0</v>
       </c>
-      <c r="ED13" s="20">
+      <c r="ED13" s="54">
         <f>+DQ14-DQ15</f>
         <v>0</v>
       </c>
-      <c r="EE13" s="20">
+      <c r="EE13" s="54">
         <f>DQ15</f>
         <v>0</v>
       </c>
-      <c r="EF13" s="20" t="s">
+      <c r="EF13" s="54" t="s">
         <v>282</v>
       </c>
-      <c r="EG13" s="20">
+      <c r="EG13" s="54">
         <f>DQ15</f>
         <v>0</v>
       </c>
-      <c r="EH13" s="20">
+      <c r="EH13" s="54">
         <f>DW13-DQ14</f>
         <v>0</v>
       </c>
-      <c r="EI13" s="20">
+      <c r="EI13" s="54">
         <f>DY13+ED13</f>
         <v>0</v>
       </c>
-      <c r="EJ13" s="20">
+      <c r="EJ13" s="54">
         <f>DZ13-EE13</f>
         <v>0</v>
       </c>
-      <c r="EK13" s="20" t="e">
+      <c r="EK13" s="54" t="e">
         <f>EA13+EF13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="EL13" s="20">
+      <c r="EL13" s="54">
         <f>EB13+EG13</f>
         <v>0</v>
       </c>
-      <c r="EM13" s="20">
+      <c r="EM13" s="54">
         <f>EC13+EH13</f>
         <v>0</v>
       </c>
-      <c r="EN13" s="21">
+      <c r="EN13" s="56">
         <f>ED13+EJ13</f>
         <v>0</v>
       </c>
-      <c r="EO13" s="21"/>
-      <c r="EP13" s="21" t="s">
+      <c r="EO13" s="56"/>
+      <c r="EP13" s="56" t="s">
         <v>283</v>
       </c>
-      <c r="EQ13" s="20" t="str">
+      <c r="EQ13" s="54" t="str">
         <f>EP13</f>
         <v>&lt;cnt_Xdr_Total_Tests_stool&gt;</v>
       </c>
     </row>
     <row r="14" spans="1:152" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="18"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
+      <c r="A14" s="57"/>
+      <c r="B14" s="55"/>
+      <c r="C14" s="55"/>
       <c r="D14" s="10" t="s">
         <v>62</v>
       </c>
@@ -3176,24 +3181,24 @@
         <f>SUM(AG14:AI14)</f>
         <v>0</v>
       </c>
-      <c r="AK14" s="19"/>
-      <c r="AL14" s="19"/>
-      <c r="AM14" s="19"/>
-      <c r="AN14" s="19"/>
-      <c r="AO14" s="19"/>
-      <c r="AP14" s="19"/>
-      <c r="AQ14" s="19"/>
-      <c r="AR14" s="19"/>
-      <c r="AS14" s="19"/>
-      <c r="AT14" s="19"/>
-      <c r="AU14" s="19"/>
-      <c r="AV14" s="19"/>
-      <c r="AW14" s="19"/>
-      <c r="AX14" s="19"/>
-      <c r="AY14" s="19"/>
-      <c r="AZ14" s="19"/>
-      <c r="BA14" s="19"/>
-      <c r="BB14" s="19"/>
+      <c r="AK14" s="55"/>
+      <c r="AL14" s="55"/>
+      <c r="AM14" s="55"/>
+      <c r="AN14" s="55"/>
+      <c r="AO14" s="55"/>
+      <c r="AP14" s="55"/>
+      <c r="AQ14" s="55"/>
+      <c r="AR14" s="55"/>
+      <c r="AS14" s="55"/>
+      <c r="AT14" s="55"/>
+      <c r="AU14" s="55"/>
+      <c r="AV14" s="55"/>
+      <c r="AW14" s="55"/>
+      <c r="AX14" s="55"/>
+      <c r="AY14" s="55"/>
+      <c r="AZ14" s="55"/>
+      <c r="BA14" s="55"/>
+      <c r="BB14" s="55"/>
       <c r="BC14" s="16" t="s">
         <v>63</v>
       </c>
@@ -3219,37 +3224,37 @@
         <f>SUM(BD14:BI14)</f>
         <v>0</v>
       </c>
-      <c r="BK14" s="19"/>
-      <c r="BL14" s="19"/>
-      <c r="BM14" s="19"/>
-      <c r="BN14" s="19"/>
-      <c r="BO14" s="19"/>
-      <c r="BP14" s="19"/>
-      <c r="BQ14" s="19"/>
-      <c r="BR14" s="19"/>
-      <c r="BS14" s="19"/>
-      <c r="BT14" s="19"/>
-      <c r="BU14" s="19"/>
-      <c r="BV14" s="19"/>
-      <c r="BW14" s="19"/>
-      <c r="BX14" s="19"/>
-      <c r="BY14" s="19"/>
-      <c r="BZ14" s="19"/>
-      <c r="CA14" s="19"/>
-      <c r="CB14" s="19"/>
-      <c r="CC14" s="19"/>
-      <c r="CD14" s="19"/>
-      <c r="CE14" s="19"/>
-      <c r="CF14" s="19"/>
-      <c r="CG14" s="19"/>
-      <c r="CH14" s="20"/>
-      <c r="CI14" s="19"/>
-      <c r="CJ14" s="19"/>
-      <c r="CK14" s="19"/>
-      <c r="CL14" s="19"/>
-      <c r="CM14" s="19"/>
-      <c r="CN14" s="19"/>
-      <c r="CO14" s="19"/>
+      <c r="BK14" s="55"/>
+      <c r="BL14" s="55"/>
+      <c r="BM14" s="55"/>
+      <c r="BN14" s="55"/>
+      <c r="BO14" s="55"/>
+      <c r="BP14" s="55"/>
+      <c r="BQ14" s="55"/>
+      <c r="BR14" s="55"/>
+      <c r="BS14" s="55"/>
+      <c r="BT14" s="55"/>
+      <c r="BU14" s="55"/>
+      <c r="BV14" s="55"/>
+      <c r="BW14" s="55"/>
+      <c r="BX14" s="55"/>
+      <c r="BY14" s="55"/>
+      <c r="BZ14" s="55"/>
+      <c r="CA14" s="55"/>
+      <c r="CB14" s="55"/>
+      <c r="CC14" s="55"/>
+      <c r="CD14" s="55"/>
+      <c r="CE14" s="55"/>
+      <c r="CF14" s="55"/>
+      <c r="CG14" s="55"/>
+      <c r="CH14" s="54"/>
+      <c r="CI14" s="55"/>
+      <c r="CJ14" s="55"/>
+      <c r="CK14" s="55"/>
+      <c r="CL14" s="55"/>
+      <c r="CM14" s="55"/>
+      <c r="CN14" s="55"/>
+      <c r="CO14" s="55"/>
       <c r="CP14" s="10" t="s">
         <v>183</v>
       </c>
@@ -3348,33 +3353,33 @@
         <f>SUM(DR14:DT14)</f>
         <v>0</v>
       </c>
-      <c r="DV14" s="19"/>
-      <c r="DW14" s="19"/>
-      <c r="DX14" s="19"/>
-      <c r="DY14" s="19"/>
-      <c r="DZ14" s="19"/>
-      <c r="EA14" s="19"/>
-      <c r="EB14" s="19"/>
-      <c r="EC14" s="19"/>
-      <c r="ED14" s="19"/>
-      <c r="EE14" s="19"/>
-      <c r="EF14" s="19"/>
-      <c r="EG14" s="19"/>
-      <c r="EH14" s="19"/>
-      <c r="EI14" s="19"/>
-      <c r="EJ14" s="19"/>
-      <c r="EK14" s="19"/>
-      <c r="EL14" s="19"/>
-      <c r="EM14" s="19"/>
-      <c r="EN14" s="19"/>
-      <c r="EO14" s="21"/>
-      <c r="EP14" s="19"/>
-      <c r="EQ14" s="19"/>
+      <c r="DV14" s="55"/>
+      <c r="DW14" s="55"/>
+      <c r="DX14" s="55"/>
+      <c r="DY14" s="55"/>
+      <c r="DZ14" s="55"/>
+      <c r="EA14" s="55"/>
+      <c r="EB14" s="55"/>
+      <c r="EC14" s="55"/>
+      <c r="ED14" s="55"/>
+      <c r="EE14" s="55"/>
+      <c r="EF14" s="55"/>
+      <c r="EG14" s="55"/>
+      <c r="EH14" s="55"/>
+      <c r="EI14" s="55"/>
+      <c r="EJ14" s="55"/>
+      <c r="EK14" s="55"/>
+      <c r="EL14" s="55"/>
+      <c r="EM14" s="55"/>
+      <c r="EN14" s="55"/>
+      <c r="EO14" s="56"/>
+      <c r="EP14" s="55"/>
+      <c r="EQ14" s="55"/>
     </row>
     <row r="15" spans="1:152" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="18"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
+      <c r="A15" s="57"/>
+      <c r="B15" s="55"/>
+      <c r="C15" s="55"/>
       <c r="D15" s="10" t="s">
         <v>64</v>
       </c>
@@ -3476,24 +3481,24 @@
         <f>SUM(AG15:AI15)</f>
         <v>0</v>
       </c>
-      <c r="AK15" s="19"/>
-      <c r="AL15" s="19"/>
-      <c r="AM15" s="19"/>
-      <c r="AN15" s="19"/>
-      <c r="AO15" s="19"/>
-      <c r="AP15" s="19"/>
-      <c r="AQ15" s="19"/>
-      <c r="AR15" s="19"/>
-      <c r="AS15" s="19"/>
-      <c r="AT15" s="19"/>
-      <c r="AU15" s="19"/>
-      <c r="AV15" s="19"/>
-      <c r="AW15" s="19"/>
-      <c r="AX15" s="19"/>
-      <c r="AY15" s="19"/>
-      <c r="AZ15" s="19"/>
-      <c r="BA15" s="19"/>
-      <c r="BB15" s="19"/>
+      <c r="AK15" s="55"/>
+      <c r="AL15" s="55"/>
+      <c r="AM15" s="55"/>
+      <c r="AN15" s="55"/>
+      <c r="AO15" s="55"/>
+      <c r="AP15" s="55"/>
+      <c r="AQ15" s="55"/>
+      <c r="AR15" s="55"/>
+      <c r="AS15" s="55"/>
+      <c r="AT15" s="55"/>
+      <c r="AU15" s="55"/>
+      <c r="AV15" s="55"/>
+      <c r="AW15" s="55"/>
+      <c r="AX15" s="55"/>
+      <c r="AY15" s="55"/>
+      <c r="AZ15" s="55"/>
+      <c r="BA15" s="55"/>
+      <c r="BB15" s="55"/>
       <c r="BC15" s="17"/>
       <c r="BD15" s="15"/>
       <c r="BE15" s="15"/>
@@ -3502,37 +3507,37 @@
       <c r="BH15" s="15"/>
       <c r="BI15" s="15"/>
       <c r="BJ15" s="15"/>
-      <c r="BK15" s="19"/>
-      <c r="BL15" s="19"/>
-      <c r="BM15" s="19"/>
-      <c r="BN15" s="19"/>
-      <c r="BO15" s="19"/>
-      <c r="BP15" s="19"/>
-      <c r="BQ15" s="19"/>
-      <c r="BR15" s="19"/>
-      <c r="BS15" s="19"/>
-      <c r="BT15" s="19"/>
-      <c r="BU15" s="19"/>
-      <c r="BV15" s="19"/>
-      <c r="BW15" s="19"/>
-      <c r="BX15" s="19"/>
-      <c r="BY15" s="19"/>
-      <c r="BZ15" s="19"/>
-      <c r="CA15" s="19"/>
-      <c r="CB15" s="19"/>
-      <c r="CC15" s="19"/>
-      <c r="CD15" s="19"/>
-      <c r="CE15" s="19"/>
-      <c r="CF15" s="19"/>
-      <c r="CG15" s="19"/>
-      <c r="CH15" s="20"/>
-      <c r="CI15" s="19"/>
-      <c r="CJ15" s="19"/>
-      <c r="CK15" s="19"/>
-      <c r="CL15" s="19"/>
-      <c r="CM15" s="19"/>
-      <c r="CN15" s="19"/>
-      <c r="CO15" s="19"/>
+      <c r="BK15" s="55"/>
+      <c r="BL15" s="55"/>
+      <c r="BM15" s="55"/>
+      <c r="BN15" s="55"/>
+      <c r="BO15" s="55"/>
+      <c r="BP15" s="55"/>
+      <c r="BQ15" s="55"/>
+      <c r="BR15" s="55"/>
+      <c r="BS15" s="55"/>
+      <c r="BT15" s="55"/>
+      <c r="BU15" s="55"/>
+      <c r="BV15" s="55"/>
+      <c r="BW15" s="55"/>
+      <c r="BX15" s="55"/>
+      <c r="BY15" s="55"/>
+      <c r="BZ15" s="55"/>
+      <c r="CA15" s="55"/>
+      <c r="CB15" s="55"/>
+      <c r="CC15" s="55"/>
+      <c r="CD15" s="55"/>
+      <c r="CE15" s="55"/>
+      <c r="CF15" s="55"/>
+      <c r="CG15" s="55"/>
+      <c r="CH15" s="54"/>
+      <c r="CI15" s="55"/>
+      <c r="CJ15" s="55"/>
+      <c r="CK15" s="55"/>
+      <c r="CL15" s="55"/>
+      <c r="CM15" s="55"/>
+      <c r="CN15" s="55"/>
+      <c r="CO15" s="55"/>
       <c r="CP15" s="10" t="s">
         <v>184</v>
       </c>
@@ -3631,28 +3636,28 @@
         <f>SUM(DR15:DT15)</f>
         <v>0</v>
       </c>
-      <c r="DV15" s="19"/>
-      <c r="DW15" s="19"/>
-      <c r="DX15" s="19"/>
-      <c r="DY15" s="19"/>
-      <c r="DZ15" s="19"/>
-      <c r="EA15" s="19"/>
-      <c r="EB15" s="19"/>
-      <c r="EC15" s="19"/>
-      <c r="ED15" s="19"/>
-      <c r="EE15" s="19"/>
-      <c r="EF15" s="19"/>
-      <c r="EG15" s="19"/>
-      <c r="EH15" s="19"/>
-      <c r="EI15" s="19"/>
-      <c r="EJ15" s="19"/>
-      <c r="EK15" s="19"/>
-      <c r="EL15" s="19"/>
-      <c r="EM15" s="19"/>
-      <c r="EN15" s="19"/>
-      <c r="EO15" s="21"/>
-      <c r="EP15" s="19"/>
-      <c r="EQ15" s="19"/>
+      <c r="DV15" s="55"/>
+      <c r="DW15" s="55"/>
+      <c r="DX15" s="55"/>
+      <c r="DY15" s="55"/>
+      <c r="DZ15" s="55"/>
+      <c r="EA15" s="55"/>
+      <c r="EB15" s="55"/>
+      <c r="EC15" s="55"/>
+      <c r="ED15" s="55"/>
+      <c r="EE15" s="55"/>
+      <c r="EF15" s="55"/>
+      <c r="EG15" s="55"/>
+      <c r="EH15" s="55"/>
+      <c r="EI15" s="55"/>
+      <c r="EJ15" s="55"/>
+      <c r="EK15" s="55"/>
+      <c r="EL15" s="55"/>
+      <c r="EM15" s="55"/>
+      <c r="EN15" s="55"/>
+      <c r="EO15" s="56"/>
+      <c r="EP15" s="55"/>
+      <c r="EQ15" s="55"/>
     </row>
     <row r="21" spans="123:123" x14ac:dyDescent="0.2">
       <c r="DS21">
@@ -3661,6 +3666,189 @@
     </row>
   </sheetData>
   <mergeCells count="207">
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="DV13:DV15"/>
+    <mergeCell ref="DW13:DW15"/>
+    <mergeCell ref="DX13:DX15"/>
+    <mergeCell ref="DY13:DY15"/>
+    <mergeCell ref="DZ13:DZ15"/>
+    <mergeCell ref="EA13:EA15"/>
+    <mergeCell ref="BK13:BK15"/>
+    <mergeCell ref="BL13:BL15"/>
+    <mergeCell ref="BM13:BM15"/>
+    <mergeCell ref="BN13:BN15"/>
+    <mergeCell ref="BO13:BO15"/>
+    <mergeCell ref="BP13:BP15"/>
+    <mergeCell ref="BQ13:BQ15"/>
+    <mergeCell ref="BR13:BR15"/>
+    <mergeCell ref="BS13:BS15"/>
+    <mergeCell ref="BT13:BT15"/>
+    <mergeCell ref="BU13:BU15"/>
+    <mergeCell ref="BV13:BV15"/>
+    <mergeCell ref="BW13:BW15"/>
+    <mergeCell ref="BX13:BX15"/>
+    <mergeCell ref="CA13:CA15"/>
+    <mergeCell ref="EB13:EB15"/>
+    <mergeCell ref="EC13:EC15"/>
+    <mergeCell ref="AK13:AK15"/>
+    <mergeCell ref="AL13:AL15"/>
+    <mergeCell ref="AM13:AM15"/>
+    <mergeCell ref="AN13:AN15"/>
+    <mergeCell ref="AO13:AO15"/>
+    <mergeCell ref="ED13:ED15"/>
+    <mergeCell ref="EE13:EE15"/>
+    <mergeCell ref="AP13:AP15"/>
+    <mergeCell ref="AQ13:AQ15"/>
+    <mergeCell ref="AR13:AR15"/>
+    <mergeCell ref="AS13:AS15"/>
+    <mergeCell ref="AT13:AT15"/>
+    <mergeCell ref="AU13:AU15"/>
+    <mergeCell ref="AV13:AV15"/>
+    <mergeCell ref="AW13:AW15"/>
+    <mergeCell ref="AX13:AX15"/>
+    <mergeCell ref="AY13:AY15"/>
+    <mergeCell ref="AZ13:AZ15"/>
+    <mergeCell ref="BA13:BA15"/>
+    <mergeCell ref="BB13:BB15"/>
+    <mergeCell ref="BY13:BY15"/>
+    <mergeCell ref="BZ13:BZ15"/>
+    <mergeCell ref="EF13:EF15"/>
+    <mergeCell ref="EG13:EG15"/>
+    <mergeCell ref="EO13:EO15"/>
+    <mergeCell ref="EP13:EP15"/>
+    <mergeCell ref="EQ13:EQ15"/>
+    <mergeCell ref="EH13:EH15"/>
+    <mergeCell ref="EI13:EI15"/>
+    <mergeCell ref="EJ13:EJ15"/>
+    <mergeCell ref="EK13:EK15"/>
+    <mergeCell ref="EL13:EL15"/>
+    <mergeCell ref="EM13:EM15"/>
+    <mergeCell ref="EN13:EN15"/>
+    <mergeCell ref="CB13:CB15"/>
+    <mergeCell ref="CC13:CC15"/>
+    <mergeCell ref="CK13:CK15"/>
+    <mergeCell ref="DJ11:DL11"/>
+    <mergeCell ref="CL13:CL15"/>
+    <mergeCell ref="CM13:CM15"/>
+    <mergeCell ref="CN13:CN15"/>
+    <mergeCell ref="CO13:CO15"/>
+    <mergeCell ref="CD13:CD15"/>
+    <mergeCell ref="CE13:CE15"/>
+    <mergeCell ref="CF13:CF15"/>
+    <mergeCell ref="CG13:CG15"/>
+    <mergeCell ref="CH13:CH15"/>
+    <mergeCell ref="CI13:CI15"/>
+    <mergeCell ref="CJ13:CJ15"/>
+    <mergeCell ref="CZ11:CZ12"/>
+    <mergeCell ref="DA11:DC11"/>
+    <mergeCell ref="DD11:DF11"/>
+    <mergeCell ref="DG11:DI11"/>
+    <mergeCell ref="BY10:CA12"/>
+    <mergeCell ref="CD11:CD12"/>
+    <mergeCell ref="CE11:CE12"/>
+    <mergeCell ref="CF11:CF12"/>
+    <mergeCell ref="CG11:CG12"/>
+    <mergeCell ref="CH11:CH12"/>
+    <mergeCell ref="EN10:EP10"/>
+    <mergeCell ref="EN11:EN12"/>
+    <mergeCell ref="EO11:EO12"/>
+    <mergeCell ref="EP11:EP12"/>
+    <mergeCell ref="EF11:EF12"/>
+    <mergeCell ref="DR11:DR12"/>
+    <mergeCell ref="DS11:DS12"/>
+    <mergeCell ref="DT11:DT12"/>
+    <mergeCell ref="DU11:DU12"/>
+    <mergeCell ref="DV10:DV12"/>
+    <mergeCell ref="EA11:EA12"/>
+    <mergeCell ref="EB11:EB12"/>
+    <mergeCell ref="ED11:ED12"/>
+    <mergeCell ref="EE11:EE12"/>
+    <mergeCell ref="DR10:DU10"/>
+    <mergeCell ref="CP11:CP12"/>
+    <mergeCell ref="CQ11:CQ12"/>
+    <mergeCell ref="CY11:CY12"/>
+    <mergeCell ref="EQ11:EQ12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="AH11:AH12"/>
+    <mergeCell ref="AI11:AI12"/>
+    <mergeCell ref="AJ11:AJ12"/>
+    <mergeCell ref="AX11:AX12"/>
+    <mergeCell ref="AY11:AY12"/>
+    <mergeCell ref="BM11:BN11"/>
+    <mergeCell ref="BO11:BP11"/>
+    <mergeCell ref="CB11:CB12"/>
+    <mergeCell ref="CC11:CC12"/>
+    <mergeCell ref="CT11:CT12"/>
+    <mergeCell ref="CU11:CU12"/>
+    <mergeCell ref="CV11:CV12"/>
+    <mergeCell ref="CW11:CW12"/>
+    <mergeCell ref="CX11:CX12"/>
+    <mergeCell ref="DY11:DY12"/>
+    <mergeCell ref="DZ11:DZ12"/>
+    <mergeCell ref="AF11:AF12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="BJ10:BJ12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:AF10"/>
+    <mergeCell ref="AG10:AJ10"/>
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="V11:X11"/>
+    <mergeCell ref="Y11:AA11"/>
+    <mergeCell ref="AB11:AD11"/>
+    <mergeCell ref="AE11:AE12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="AP11:AP12"/>
+    <mergeCell ref="AQ11:AQ12"/>
+    <mergeCell ref="AS11:AS12"/>
+    <mergeCell ref="AT11:AT12"/>
+    <mergeCell ref="AU11:AU12"/>
+    <mergeCell ref="AV11:AV12"/>
+    <mergeCell ref="AK10:AK12"/>
+    <mergeCell ref="AL10:AL12"/>
+    <mergeCell ref="AM10:AM12"/>
+    <mergeCell ref="AN10:AQ10"/>
+    <mergeCell ref="AR10:AR12"/>
+    <mergeCell ref="AS10:AV10"/>
+    <mergeCell ref="AO11:AO12"/>
+    <mergeCell ref="BQ11:BR11"/>
+    <mergeCell ref="BS11:BT11"/>
+    <mergeCell ref="BU11:BV11"/>
+    <mergeCell ref="BW11:BX11"/>
+    <mergeCell ref="BK10:BK12"/>
+    <mergeCell ref="BL10:BL12"/>
+    <mergeCell ref="BM10:BR10"/>
+    <mergeCell ref="BS10:BX10"/>
+    <mergeCell ref="DQ11:DQ12"/>
+    <mergeCell ref="CR11:CR12"/>
+    <mergeCell ref="CS11:CS12"/>
+    <mergeCell ref="CB10:CD10"/>
+    <mergeCell ref="CE10:CM10"/>
+    <mergeCell ref="CN10:CO10"/>
+    <mergeCell ref="CP10:CR10"/>
+    <mergeCell ref="CS10:DQ10"/>
+    <mergeCell ref="DP11:DP12"/>
+    <mergeCell ref="CI11:CI12"/>
+    <mergeCell ref="CJ11:CJ12"/>
+    <mergeCell ref="CK11:CK12"/>
+    <mergeCell ref="CL11:CL12"/>
+    <mergeCell ref="CM11:CM12"/>
+    <mergeCell ref="CN11:CN12"/>
+    <mergeCell ref="CO11:CO12"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="EM10:EM12"/>
@@ -3685,189 +3873,6 @@
     <mergeCell ref="ED10:EG10"/>
     <mergeCell ref="EH10:EH12"/>
     <mergeCell ref="DM11:DO11"/>
-    <mergeCell ref="BQ11:BR11"/>
-    <mergeCell ref="BS11:BT11"/>
-    <mergeCell ref="BU11:BV11"/>
-    <mergeCell ref="BW11:BX11"/>
-    <mergeCell ref="BK10:BK12"/>
-    <mergeCell ref="BL10:BL12"/>
-    <mergeCell ref="BM10:BR10"/>
-    <mergeCell ref="BS10:BX10"/>
-    <mergeCell ref="DQ11:DQ12"/>
-    <mergeCell ref="CR11:CR12"/>
-    <mergeCell ref="CS11:CS12"/>
-    <mergeCell ref="CB10:CD10"/>
-    <mergeCell ref="CE10:CM10"/>
-    <mergeCell ref="CN10:CO10"/>
-    <mergeCell ref="CP10:CR10"/>
-    <mergeCell ref="CS10:DQ10"/>
-    <mergeCell ref="DP11:DP12"/>
-    <mergeCell ref="CI11:CI12"/>
-    <mergeCell ref="CJ11:CJ12"/>
-    <mergeCell ref="CK11:CK12"/>
-    <mergeCell ref="CL11:CL12"/>
-    <mergeCell ref="CM11:CM12"/>
-    <mergeCell ref="CN11:CN12"/>
-    <mergeCell ref="CO11:CO12"/>
-    <mergeCell ref="AP11:AP12"/>
-    <mergeCell ref="AQ11:AQ12"/>
-    <mergeCell ref="AS11:AS12"/>
-    <mergeCell ref="AT11:AT12"/>
-    <mergeCell ref="AU11:AU12"/>
-    <mergeCell ref="AV11:AV12"/>
-    <mergeCell ref="AK10:AK12"/>
-    <mergeCell ref="AL10:AL12"/>
-    <mergeCell ref="AM10:AM12"/>
-    <mergeCell ref="AN10:AQ10"/>
-    <mergeCell ref="AR10:AR12"/>
-    <mergeCell ref="AS10:AV10"/>
-    <mergeCell ref="AO11:AO12"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:AF10"/>
-    <mergeCell ref="AG10:AJ10"/>
-    <mergeCell ref="AN11:AN12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="S11:U11"/>
-    <mergeCell ref="V11:X11"/>
-    <mergeCell ref="Y11:AA11"/>
-    <mergeCell ref="AB11:AD11"/>
-    <mergeCell ref="AE11:AE12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="EQ11:EQ12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="AG11:AG12"/>
-    <mergeCell ref="AH11:AH12"/>
-    <mergeCell ref="AI11:AI12"/>
-    <mergeCell ref="AJ11:AJ12"/>
-    <mergeCell ref="AX11:AX12"/>
-    <mergeCell ref="AY11:AY12"/>
-    <mergeCell ref="BM11:BN11"/>
-    <mergeCell ref="BO11:BP11"/>
-    <mergeCell ref="CB11:CB12"/>
-    <mergeCell ref="CC11:CC12"/>
-    <mergeCell ref="CT11:CT12"/>
-    <mergeCell ref="CU11:CU12"/>
-    <mergeCell ref="CV11:CV12"/>
-    <mergeCell ref="CW11:CW12"/>
-    <mergeCell ref="CX11:CX12"/>
-    <mergeCell ref="DY11:DY12"/>
-    <mergeCell ref="DZ11:DZ12"/>
-    <mergeCell ref="AF11:AF12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="BJ10:BJ12"/>
-    <mergeCell ref="BY10:CA12"/>
-    <mergeCell ref="CD11:CD12"/>
-    <mergeCell ref="CE11:CE12"/>
-    <mergeCell ref="CF11:CF12"/>
-    <mergeCell ref="CG11:CG12"/>
-    <mergeCell ref="CH11:CH12"/>
-    <mergeCell ref="EN10:EP10"/>
-    <mergeCell ref="EN11:EN12"/>
-    <mergeCell ref="EO11:EO12"/>
-    <mergeCell ref="EP11:EP12"/>
-    <mergeCell ref="EF11:EF12"/>
-    <mergeCell ref="DR11:DR12"/>
-    <mergeCell ref="DS11:DS12"/>
-    <mergeCell ref="DT11:DT12"/>
-    <mergeCell ref="DU11:DU12"/>
-    <mergeCell ref="DV10:DV12"/>
-    <mergeCell ref="EA11:EA12"/>
-    <mergeCell ref="EB11:EB12"/>
-    <mergeCell ref="ED11:ED12"/>
-    <mergeCell ref="EE11:EE12"/>
-    <mergeCell ref="DR10:DU10"/>
-    <mergeCell ref="CP11:CP12"/>
-    <mergeCell ref="CQ11:CQ12"/>
-    <mergeCell ref="CY11:CY12"/>
-    <mergeCell ref="CB13:CB15"/>
-    <mergeCell ref="CC13:CC15"/>
-    <mergeCell ref="CK13:CK15"/>
-    <mergeCell ref="DJ11:DL11"/>
-    <mergeCell ref="CL13:CL15"/>
-    <mergeCell ref="CM13:CM15"/>
-    <mergeCell ref="CN13:CN15"/>
-    <mergeCell ref="CO13:CO15"/>
-    <mergeCell ref="CD13:CD15"/>
-    <mergeCell ref="CE13:CE15"/>
-    <mergeCell ref="CF13:CF15"/>
-    <mergeCell ref="CG13:CG15"/>
-    <mergeCell ref="CH13:CH15"/>
-    <mergeCell ref="CI13:CI15"/>
-    <mergeCell ref="CJ13:CJ15"/>
-    <mergeCell ref="CZ11:CZ12"/>
-    <mergeCell ref="DA11:DC11"/>
-    <mergeCell ref="DD11:DF11"/>
-    <mergeCell ref="DG11:DI11"/>
-    <mergeCell ref="EF13:EF15"/>
-    <mergeCell ref="EG13:EG15"/>
-    <mergeCell ref="EO13:EO15"/>
-    <mergeCell ref="EP13:EP15"/>
-    <mergeCell ref="EQ13:EQ15"/>
-    <mergeCell ref="EH13:EH15"/>
-    <mergeCell ref="EI13:EI15"/>
-    <mergeCell ref="EJ13:EJ15"/>
-    <mergeCell ref="EK13:EK15"/>
-    <mergeCell ref="EL13:EL15"/>
-    <mergeCell ref="EM13:EM15"/>
-    <mergeCell ref="EN13:EN15"/>
-    <mergeCell ref="EB13:EB15"/>
-    <mergeCell ref="EC13:EC15"/>
-    <mergeCell ref="AK13:AK15"/>
-    <mergeCell ref="AL13:AL15"/>
-    <mergeCell ref="AM13:AM15"/>
-    <mergeCell ref="AN13:AN15"/>
-    <mergeCell ref="AO13:AO15"/>
-    <mergeCell ref="ED13:ED15"/>
-    <mergeCell ref="EE13:EE15"/>
-    <mergeCell ref="AP13:AP15"/>
-    <mergeCell ref="AQ13:AQ15"/>
-    <mergeCell ref="AR13:AR15"/>
-    <mergeCell ref="AS13:AS15"/>
-    <mergeCell ref="AT13:AT15"/>
-    <mergeCell ref="AU13:AU15"/>
-    <mergeCell ref="AV13:AV15"/>
-    <mergeCell ref="AW13:AW15"/>
-    <mergeCell ref="AX13:AX15"/>
-    <mergeCell ref="AY13:AY15"/>
-    <mergeCell ref="AZ13:AZ15"/>
-    <mergeCell ref="BA13:BA15"/>
-    <mergeCell ref="BB13:BB15"/>
-    <mergeCell ref="BY13:BY15"/>
-    <mergeCell ref="BZ13:BZ15"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="DV13:DV15"/>
-    <mergeCell ref="DW13:DW15"/>
-    <mergeCell ref="DX13:DX15"/>
-    <mergeCell ref="DY13:DY15"/>
-    <mergeCell ref="DZ13:DZ15"/>
-    <mergeCell ref="EA13:EA15"/>
-    <mergeCell ref="BK13:BK15"/>
-    <mergeCell ref="BL13:BL15"/>
-    <mergeCell ref="BM13:BM15"/>
-    <mergeCell ref="BN13:BN15"/>
-    <mergeCell ref="BO13:BO15"/>
-    <mergeCell ref="BP13:BP15"/>
-    <mergeCell ref="BQ13:BQ15"/>
-    <mergeCell ref="BR13:BR15"/>
-    <mergeCell ref="BS13:BS15"/>
-    <mergeCell ref="BT13:BT15"/>
-    <mergeCell ref="BU13:BU15"/>
-    <mergeCell ref="BV13:BV15"/>
-    <mergeCell ref="BW13:BW15"/>
-    <mergeCell ref="BX13:BX15"/>
-    <mergeCell ref="CA13:CA15"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>

</xml_diff>

<commit_message>
[feat/HD-15447] Fixed Elegible for XDR — cell CN13
</commit_message>
<xml_diff>
--- a/api/templates/results_ntp_use/en.xlsx
+++ b/api/templates/results_ntp_use/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/results_ntp_use/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D274E277-4BA3-334C-9311-61E7DE46838C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7F6E49-0D4E-E44C-88FC-9E3DC92399BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="840" yWindow="760" windowWidth="33720" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2898,7 +2898,10 @@
       <c r="CK13" s="20"/>
       <c r="CL13" s="20"/>
       <c r="CM13" s="20"/>
-      <c r="CN13" s="21"/>
+      <c r="CN13" s="21">
+        <f>AS13+AY13</f>
+        <v>0</v>
+      </c>
       <c r="CO13" s="21"/>
       <c r="CP13" s="10" t="s">
         <v>179</v>
@@ -3170,7 +3173,7 @@
         <v>0</v>
       </c>
       <c r="AF14" s="9">
-        <f>SUM(H13:U14)+AE14</f>
+        <f>SUM(H14:U14)+AE14</f>
         <v>0</v>
       </c>
       <c r="AG14" s="9" t="s">
@@ -3670,7 +3673,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A9:EQ15" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="207">
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:B12"/>

</xml_diff>

<commit_message>
[feat/HD-15447] Fixed Covid data
</commit_message>
<xml_diff>
--- a/api/templates/results_ntp_use/en.xlsx
+++ b/api/templates/results_ntp_use/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/results_ntp_use/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7F6E49-0D4E-E44C-88FC-9E3DC92399BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26D0400-45BD-B94F-8823-2E42C28D22AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="840" yWindow="760" windowWidth="33720" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -904,7 +904,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -955,13 +955,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -977,20 +970,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1" tint="0.34998626667073579"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
@@ -998,6 +977,32 @@
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1" tint="0.34998626667073579"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1239,150 +1244,150 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="3" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1626,12 +1631,26 @@
     <col min="11" max="11" width="14.5" customWidth="1"/>
     <col min="12" max="14" width="16.6640625" customWidth="1"/>
     <col min="15" max="15" width="60.6640625" customWidth="1"/>
-    <col min="31" max="32" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="10.5" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="12" customWidth="1"/>
-    <col min="36" max="36" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="37" max="41" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="46" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="51" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="9" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="11.33203125" customWidth="1"/>
+    <col min="62" max="62" width="8.83203125" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="13.5" customWidth="1"/>
     <col min="64" max="64" width="11.33203125" customWidth="1"/>
+    <col min="92" max="92" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="120" max="121" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="125" max="130" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="132" max="135" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="137" max="140" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="9" bestFit="1" customWidth="1"/>
+    <col min="142" max="144" width="8.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:152" ht="21" x14ac:dyDescent="0.25">
@@ -1805,232 +1824,232 @@
       <c r="O9" s="4"/>
     </row>
     <row r="10" spans="1:152" s="6" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="44" t="s">
+      <c r="A10" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="44" t="s">
+      <c r="C10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="45"/>
-      <c r="E10" s="48" t="s">
+      <c r="D10" s="39"/>
+      <c r="E10" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="22" t="s">
+      <c r="F10" s="18"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="23"/>
-      <c r="Q10" s="23"/>
-      <c r="R10" s="23"/>
-      <c r="S10" s="23"/>
-      <c r="T10" s="23"/>
-      <c r="U10" s="23"/>
-      <c r="V10" s="23"/>
-      <c r="W10" s="23"/>
-      <c r="X10" s="23"/>
-      <c r="Y10" s="23"/>
-      <c r="Z10" s="23"/>
-      <c r="AA10" s="23"/>
-      <c r="AB10" s="23"/>
-      <c r="AC10" s="23"/>
-      <c r="AD10" s="23"/>
-      <c r="AE10" s="23"/>
-      <c r="AF10" s="24"/>
-      <c r="AG10" s="22" t="s">
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="18"/>
+      <c r="T10" s="18"/>
+      <c r="U10" s="18"/>
+      <c r="V10" s="18"/>
+      <c r="W10" s="18"/>
+      <c r="X10" s="18"/>
+      <c r="Y10" s="18"/>
+      <c r="Z10" s="18"/>
+      <c r="AA10" s="18"/>
+      <c r="AB10" s="18"/>
+      <c r="AC10" s="18"/>
+      <c r="AD10" s="18"/>
+      <c r="AE10" s="18"/>
+      <c r="AF10" s="19"/>
+      <c r="AG10" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="AH10" s="23"/>
-      <c r="AI10" s="23"/>
-      <c r="AJ10" s="24"/>
-      <c r="AK10" s="38" t="s">
+      <c r="AH10" s="18"/>
+      <c r="AI10" s="18"/>
+      <c r="AJ10" s="19"/>
+      <c r="AK10" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="AL10" s="38" t="s">
+      <c r="AL10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="AM10" s="38" t="s">
+      <c r="AM10" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="AN10" s="37" t="s">
+      <c r="AN10" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="AO10" s="23"/>
-      <c r="AP10" s="23"/>
-      <c r="AQ10" s="24"/>
-      <c r="AR10" s="38" t="s">
+      <c r="AO10" s="18"/>
+      <c r="AP10" s="18"/>
+      <c r="AQ10" s="19"/>
+      <c r="AR10" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="AS10" s="37" t="s">
+      <c r="AS10" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="AT10" s="23"/>
-      <c r="AU10" s="23"/>
-      <c r="AV10" s="24"/>
-      <c r="AW10" s="50" t="s">
+      <c r="AT10" s="18"/>
+      <c r="AU10" s="18"/>
+      <c r="AV10" s="19"/>
+      <c r="AW10" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="AX10" s="37" t="s">
+      <c r="AX10" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="AY10" s="23"/>
-      <c r="AZ10" s="23"/>
-      <c r="BA10" s="24"/>
-      <c r="BB10" s="50" t="s">
+      <c r="AY10" s="18"/>
+      <c r="AZ10" s="18"/>
+      <c r="BA10" s="19"/>
+      <c r="BB10" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="BC10" s="36" t="s">
+      <c r="BC10" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="BD10" s="51" t="s">
+      <c r="BD10" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="BE10" s="52"/>
-      <c r="BF10" s="53"/>
-      <c r="BG10" s="57" t="s">
+      <c r="BE10" s="24"/>
+      <c r="BF10" s="25"/>
+      <c r="BG10" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="BH10" s="28"/>
-      <c r="BI10" s="29"/>
+      <c r="BH10" s="30"/>
+      <c r="BI10" s="31"/>
       <c r="BJ10" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="BK10" s="36" t="s">
+      <c r="BK10" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="BL10" s="36" t="s">
+      <c r="BL10" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="BM10" s="42" t="s">
+      <c r="BM10" s="35" t="s">
         <v>160</v>
       </c>
-      <c r="BN10" s="23"/>
-      <c r="BO10" s="23"/>
-      <c r="BP10" s="23"/>
-      <c r="BQ10" s="23"/>
-      <c r="BR10" s="24"/>
-      <c r="BS10" s="42" t="s">
+      <c r="BN10" s="18"/>
+      <c r="BO10" s="18"/>
+      <c r="BP10" s="18"/>
+      <c r="BQ10" s="18"/>
+      <c r="BR10" s="19"/>
+      <c r="BS10" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="BT10" s="23"/>
-      <c r="BU10" s="23"/>
-      <c r="BV10" s="23"/>
-      <c r="BW10" s="23"/>
-      <c r="BX10" s="24"/>
-      <c r="BY10" s="27" t="s">
+      <c r="BT10" s="18"/>
+      <c r="BU10" s="18"/>
+      <c r="BV10" s="18"/>
+      <c r="BW10" s="18"/>
+      <c r="BX10" s="19"/>
+      <c r="BY10" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="BZ10" s="28"/>
-      <c r="CA10" s="29"/>
-      <c r="CB10" s="42" t="s">
+      <c r="BZ10" s="30"/>
+      <c r="CA10" s="31"/>
+      <c r="CB10" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="CC10" s="23"/>
-      <c r="CD10" s="24"/>
-      <c r="CE10" s="42" t="s">
+      <c r="CC10" s="18"/>
+      <c r="CD10" s="19"/>
+      <c r="CE10" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="CF10" s="23"/>
-      <c r="CG10" s="23"/>
-      <c r="CH10" s="23"/>
-      <c r="CI10" s="23"/>
-      <c r="CJ10" s="23"/>
-      <c r="CK10" s="23"/>
-      <c r="CL10" s="23"/>
-      <c r="CM10" s="24"/>
-      <c r="CN10" s="42" t="s">
+      <c r="CF10" s="18"/>
+      <c r="CG10" s="18"/>
+      <c r="CH10" s="18"/>
+      <c r="CI10" s="18"/>
+      <c r="CJ10" s="18"/>
+      <c r="CK10" s="18"/>
+      <c r="CL10" s="18"/>
+      <c r="CM10" s="19"/>
+      <c r="CN10" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="CO10" s="24"/>
-      <c r="CP10" s="48" t="s">
+      <c r="CO10" s="19"/>
+      <c r="CP10" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="CQ10" s="23"/>
-      <c r="CR10" s="24"/>
-      <c r="CS10" s="22" t="s">
+      <c r="CQ10" s="18"/>
+      <c r="CR10" s="19"/>
+      <c r="CS10" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="CT10" s="23"/>
-      <c r="CU10" s="23"/>
-      <c r="CV10" s="23"/>
-      <c r="CW10" s="23"/>
-      <c r="CX10" s="23"/>
-      <c r="CY10" s="23"/>
-      <c r="CZ10" s="23"/>
-      <c r="DA10" s="23"/>
-      <c r="DB10" s="23"/>
-      <c r="DC10" s="23"/>
-      <c r="DD10" s="23"/>
-      <c r="DE10" s="23"/>
-      <c r="DF10" s="23"/>
-      <c r="DG10" s="23"/>
-      <c r="DH10" s="23"/>
-      <c r="DI10" s="23"/>
-      <c r="DJ10" s="23"/>
-      <c r="DK10" s="23"/>
-      <c r="DL10" s="23"/>
-      <c r="DM10" s="23"/>
-      <c r="DN10" s="23"/>
-      <c r="DO10" s="23"/>
-      <c r="DP10" s="23"/>
-      <c r="DQ10" s="24"/>
-      <c r="DR10" s="22" t="s">
+      <c r="CT10" s="18"/>
+      <c r="CU10" s="18"/>
+      <c r="CV10" s="18"/>
+      <c r="CW10" s="18"/>
+      <c r="CX10" s="18"/>
+      <c r="CY10" s="18"/>
+      <c r="CZ10" s="18"/>
+      <c r="DA10" s="18"/>
+      <c r="DB10" s="18"/>
+      <c r="DC10" s="18"/>
+      <c r="DD10" s="18"/>
+      <c r="DE10" s="18"/>
+      <c r="DF10" s="18"/>
+      <c r="DG10" s="18"/>
+      <c r="DH10" s="18"/>
+      <c r="DI10" s="18"/>
+      <c r="DJ10" s="18"/>
+      <c r="DK10" s="18"/>
+      <c r="DL10" s="18"/>
+      <c r="DM10" s="18"/>
+      <c r="DN10" s="18"/>
+      <c r="DO10" s="18"/>
+      <c r="DP10" s="18"/>
+      <c r="DQ10" s="19"/>
+      <c r="DR10" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="DS10" s="23"/>
-      <c r="DT10" s="23"/>
-      <c r="DU10" s="24"/>
-      <c r="DV10" s="38" t="s">
+      <c r="DS10" s="18"/>
+      <c r="DT10" s="18"/>
+      <c r="DU10" s="19"/>
+      <c r="DV10" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="DW10" s="38" t="s">
+      <c r="DW10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="DX10" s="38" t="s">
+      <c r="DX10" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="DY10" s="37" t="s">
+      <c r="DY10" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="DZ10" s="23"/>
-      <c r="EA10" s="23"/>
-      <c r="EB10" s="24"/>
-      <c r="EC10" s="38" t="s">
+      <c r="DZ10" s="18"/>
+      <c r="EA10" s="18"/>
+      <c r="EB10" s="19"/>
+      <c r="EC10" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="ED10" s="37" t="s">
+      <c r="ED10" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="EE10" s="23"/>
-      <c r="EF10" s="23"/>
-      <c r="EG10" s="24"/>
-      <c r="EH10" s="50" t="s">
+      <c r="EE10" s="18"/>
+      <c r="EF10" s="18"/>
+      <c r="EG10" s="19"/>
+      <c r="EH10" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="EI10" s="37" t="s">
+      <c r="EI10" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="EJ10" s="23"/>
-      <c r="EK10" s="23"/>
-      <c r="EL10" s="24"/>
-      <c r="EM10" s="50" t="s">
+      <c r="EJ10" s="18"/>
+      <c r="EK10" s="18"/>
+      <c r="EL10" s="19"/>
+      <c r="EM10" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="EN10" s="37" t="s">
+      <c r="EN10" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="EO10" s="23"/>
-      <c r="EP10" s="24"/>
+      <c r="EO10" s="18"/>
+      <c r="EP10" s="19"/>
       <c r="EQ10" s="7" t="s">
         <v>27</v>
       </c>
@@ -2041,335 +2060,335 @@
       <c r="EV10"/>
     </row>
     <row r="11" spans="1:152" s="6" customFormat="1" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="39"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="40" t="s">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="25" t="s">
+      <c r="G11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="49" t="s">
+      <c r="H11" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="I11" s="25" t="s">
+      <c r="I11" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="J11" s="25" t="s">
+      <c r="J11" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="K11" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="25" t="s">
+      <c r="L11" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="M11" s="25" t="s">
+      <c r="M11" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="N11" s="25" t="s">
+      <c r="N11" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="O11" s="25" t="s">
+      <c r="O11" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="P11" s="22" t="s">
+      <c r="P11" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="Q11" s="23"/>
-      <c r="R11" s="24"/>
-      <c r="S11" s="22" t="s">
+      <c r="Q11" s="18"/>
+      <c r="R11" s="19"/>
+      <c r="S11" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="T11" s="23"/>
-      <c r="U11" s="24"/>
-      <c r="V11" s="22" t="s">
+      <c r="T11" s="18"/>
+      <c r="U11" s="19"/>
+      <c r="V11" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="W11" s="23"/>
-      <c r="X11" s="24"/>
-      <c r="Y11" s="22" t="s">
+      <c r="W11" s="18"/>
+      <c r="X11" s="19"/>
+      <c r="Y11" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="Z11" s="23"/>
-      <c r="AA11" s="24"/>
-      <c r="AB11" s="22" t="s">
+      <c r="Z11" s="18"/>
+      <c r="AA11" s="19"/>
+      <c r="AB11" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="AC11" s="23"/>
-      <c r="AD11" s="24"/>
-      <c r="AE11" s="25" t="s">
+      <c r="AC11" s="18"/>
+      <c r="AD11" s="19"/>
+      <c r="AE11" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="AF11" s="25" t="s">
+      <c r="AF11" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="AG11" s="25" t="s">
+      <c r="AG11" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="AH11" s="25" t="s">
+      <c r="AH11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="AI11" s="25" t="s">
+      <c r="AI11" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="AJ11" s="25" t="s">
+      <c r="AJ11" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="AK11" s="39"/>
-      <c r="AL11" s="39"/>
-      <c r="AM11" s="39"/>
-      <c r="AN11" s="38" t="s">
+      <c r="AK11" s="12"/>
+      <c r="AL11" s="12"/>
+      <c r="AM11" s="12"/>
+      <c r="AN11" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="AO11" s="38" t="s">
+      <c r="AO11" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="AP11" s="38" t="s">
+      <c r="AP11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="AQ11" s="38" t="s">
+      <c r="AQ11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="AR11" s="39"/>
-      <c r="AS11" s="38" t="s">
+      <c r="AR11" s="12"/>
+      <c r="AS11" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="AT11" s="38" t="s">
+      <c r="AT11" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="AU11" s="38" t="s">
+      <c r="AU11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="AV11" s="38" t="s">
+      <c r="AV11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="AW11" s="32"/>
-      <c r="AX11" s="41" t="s">
+      <c r="AW11" s="15"/>
+      <c r="AX11" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="AY11" s="41" t="s">
+      <c r="AY11" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="AZ11" s="41" t="s">
+      <c r="AZ11" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="BA11" s="38" t="s">
+      <c r="BA11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="BB11" s="32"/>
-      <c r="BC11" s="39"/>
-      <c r="BD11" s="54"/>
-      <c r="BE11" s="55"/>
-      <c r="BF11" s="56"/>
-      <c r="BG11" s="33"/>
-      <c r="BH11" s="34"/>
-      <c r="BI11" s="35"/>
-      <c r="BJ11" s="39"/>
-      <c r="BK11" s="39"/>
-      <c r="BL11" s="39"/>
-      <c r="BM11" s="42" t="s">
+      <c r="BB11" s="15"/>
+      <c r="BC11" s="12"/>
+      <c r="BD11" s="26"/>
+      <c r="BE11" s="27"/>
+      <c r="BF11" s="28"/>
+      <c r="BG11" s="32"/>
+      <c r="BH11" s="33"/>
+      <c r="BI11" s="16"/>
+      <c r="BJ11" s="12"/>
+      <c r="BK11" s="12"/>
+      <c r="BL11" s="12"/>
+      <c r="BM11" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="BN11" s="24"/>
-      <c r="BO11" s="42" t="s">
+      <c r="BN11" s="19"/>
+      <c r="BO11" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="BP11" s="24"/>
-      <c r="BQ11" s="42" t="s">
+      <c r="BP11" s="19"/>
+      <c r="BQ11" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="BR11" s="24"/>
-      <c r="BS11" s="42" t="s">
+      <c r="BR11" s="19"/>
+      <c r="BS11" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="BT11" s="24"/>
-      <c r="BU11" s="42" t="s">
+      <c r="BT11" s="19"/>
+      <c r="BU11" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="BV11" s="24"/>
-      <c r="BW11" s="42" t="s">
+      <c r="BV11" s="19"/>
+      <c r="BW11" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="BX11" s="24"/>
-      <c r="BY11" s="30"/>
-      <c r="BZ11" s="31"/>
-      <c r="CA11" s="32"/>
-      <c r="CB11" s="36" t="s">
+      <c r="BX11" s="19"/>
+      <c r="BY11" s="45"/>
+      <c r="BZ11" s="46"/>
+      <c r="CA11" s="15"/>
+      <c r="CB11" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="CC11" s="36" t="s">
+      <c r="CC11" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="CD11" s="36" t="s">
+      <c r="CD11" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="CE11" s="36" t="s">
+      <c r="CE11" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="CF11" s="36" t="s">
+      <c r="CF11" s="22" t="s">
         <v>171</v>
       </c>
-      <c r="CG11" s="36" t="s">
+      <c r="CG11" s="22" t="s">
         <v>172</v>
       </c>
-      <c r="CH11" s="36" t="s">
+      <c r="CH11" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="CI11" s="36" t="s">
+      <c r="CI11" s="22" t="s">
         <v>174</v>
       </c>
-      <c r="CJ11" s="36" t="s">
+      <c r="CJ11" s="22" t="s">
         <v>175</v>
       </c>
-      <c r="CK11" s="36" t="s">
+      <c r="CK11" s="22" t="s">
         <v>176</v>
       </c>
-      <c r="CL11" s="36" t="s">
+      <c r="CL11" s="22" t="s">
         <v>177</v>
       </c>
-      <c r="CM11" s="36" t="s">
+      <c r="CM11" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="CN11" s="36" t="s">
+      <c r="CN11" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="CO11" s="36" t="s">
+      <c r="CO11" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="CP11" s="40" t="s">
+      <c r="CP11" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="CQ11" s="25" t="s">
+      <c r="CQ11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="CR11" s="25" t="s">
+      <c r="CR11" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="CS11" s="49" t="s">
+      <c r="CS11" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="CT11" s="25" t="s">
+      <c r="CT11" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="CU11" s="25" t="s">
+      <c r="CU11" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="CV11" s="25" t="s">
+      <c r="CV11" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="CW11" s="25" t="s">
+      <c r="CW11" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="CX11" s="25" t="s">
+      <c r="CX11" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="CY11" s="25" t="s">
+      <c r="CY11" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="CZ11" s="25" t="s">
+      <c r="CZ11" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="DA11" s="22" t="s">
+      <c r="DA11" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="DB11" s="23"/>
-      <c r="DC11" s="24"/>
-      <c r="DD11" s="22" t="s">
+      <c r="DB11" s="18"/>
+      <c r="DC11" s="19"/>
+      <c r="DD11" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="DE11" s="23"/>
-      <c r="DF11" s="24"/>
-      <c r="DG11" s="22" t="s">
+      <c r="DE11" s="18"/>
+      <c r="DF11" s="19"/>
+      <c r="DG11" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="DH11" s="23"/>
-      <c r="DI11" s="24"/>
-      <c r="DJ11" s="22" t="s">
+      <c r="DH11" s="18"/>
+      <c r="DI11" s="19"/>
+      <c r="DJ11" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="DK11" s="23"/>
-      <c r="DL11" s="24"/>
-      <c r="DM11" s="22" t="s">
+      <c r="DK11" s="18"/>
+      <c r="DL11" s="19"/>
+      <c r="DM11" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="DN11" s="23"/>
-      <c r="DO11" s="24"/>
-      <c r="DP11" s="25" t="s">
+      <c r="DN11" s="18"/>
+      <c r="DO11" s="19"/>
+      <c r="DP11" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="DQ11" s="25" t="s">
+      <c r="DQ11" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="DR11" s="25" t="s">
+      <c r="DR11" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="DS11" s="25" t="s">
+      <c r="DS11" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="DT11" s="25" t="s">
+      <c r="DT11" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="DU11" s="25" t="s">
+      <c r="DU11" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="DV11" s="39"/>
-      <c r="DW11" s="39"/>
-      <c r="DX11" s="39"/>
-      <c r="DY11" s="38" t="s">
+      <c r="DV11" s="12"/>
+      <c r="DW11" s="12"/>
+      <c r="DX11" s="12"/>
+      <c r="DY11" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="DZ11" s="38" t="s">
+      <c r="DZ11" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="EA11" s="38" t="s">
+      <c r="EA11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="EB11" s="38" t="s">
+      <c r="EB11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="EC11" s="39"/>
-      <c r="ED11" s="38" t="s">
+      <c r="EC11" s="12"/>
+      <c r="ED11" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="EE11" s="38" t="s">
+      <c r="EE11" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="EF11" s="38" t="s">
+      <c r="EF11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="EG11" s="38" t="s">
+      <c r="EG11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="EH11" s="32"/>
-      <c r="EI11" s="41" t="s">
+      <c r="EH11" s="15"/>
+      <c r="EI11" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="EJ11" s="41" t="s">
+      <c r="EJ11" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="EK11" s="41" t="s">
+      <c r="EK11" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="EL11" s="38" t="s">
+      <c r="EL11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="EM11" s="32"/>
-      <c r="EN11" s="38" t="s">
+      <c r="EM11" s="15"/>
+      <c r="EN11" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="EO11" s="38" t="s">
+      <c r="EO11" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="EP11" s="38" t="s">
+      <c r="EP11" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="EQ11" s="36" t="s">
+      <c r="EQ11" s="22" t="s">
         <v>52</v>
       </c>
       <c r="ER11"/>
@@ -2379,91 +2398,91 @@
       <c r="EV11"/>
     </row>
     <row r="12" spans="1:152" s="6" customFormat="1" ht="79.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="26"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="26"/>
-      <c r="O12" s="26"/>
-      <c r="P12" s="13" t="s">
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="Q12" s="13" t="s">
+      <c r="Q12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="R12" s="13" t="s">
+      <c r="R12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="S12" s="13" t="s">
+      <c r="S12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="T12" s="13" t="s">
+      <c r="T12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="U12" s="13" t="s">
+      <c r="U12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="V12" s="13" t="s">
+      <c r="V12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="W12" s="13" t="s">
+      <c r="W12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="X12" s="14" t="s">
+      <c r="X12" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="Y12" s="13" t="s">
+      <c r="Y12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="Z12" s="13" t="s">
+      <c r="Z12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="AA12" s="13" t="s">
+      <c r="AA12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="AB12" s="13" t="s">
+      <c r="AB12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="AC12" s="13" t="s">
+      <c r="AC12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="AD12" s="13" t="s">
+      <c r="AD12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="AE12" s="26"/>
-      <c r="AF12" s="26"/>
-      <c r="AG12" s="26"/>
-      <c r="AH12" s="26"/>
-      <c r="AI12" s="26"/>
-      <c r="AJ12" s="26"/>
-      <c r="AK12" s="26"/>
-      <c r="AL12" s="26"/>
-      <c r="AM12" s="26"/>
-      <c r="AN12" s="26"/>
-      <c r="AO12" s="26"/>
-      <c r="AP12" s="26"/>
-      <c r="AQ12" s="26"/>
-      <c r="AR12" s="26"/>
-      <c r="AS12" s="26"/>
-      <c r="AT12" s="26"/>
-      <c r="AU12" s="26"/>
-      <c r="AV12" s="26"/>
-      <c r="AW12" s="35"/>
-      <c r="AX12" s="26"/>
-      <c r="AY12" s="26"/>
-      <c r="AZ12" s="26"/>
-      <c r="BA12" s="26"/>
-      <c r="BB12" s="35"/>
-      <c r="BC12" s="26"/>
+      <c r="AE12" s="13"/>
+      <c r="AF12" s="13"/>
+      <c r="AG12" s="13"/>
+      <c r="AH12" s="13"/>
+      <c r="AI12" s="13"/>
+      <c r="AJ12" s="13"/>
+      <c r="AK12" s="13"/>
+      <c r="AL12" s="13"/>
+      <c r="AM12" s="13"/>
+      <c r="AN12" s="13"/>
+      <c r="AO12" s="13"/>
+      <c r="AP12" s="13"/>
+      <c r="AQ12" s="13"/>
+      <c r="AR12" s="13"/>
+      <c r="AS12" s="13"/>
+      <c r="AT12" s="13"/>
+      <c r="AU12" s="13"/>
+      <c r="AV12" s="13"/>
+      <c r="AW12" s="16"/>
+      <c r="AX12" s="13"/>
+      <c r="AY12" s="13"/>
+      <c r="AZ12" s="13"/>
+      <c r="BA12" s="13"/>
+      <c r="BB12" s="16"/>
+      <c r="BC12" s="13"/>
       <c r="BD12" s="8" t="s">
         <v>55</v>
       </c>
@@ -2482,9 +2501,9 @@
       <c r="BI12" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="BJ12" s="26"/>
-      <c r="BK12" s="26"/>
-      <c r="BL12" s="26"/>
+      <c r="BJ12" s="13"/>
+      <c r="BK12" s="13"/>
+      <c r="BL12" s="13"/>
       <c r="BM12" s="8" t="s">
         <v>58</v>
       </c>
@@ -2521,107 +2540,107 @@
       <c r="BX12" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="BY12" s="33"/>
-      <c r="BZ12" s="34"/>
-      <c r="CA12" s="35"/>
-      <c r="CB12" s="26"/>
-      <c r="CC12" s="26"/>
-      <c r="CD12" s="26"/>
-      <c r="CE12" s="26"/>
-      <c r="CF12" s="26"/>
-      <c r="CG12" s="26"/>
-      <c r="CH12" s="26"/>
-      <c r="CI12" s="26"/>
-      <c r="CJ12" s="26"/>
-      <c r="CK12" s="26"/>
-      <c r="CL12" s="26"/>
-      <c r="CM12" s="26"/>
-      <c r="CN12" s="26"/>
-      <c r="CO12" s="26"/>
-      <c r="CP12" s="26"/>
-      <c r="CQ12" s="26"/>
-      <c r="CR12" s="26"/>
-      <c r="CS12" s="26"/>
-      <c r="CT12" s="26"/>
-      <c r="CU12" s="26"/>
-      <c r="CV12" s="26"/>
-      <c r="CW12" s="26"/>
-      <c r="CX12" s="26"/>
-      <c r="CY12" s="26"/>
-      <c r="CZ12" s="26"/>
-      <c r="DA12" s="13" t="s">
+      <c r="BY12" s="32"/>
+      <c r="BZ12" s="33"/>
+      <c r="CA12" s="16"/>
+      <c r="CB12" s="13"/>
+      <c r="CC12" s="13"/>
+      <c r="CD12" s="13"/>
+      <c r="CE12" s="13"/>
+      <c r="CF12" s="13"/>
+      <c r="CG12" s="13"/>
+      <c r="CH12" s="13"/>
+      <c r="CI12" s="13"/>
+      <c r="CJ12" s="13"/>
+      <c r="CK12" s="13"/>
+      <c r="CL12" s="13"/>
+      <c r="CM12" s="13"/>
+      <c r="CN12" s="13"/>
+      <c r="CO12" s="13"/>
+      <c r="CP12" s="13"/>
+      <c r="CQ12" s="13"/>
+      <c r="CR12" s="13"/>
+      <c r="CS12" s="13"/>
+      <c r="CT12" s="13"/>
+      <c r="CU12" s="13"/>
+      <c r="CV12" s="13"/>
+      <c r="CW12" s="13"/>
+      <c r="CX12" s="13"/>
+      <c r="CY12" s="13"/>
+      <c r="CZ12" s="13"/>
+      <c r="DA12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="DB12" s="13" t="s">
+      <c r="DB12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="DC12" s="13" t="s">
+      <c r="DC12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="DD12" s="13" t="s">
+      <c r="DD12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="DE12" s="13" t="s">
+      <c r="DE12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="DF12" s="13" t="s">
+      <c r="DF12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="DG12" s="13" t="s">
+      <c r="DG12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="DH12" s="13" t="s">
+      <c r="DH12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="DI12" s="14" t="s">
+      <c r="DI12" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="DJ12" s="13" t="s">
+      <c r="DJ12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="DK12" s="13" t="s">
+      <c r="DK12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="DL12" s="13" t="s">
+      <c r="DL12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="DM12" s="13" t="s">
+      <c r="DM12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="DN12" s="13" t="s">
+      <c r="DN12" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="DO12" s="13" t="s">
+      <c r="DO12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="DP12" s="26"/>
-      <c r="DQ12" s="26"/>
-      <c r="DR12" s="26"/>
-      <c r="DS12" s="26"/>
-      <c r="DT12" s="26"/>
-      <c r="DU12" s="26"/>
-      <c r="DV12" s="26"/>
-      <c r="DW12" s="26"/>
-      <c r="DX12" s="26"/>
-      <c r="DY12" s="26"/>
-      <c r="DZ12" s="26"/>
-      <c r="EA12" s="26"/>
-      <c r="EB12" s="26"/>
-      <c r="EC12" s="26"/>
-      <c r="ED12" s="26"/>
-      <c r="EE12" s="26"/>
-      <c r="EF12" s="26"/>
-      <c r="EG12" s="26"/>
-      <c r="EH12" s="35"/>
-      <c r="EI12" s="26"/>
-      <c r="EJ12" s="26"/>
-      <c r="EK12" s="26"/>
-      <c r="EL12" s="26"/>
-      <c r="EM12" s="35"/>
-      <c r="EN12" s="26"/>
-      <c r="EO12" s="26"/>
-      <c r="EP12" s="26"/>
-      <c r="EQ12" s="26"/>
+      <c r="DP12" s="13"/>
+      <c r="DQ12" s="13"/>
+      <c r="DR12" s="13"/>
+      <c r="DS12" s="13"/>
+      <c r="DT12" s="13"/>
+      <c r="DU12" s="13"/>
+      <c r="DV12" s="13"/>
+      <c r="DW12" s="13"/>
+      <c r="DX12" s="13"/>
+      <c r="DY12" s="13"/>
+      <c r="DZ12" s="13"/>
+      <c r="EA12" s="13"/>
+      <c r="EB12" s="13"/>
+      <c r="EC12" s="13"/>
+      <c r="ED12" s="13"/>
+      <c r="EE12" s="13"/>
+      <c r="EF12" s="13"/>
+      <c r="EG12" s="13"/>
+      <c r="EH12" s="16"/>
+      <c r="EI12" s="13"/>
+      <c r="EJ12" s="13"/>
+      <c r="EK12" s="13"/>
+      <c r="EL12" s="13"/>
+      <c r="EM12" s="16"/>
+      <c r="EN12" s="13"/>
+      <c r="EO12" s="13"/>
+      <c r="EP12" s="13"/>
+      <c r="EQ12" s="13"/>
       <c r="ER12"/>
       <c r="ES12"/>
       <c r="ET12"/>
@@ -2629,1043 +2648,1043 @@
       <c r="EV12"/>
     </row>
     <row r="13" spans="1:152" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="47" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="47" t="s">
         <v>259</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="49">
         <f>SUM(E13:F13)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="I13" s="49" t="s">
         <v>75</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="49" t="s">
         <v>78</v>
       </c>
-      <c r="K13" s="11" t="s">
+      <c r="K13" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="L13" s="11" t="s">
+      <c r="L13" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="M13" s="11" t="s">
+      <c r="M13" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="N13" s="11" t="s">
+      <c r="N13" s="49" t="s">
         <v>89</v>
       </c>
-      <c r="O13" s="11" t="s">
+      <c r="O13" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="P13" s="11" t="s">
+      <c r="P13" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="Q13" s="11" t="s">
+      <c r="Q13" s="49" t="s">
         <v>96</v>
       </c>
-      <c r="R13" s="11" t="s">
+      <c r="R13" s="49" t="s">
         <v>97</v>
       </c>
-      <c r="S13" s="11" t="s">
+      <c r="S13" s="49" t="s">
         <v>103</v>
       </c>
-      <c r="T13" s="11" t="s">
+      <c r="T13" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="U13" s="11" t="s">
+      <c r="U13" s="49" t="s">
         <v>109</v>
       </c>
-      <c r="V13" s="11" t="s">
+      <c r="V13" s="49" t="s">
         <v>112</v>
       </c>
-      <c r="W13" s="11" t="s">
+      <c r="W13" s="49" t="s">
         <v>228</v>
       </c>
-      <c r="X13" s="11" t="s">
+      <c r="X13" s="49" t="s">
         <v>117</v>
       </c>
-      <c r="Y13" s="11" t="s">
+      <c r="Y13" s="49" t="s">
         <v>120</v>
       </c>
-      <c r="Z13" s="11" t="s">
+      <c r="Z13" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="AA13" s="11" t="s">
+      <c r="AA13" s="49" t="s">
         <v>126</v>
       </c>
-      <c r="AB13" s="11" t="s">
+      <c r="AB13" s="49" t="s">
         <v>129</v>
       </c>
-      <c r="AC13" s="11" t="s">
+      <c r="AC13" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="AD13" s="11"/>
-      <c r="AE13" s="9">
+      <c r="AD13" s="49"/>
+      <c r="AE13" s="50">
         <f>SUM(V13:AC13)</f>
         <v>0</v>
       </c>
-      <c r="AF13" s="9">
+      <c r="AF13" s="50">
         <f>SUM(H13:U13)+AE13</f>
         <v>0</v>
       </c>
-      <c r="AG13" s="9" t="s">
+      <c r="AG13" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="AH13" s="9" t="s">
+      <c r="AH13" s="50" t="s">
         <v>140</v>
       </c>
-      <c r="AI13" s="9" t="s">
+      <c r="AI13" s="50" t="s">
         <v>141</v>
       </c>
-      <c r="AJ13" s="9">
+      <c r="AJ13" s="50">
         <f>SUM(AG13:AI13)</f>
         <v>0</v>
       </c>
-      <c r="AK13" s="20">
+      <c r="AK13" s="51">
         <f>G13+AJ13</f>
         <v>0</v>
       </c>
-      <c r="AL13" s="20">
+      <c r="AL13" s="51">
         <f>AF13</f>
         <v>0</v>
       </c>
-      <c r="AM13" s="20">
+      <c r="AM13" s="51">
         <f>AK13+AL13</f>
         <v>0</v>
       </c>
-      <c r="AN13" s="20">
+      <c r="AN13" s="51">
         <f>G14+AJ14-G15-AJ15</f>
         <v>0</v>
       </c>
-      <c r="AO13" s="20">
+      <c r="AO13" s="51">
         <f>G15+AJ15</f>
         <v>0</v>
       </c>
-      <c r="AP13" s="20" t="s">
+      <c r="AP13" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="AQ13" s="20" t="s">
+      <c r="AQ13" s="51" t="s">
         <v>286</v>
       </c>
-      <c r="AR13" s="20">
+      <c r="AR13" s="51">
         <f>AK13-G14-AJ14</f>
         <v>0</v>
       </c>
-      <c r="AS13" s="20">
+      <c r="AS13" s="51">
         <f>+AF14-AF15</f>
         <v>0</v>
       </c>
-      <c r="AT13" s="20">
+      <c r="AT13" s="51">
         <f>AF15</f>
         <v>0</v>
       </c>
-      <c r="AU13" s="20" t="s">
+      <c r="AU13" s="51" t="s">
         <v>145</v>
       </c>
-      <c r="AV13" s="20">
+      <c r="AV13" s="51">
         <f>AF15</f>
         <v>0</v>
       </c>
-      <c r="AW13" s="20">
+      <c r="AW13" s="51">
         <f>AL13-AF14</f>
         <v>0</v>
       </c>
-      <c r="AX13" s="20">
+      <c r="AX13" s="51">
         <f>AN13+AS13</f>
         <v>0</v>
       </c>
-      <c r="AY13" s="20">
+      <c r="AY13" s="51">
         <f>AO13+AT13</f>
         <v>0</v>
       </c>
-      <c r="AZ13" s="20" t="e">
+      <c r="AZ13" s="51" t="e">
         <f>AP13+AU13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BA13" s="20" t="e">
+      <c r="BA13" s="51" t="e">
         <f>AQ13+AV13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="BB13" s="20">
+      <c r="BB13" s="51">
         <f>AR13+AW13</f>
         <v>0</v>
       </c>
-      <c r="BC13" s="16" t="s">
+      <c r="BC13" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="BD13" s="15" t="s">
+      <c r="BD13" s="53" t="s">
         <v>146</v>
       </c>
-      <c r="BE13" s="15" t="s">
+      <c r="BE13" s="53" t="s">
         <v>147</v>
       </c>
-      <c r="BF13" s="15" t="s">
+      <c r="BF13" s="53" t="s">
         <v>148</v>
       </c>
-      <c r="BG13" s="15" t="s">
+      <c r="BG13" s="53" t="s">
         <v>149</v>
       </c>
-      <c r="BH13" s="15" t="s">
+      <c r="BH13" s="53" t="s">
         <v>150</v>
       </c>
-      <c r="BI13" s="15" t="s">
+      <c r="BI13" s="53" t="s">
         <v>151</v>
       </c>
-      <c r="BJ13" s="15">
+      <c r="BJ13" s="53">
         <f>SUM(BD13:BI13)</f>
         <v>0</v>
       </c>
-      <c r="BK13" s="20"/>
-      <c r="BL13" s="20"/>
-      <c r="BM13" s="20" t="s">
+      <c r="BK13" s="51"/>
+      <c r="BL13" s="51"/>
+      <c r="BM13" s="51" t="s">
         <v>263</v>
       </c>
-      <c r="BN13" s="20" t="s">
+      <c r="BN13" s="51" t="s">
         <v>264</v>
       </c>
-      <c r="BO13" s="20" t="s">
+      <c r="BO13" s="51" t="s">
         <v>265</v>
       </c>
-      <c r="BP13" s="20" t="s">
+      <c r="BP13" s="51" t="s">
         <v>266</v>
       </c>
-      <c r="BQ13" s="20" t="s">
+      <c r="BQ13" s="51" t="s">
         <v>267</v>
       </c>
-      <c r="BR13" s="20" t="s">
+      <c r="BR13" s="51" t="s">
         <v>268</v>
       </c>
-      <c r="BS13" s="20" t="s">
+      <c r="BS13" s="51" t="s">
         <v>269</v>
       </c>
-      <c r="BT13" s="20" t="s">
+      <c r="BT13" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="BU13" s="20" t="s">
+      <c r="BU13" s="51" t="s">
         <v>271</v>
       </c>
-      <c r="BV13" s="20" t="s">
+      <c r="BV13" s="51" t="s">
         <v>272</v>
       </c>
-      <c r="BW13" s="20" t="s">
+      <c r="BW13" s="51" t="s">
         <v>273</v>
       </c>
-      <c r="BX13" s="20" t="s">
+      <c r="BX13" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="BY13" s="20" t="s">
+      <c r="BY13" s="51" t="s">
         <v>275</v>
       </c>
-      <c r="BZ13" s="20" t="s">
+      <c r="BZ13" s="51" t="s">
         <v>276</v>
       </c>
-      <c r="CA13" s="20" t="s">
+      <c r="CA13" s="51" t="s">
         <v>277</v>
       </c>
-      <c r="CB13" s="20" t="s">
+      <c r="CB13" s="51" t="s">
         <v>278</v>
       </c>
-      <c r="CC13" s="20" t="s">
+      <c r="CC13" s="51" t="s">
         <v>279</v>
       </c>
-      <c r="CD13" s="20" t="s">
+      <c r="CD13" s="51" t="s">
         <v>280</v>
       </c>
-      <c r="CE13" s="20"/>
-      <c r="CF13" s="20"/>
-      <c r="CG13" s="20"/>
-      <c r="CH13" s="20"/>
-      <c r="CI13" s="20"/>
-      <c r="CJ13" s="20"/>
-      <c r="CK13" s="20"/>
-      <c r="CL13" s="20"/>
-      <c r="CM13" s="20"/>
-      <c r="CN13" s="21">
+      <c r="CE13" s="51"/>
+      <c r="CF13" s="51"/>
+      <c r="CG13" s="51"/>
+      <c r="CH13" s="51"/>
+      <c r="CI13" s="51"/>
+      <c r="CJ13" s="51"/>
+      <c r="CK13" s="51"/>
+      <c r="CL13" s="51"/>
+      <c r="CM13" s="51"/>
+      <c r="CN13" s="54">
         <f>AS13+AY13</f>
         <v>0</v>
       </c>
-      <c r="CO13" s="21"/>
-      <c r="CP13" s="10" t="s">
+      <c r="CO13" s="54"/>
+      <c r="CP13" s="48" t="s">
         <v>179</v>
       </c>
-      <c r="CQ13" s="10" t="s">
+      <c r="CQ13" s="48" t="s">
         <v>181</v>
       </c>
-      <c r="CR13" s="10">
+      <c r="CR13" s="48">
         <f>SUM(CP13:CQ13)</f>
         <v>0</v>
       </c>
-      <c r="CS13" s="10" t="s">
+      <c r="CS13" s="48" t="s">
         <v>186</v>
       </c>
-      <c r="CT13" s="10" t="s">
+      <c r="CT13" s="48" t="s">
         <v>189</v>
       </c>
-      <c r="CU13" s="10" t="s">
+      <c r="CU13" s="48" t="s">
         <v>192</v>
       </c>
-      <c r="CV13" s="10" t="s">
+      <c r="CV13" s="48" t="s">
         <v>197</v>
       </c>
-      <c r="CW13" s="10" t="s">
+      <c r="CW13" s="48" t="s">
         <v>198</v>
       </c>
-      <c r="CX13" s="10" t="s">
+      <c r="CX13" s="48" t="s">
         <v>201</v>
       </c>
-      <c r="CY13" s="10" t="s">
+      <c r="CY13" s="48" t="s">
         <v>203</v>
       </c>
-      <c r="CZ13" s="10" t="s">
+      <c r="CZ13" s="48" t="s">
         <v>206</v>
       </c>
-      <c r="DA13" s="11" t="s">
+      <c r="DA13" s="49" t="s">
         <v>209</v>
       </c>
-      <c r="DB13" s="11" t="s">
+      <c r="DB13" s="49" t="s">
         <v>210</v>
       </c>
-      <c r="DC13" s="11" t="s">
+      <c r="DC13" s="49" t="s">
         <v>213</v>
       </c>
-      <c r="DD13" s="11" t="s">
+      <c r="DD13" s="49" t="s">
         <v>216</v>
       </c>
-      <c r="DE13" s="11" t="s">
+      <c r="DE13" s="49" t="s">
         <v>219</v>
       </c>
-      <c r="DF13" s="11" t="s">
+      <c r="DF13" s="49" t="s">
         <v>222</v>
       </c>
-      <c r="DG13" s="11" t="s">
+      <c r="DG13" s="49" t="s">
         <v>225</v>
       </c>
-      <c r="DH13" s="11" t="s">
+      <c r="DH13" s="49" t="s">
         <v>229</v>
       </c>
-      <c r="DI13" s="11" t="s">
+      <c r="DI13" s="49" t="s">
         <v>232</v>
       </c>
-      <c r="DJ13" s="11" t="s">
+      <c r="DJ13" s="49" t="s">
         <v>235</v>
       </c>
-      <c r="DK13" s="11" t="s">
+      <c r="DK13" s="49" t="s">
         <v>238</v>
       </c>
-      <c r="DL13" s="11" t="s">
+      <c r="DL13" s="49" t="s">
         <v>241</v>
       </c>
-      <c r="DM13" s="11" t="s">
+      <c r="DM13" s="49" t="s">
         <v>244</v>
       </c>
-      <c r="DN13" s="11" t="s">
+      <c r="DN13" s="49" t="s">
         <v>247</v>
       </c>
-      <c r="DO13" s="12"/>
-      <c r="DP13" s="9">
+      <c r="DO13" s="55"/>
+      <c r="DP13" s="50">
         <f>SUM(DG13:DN13)</f>
         <v>0</v>
       </c>
-      <c r="DQ13" s="9">
+      <c r="DQ13" s="50">
         <f>SUM(CS13:DF13)+DP13</f>
         <v>0</v>
       </c>
-      <c r="DR13" s="9" t="s">
+      <c r="DR13" s="50" t="s">
         <v>250</v>
       </c>
-      <c r="DS13" s="9" t="s">
+      <c r="DS13" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="DT13" s="9" t="s">
+      <c r="DT13" s="50" t="s">
         <v>256</v>
       </c>
-      <c r="DU13" s="9">
+      <c r="DU13" s="50">
         <f>SUM(DR13:DT13)</f>
         <v>0</v>
       </c>
-      <c r="DV13" s="20">
+      <c r="DV13" s="51">
         <f>SUM(CR13:DU13)</f>
         <v>0</v>
       </c>
-      <c r="DW13" s="20">
+      <c r="DW13" s="51">
         <f>DQ13</f>
         <v>0</v>
       </c>
-      <c r="DX13" s="20">
+      <c r="DX13" s="51">
         <f>DV13+DW13</f>
         <v>0</v>
       </c>
-      <c r="DY13" s="20">
+      <c r="DY13" s="51">
         <f>CR14+DQ14-CR15-DQ15</f>
         <v>0</v>
       </c>
-      <c r="DZ13" s="20">
+      <c r="DZ13" s="51">
         <f>CR15+DQ15</f>
         <v>0</v>
       </c>
-      <c r="EA13" s="20" t="s">
+      <c r="EA13" s="51" t="s">
         <v>281</v>
       </c>
-      <c r="EB13" s="20">
+      <c r="EB13" s="51">
         <f>DP15</f>
         <v>0</v>
       </c>
-      <c r="EC13" s="20">
+      <c r="EC13" s="51">
         <f>DV13-DU14-CR14</f>
         <v>0</v>
       </c>
-      <c r="ED13" s="20">
+      <c r="ED13" s="51">
         <f>+DQ14-DQ15</f>
         <v>0</v>
       </c>
-      <c r="EE13" s="20">
+      <c r="EE13" s="51">
         <f>DQ15</f>
         <v>0</v>
       </c>
-      <c r="EF13" s="20" t="s">
+      <c r="EF13" s="51" t="s">
         <v>282</v>
       </c>
-      <c r="EG13" s="20">
+      <c r="EG13" s="51">
         <f>DQ15</f>
         <v>0</v>
       </c>
-      <c r="EH13" s="20">
+      <c r="EH13" s="51">
         <f>DW13-DQ14</f>
         <v>0</v>
       </c>
-      <c r="EI13" s="20">
+      <c r="EI13" s="51">
         <f>DY13+ED13</f>
         <v>0</v>
       </c>
-      <c r="EJ13" s="20">
+      <c r="EJ13" s="51">
         <f>DZ13-EE13</f>
         <v>0</v>
       </c>
-      <c r="EK13" s="20" t="e">
+      <c r="EK13" s="51" t="e">
         <f>EA13+EF13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="EL13" s="20">
+      <c r="EL13" s="51">
         <f>EB13+EG13</f>
         <v>0</v>
       </c>
-      <c r="EM13" s="20">
+      <c r="EM13" s="51">
         <f>EC13+EH13</f>
         <v>0</v>
       </c>
-      <c r="EN13" s="21">
+      <c r="EN13" s="54">
         <f>ED13+EJ13</f>
         <v>0</v>
       </c>
-      <c r="EO13" s="21"/>
-      <c r="EP13" s="21" t="s">
+      <c r="EO13" s="54"/>
+      <c r="EP13" s="54" t="s">
         <v>283</v>
       </c>
-      <c r="EQ13" s="20" t="str">
+      <c r="EQ13" s="51" t="str">
         <f>EP13</f>
         <v>&lt;cnt_Xdr_Total_Tests_stool&gt;</v>
       </c>
     </row>
     <row r="14" spans="1:152" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="18"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="10" t="s">
+      <c r="A14" s="47"/>
+      <c r="B14" s="56"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="49" t="s">
         <v>67</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="49" t="s">
         <v>70</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="49">
         <f>SUM(E14:F14)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="I14" s="11" t="s">
+      <c r="I14" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="J14" s="11" t="s">
+      <c r="J14" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="K14" s="11" t="s">
+      <c r="K14" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="L14" s="11" t="s">
+      <c r="L14" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="M14" s="11" t="s">
+      <c r="M14" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="N14" s="11" t="s">
+      <c r="N14" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="O14" s="11" t="s">
+      <c r="O14" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="P14" s="11" t="s">
+      <c r="P14" s="49" t="s">
         <v>98</v>
       </c>
-      <c r="Q14" s="11" t="s">
+      <c r="Q14" s="49" t="s">
         <v>99</v>
       </c>
-      <c r="R14" s="11" t="s">
+      <c r="R14" s="49" t="s">
         <v>101</v>
       </c>
-      <c r="S14" s="11" t="s">
+      <c r="S14" s="49" t="s">
         <v>104</v>
       </c>
-      <c r="T14" s="11" t="s">
+      <c r="T14" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="U14" s="11" t="s">
+      <c r="U14" s="49" t="s">
         <v>110</v>
       </c>
-      <c r="V14" s="11" t="s">
+      <c r="V14" s="49" t="s">
         <v>113</v>
       </c>
-      <c r="W14" s="11" t="s">
+      <c r="W14" s="49" t="s">
         <v>115</v>
       </c>
-      <c r="X14" s="11" t="s">
+      <c r="X14" s="49" t="s">
         <v>118</v>
       </c>
-      <c r="Y14" s="11" t="s">
+      <c r="Y14" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="Z14" s="11" t="s">
+      <c r="Z14" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="AA14" s="11" t="s">
+      <c r="AA14" s="49" t="s">
         <v>127</v>
       </c>
-      <c r="AB14" s="11" t="s">
+      <c r="AB14" s="49" t="s">
         <v>130</v>
       </c>
-      <c r="AC14" s="11" t="s">
+      <c r="AC14" s="49" t="s">
         <v>133</v>
       </c>
-      <c r="AD14" s="11"/>
-      <c r="AE14" s="9">
+      <c r="AD14" s="49"/>
+      <c r="AE14" s="50">
         <f>SUM(V14:AC14)</f>
         <v>0</v>
       </c>
-      <c r="AF14" s="9">
+      <c r="AF14" s="50">
         <f>SUM(H14:U14)+AE14</f>
         <v>0</v>
       </c>
-      <c r="AG14" s="9" t="s">
+      <c r="AG14" s="50" t="s">
         <v>136</v>
       </c>
-      <c r="AH14" s="9" t="s">
+      <c r="AH14" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="AI14" s="9" t="s">
+      <c r="AI14" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="AJ14" s="9">
+      <c r="AJ14" s="50">
         <f>SUM(AG14:AI14)</f>
         <v>0</v>
       </c>
-      <c r="AK14" s="19"/>
-      <c r="AL14" s="19"/>
-      <c r="AM14" s="19"/>
-      <c r="AN14" s="19"/>
-      <c r="AO14" s="19"/>
-      <c r="AP14" s="19"/>
-      <c r="AQ14" s="19"/>
-      <c r="AR14" s="19"/>
-      <c r="AS14" s="19"/>
-      <c r="AT14" s="19"/>
-      <c r="AU14" s="19"/>
-      <c r="AV14" s="19"/>
-      <c r="AW14" s="19"/>
-      <c r="AX14" s="19"/>
-      <c r="AY14" s="19"/>
-      <c r="AZ14" s="19"/>
-      <c r="BA14" s="19"/>
-      <c r="BB14" s="19"/>
-      <c r="BC14" s="16" t="s">
+      <c r="AK14" s="56"/>
+      <c r="AL14" s="56"/>
+      <c r="AM14" s="56"/>
+      <c r="AN14" s="56"/>
+      <c r="AO14" s="56"/>
+      <c r="AP14" s="56"/>
+      <c r="AQ14" s="56"/>
+      <c r="AR14" s="56"/>
+      <c r="AS14" s="56"/>
+      <c r="AT14" s="56"/>
+      <c r="AU14" s="56"/>
+      <c r="AV14" s="56"/>
+      <c r="AW14" s="56"/>
+      <c r="AX14" s="56"/>
+      <c r="AY14" s="56"/>
+      <c r="AZ14" s="56"/>
+      <c r="BA14" s="56"/>
+      <c r="BB14" s="56"/>
+      <c r="BC14" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="BD14" s="15" t="s">
+      <c r="BD14" s="53" t="s">
         <v>152</v>
       </c>
-      <c r="BE14" s="15" t="s">
+      <c r="BE14" s="53" t="s">
         <v>153</v>
       </c>
-      <c r="BF14" s="15" t="s">
+      <c r="BF14" s="53" t="s">
         <v>154</v>
       </c>
-      <c r="BG14" s="15" t="s">
+      <c r="BG14" s="53" t="s">
         <v>155</v>
       </c>
-      <c r="BH14" s="15" t="s">
+      <c r="BH14" s="53" t="s">
         <v>156</v>
       </c>
-      <c r="BI14" s="15" t="s">
+      <c r="BI14" s="53" t="s">
         <v>157</v>
       </c>
-      <c r="BJ14" s="15">
+      <c r="BJ14" s="53">
         <f>SUM(BD14:BI14)</f>
         <v>0</v>
       </c>
-      <c r="BK14" s="19"/>
-      <c r="BL14" s="19"/>
-      <c r="BM14" s="19"/>
-      <c r="BN14" s="19"/>
-      <c r="BO14" s="19"/>
-      <c r="BP14" s="19"/>
-      <c r="BQ14" s="19"/>
-      <c r="BR14" s="19"/>
-      <c r="BS14" s="19"/>
-      <c r="BT14" s="19"/>
-      <c r="BU14" s="19"/>
-      <c r="BV14" s="19"/>
-      <c r="BW14" s="19"/>
-      <c r="BX14" s="19"/>
-      <c r="BY14" s="19"/>
-      <c r="BZ14" s="19"/>
-      <c r="CA14" s="19"/>
-      <c r="CB14" s="19"/>
-      <c r="CC14" s="19"/>
-      <c r="CD14" s="19"/>
-      <c r="CE14" s="19"/>
-      <c r="CF14" s="19"/>
-      <c r="CG14" s="19"/>
-      <c r="CH14" s="20"/>
-      <c r="CI14" s="19"/>
-      <c r="CJ14" s="19"/>
-      <c r="CK14" s="19"/>
-      <c r="CL14" s="19"/>
-      <c r="CM14" s="19"/>
-      <c r="CN14" s="19"/>
-      <c r="CO14" s="19"/>
-      <c r="CP14" s="10" t="s">
+      <c r="BK14" s="56"/>
+      <c r="BL14" s="56"/>
+      <c r="BM14" s="56"/>
+      <c r="BN14" s="56"/>
+      <c r="BO14" s="56"/>
+      <c r="BP14" s="56"/>
+      <c r="BQ14" s="56"/>
+      <c r="BR14" s="56"/>
+      <c r="BS14" s="56"/>
+      <c r="BT14" s="56"/>
+      <c r="BU14" s="56"/>
+      <c r="BV14" s="56"/>
+      <c r="BW14" s="56"/>
+      <c r="BX14" s="56"/>
+      <c r="BY14" s="56"/>
+      <c r="BZ14" s="56"/>
+      <c r="CA14" s="56"/>
+      <c r="CB14" s="56"/>
+      <c r="CC14" s="56"/>
+      <c r="CD14" s="56"/>
+      <c r="CE14" s="56"/>
+      <c r="CF14" s="56"/>
+      <c r="CG14" s="56"/>
+      <c r="CH14" s="51"/>
+      <c r="CI14" s="56"/>
+      <c r="CJ14" s="56"/>
+      <c r="CK14" s="56"/>
+      <c r="CL14" s="56"/>
+      <c r="CM14" s="56"/>
+      <c r="CN14" s="56"/>
+      <c r="CO14" s="56"/>
+      <c r="CP14" s="48" t="s">
         <v>183</v>
       </c>
-      <c r="CQ14" s="10" t="s">
+      <c r="CQ14" s="48" t="s">
         <v>182</v>
       </c>
-      <c r="CR14" s="10">
+      <c r="CR14" s="48">
         <f>SUM(CP14:CQ14)</f>
         <v>0</v>
       </c>
-      <c r="CS14" s="10" t="s">
+      <c r="CS14" s="48" t="s">
         <v>187</v>
       </c>
-      <c r="CT14" s="10" t="s">
+      <c r="CT14" s="48" t="s">
         <v>190</v>
       </c>
-      <c r="CU14" s="10" t="s">
+      <c r="CU14" s="48" t="s">
         <v>193</v>
       </c>
-      <c r="CV14" s="10" t="s">
+      <c r="CV14" s="48" t="s">
         <v>195</v>
       </c>
-      <c r="CW14" s="10" t="s">
+      <c r="CW14" s="48" t="s">
         <v>199</v>
       </c>
-      <c r="CX14" s="10" t="s">
+      <c r="CX14" s="48" t="s">
         <v>284</v>
       </c>
-      <c r="CY14" s="10" t="s">
+      <c r="CY14" s="48" t="s">
         <v>204</v>
       </c>
-      <c r="CZ14" s="10" t="s">
+      <c r="CZ14" s="48" t="s">
         <v>207</v>
       </c>
-      <c r="DA14" s="11" t="s">
+      <c r="DA14" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="DB14" s="11" t="s">
+      <c r="DB14" s="49" t="s">
         <v>211</v>
       </c>
-      <c r="DC14" s="11" t="s">
+      <c r="DC14" s="49" t="s">
         <v>214</v>
       </c>
-      <c r="DD14" s="11" t="s">
+      <c r="DD14" s="49" t="s">
         <v>217</v>
       </c>
-      <c r="DE14" s="11" t="s">
+      <c r="DE14" s="49" t="s">
         <v>220</v>
       </c>
-      <c r="DF14" s="11" t="s">
+      <c r="DF14" s="49" t="s">
         <v>223</v>
       </c>
-      <c r="DG14" s="11" t="s">
+      <c r="DG14" s="49" t="s">
         <v>226</v>
       </c>
-      <c r="DH14" s="11" t="s">
+      <c r="DH14" s="49" t="s">
         <v>230</v>
       </c>
-      <c r="DI14" s="11" t="s">
+      <c r="DI14" s="49" t="s">
         <v>233</v>
       </c>
-      <c r="DJ14" s="11" t="s">
+      <c r="DJ14" s="49" t="s">
         <v>236</v>
       </c>
-      <c r="DK14" s="11" t="s">
+      <c r="DK14" s="49" t="s">
         <v>239</v>
       </c>
-      <c r="DL14" s="11" t="s">
+      <c r="DL14" s="49" t="s">
         <v>242</v>
       </c>
-      <c r="DM14" s="11" t="s">
+      <c r="DM14" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="DN14" s="11" t="s">
+      <c r="DN14" s="49" t="s">
         <v>248</v>
       </c>
-      <c r="DO14" s="12"/>
-      <c r="DP14" s="9">
+      <c r="DO14" s="55"/>
+      <c r="DP14" s="50">
         <f>SUM(DG14:DN14)</f>
         <v>0</v>
       </c>
-      <c r="DQ14" s="9">
+      <c r="DQ14" s="50">
         <f>SUM(CS14:DF14)+DP14</f>
         <v>0</v>
       </c>
-      <c r="DR14" s="9" t="s">
+      <c r="DR14" s="50" t="s">
         <v>251</v>
       </c>
-      <c r="DS14" s="9" t="s">
+      <c r="DS14" s="50" t="s">
         <v>254</v>
       </c>
-      <c r="DT14" s="9" t="s">
+      <c r="DT14" s="50" t="s">
         <v>257</v>
       </c>
-      <c r="DU14" s="9">
+      <c r="DU14" s="50">
         <f>SUM(DR14:DT14)</f>
         <v>0</v>
       </c>
-      <c r="DV14" s="19"/>
-      <c r="DW14" s="19"/>
-      <c r="DX14" s="19"/>
-      <c r="DY14" s="19"/>
-      <c r="DZ14" s="19"/>
-      <c r="EA14" s="19"/>
-      <c r="EB14" s="19"/>
-      <c r="EC14" s="19"/>
-      <c r="ED14" s="19"/>
-      <c r="EE14" s="19"/>
-      <c r="EF14" s="19"/>
-      <c r="EG14" s="19"/>
-      <c r="EH14" s="19"/>
-      <c r="EI14" s="19"/>
-      <c r="EJ14" s="19"/>
-      <c r="EK14" s="19"/>
-      <c r="EL14" s="19"/>
-      <c r="EM14" s="19"/>
-      <c r="EN14" s="19"/>
-      <c r="EO14" s="21"/>
-      <c r="EP14" s="19"/>
-      <c r="EQ14" s="19"/>
+      <c r="DV14" s="56"/>
+      <c r="DW14" s="56"/>
+      <c r="DX14" s="56"/>
+      <c r="DY14" s="56"/>
+      <c r="DZ14" s="56"/>
+      <c r="EA14" s="56"/>
+      <c r="EB14" s="56"/>
+      <c r="EC14" s="56"/>
+      <c r="ED14" s="56"/>
+      <c r="EE14" s="56"/>
+      <c r="EF14" s="56"/>
+      <c r="EG14" s="56"/>
+      <c r="EH14" s="56"/>
+      <c r="EI14" s="56"/>
+      <c r="EJ14" s="56"/>
+      <c r="EK14" s="56"/>
+      <c r="EL14" s="56"/>
+      <c r="EM14" s="56"/>
+      <c r="EN14" s="56"/>
+      <c r="EO14" s="54"/>
+      <c r="EP14" s="56"/>
+      <c r="EQ14" s="56"/>
     </row>
     <row r="15" spans="1:152" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="18"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="10" t="s">
+      <c r="A15" s="47"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="49">
         <f>SUM(E15:F15)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="49" t="s">
         <v>74</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="I15" s="49" t="s">
         <v>77</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="K15" s="11" t="s">
+      <c r="K15" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="L15" s="11" t="s">
+      <c r="L15" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="M15" s="11" t="s">
+      <c r="M15" s="49" t="s">
         <v>88</v>
       </c>
-      <c r="N15" s="11" t="s">
+      <c r="N15" s="49" t="s">
         <v>91</v>
       </c>
-      <c r="O15" s="11" t="s">
+      <c r="O15" s="49" t="s">
         <v>94</v>
       </c>
-      <c r="P15" s="11" t="s">
+      <c r="P15" s="49" t="s">
         <v>98</v>
       </c>
-      <c r="Q15" s="11" t="s">
+      <c r="Q15" s="49" t="s">
         <v>100</v>
       </c>
-      <c r="R15" s="11" t="s">
+      <c r="R15" s="49" t="s">
         <v>102</v>
       </c>
-      <c r="S15" s="11" t="s">
+      <c r="S15" s="49" t="s">
         <v>105</v>
       </c>
-      <c r="T15" s="11" t="s">
+      <c r="T15" s="49" t="s">
         <v>108</v>
       </c>
-      <c r="U15" s="11" t="s">
+      <c r="U15" s="49" t="s">
         <v>111</v>
       </c>
-      <c r="V15" s="11" t="s">
+      <c r="V15" s="49" t="s">
         <v>114</v>
       </c>
-      <c r="W15" s="11" t="s">
+      <c r="W15" s="49" t="s">
         <v>116</v>
       </c>
-      <c r="X15" s="11" t="s">
+      <c r="X15" s="49" t="s">
         <v>119</v>
       </c>
-      <c r="Y15" s="11" t="s">
+      <c r="Y15" s="49" t="s">
         <v>122</v>
       </c>
-      <c r="Z15" s="11" t="s">
+      <c r="Z15" s="49" t="s">
         <v>125</v>
       </c>
-      <c r="AA15" s="11" t="s">
+      <c r="AA15" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="AB15" s="11" t="s">
+      <c r="AB15" s="49" t="s">
         <v>131</v>
       </c>
-      <c r="AC15" s="11" t="s">
+      <c r="AC15" s="49" t="s">
         <v>134</v>
       </c>
-      <c r="AD15" s="11"/>
-      <c r="AE15" s="9">
+      <c r="AD15" s="49"/>
+      <c r="AE15" s="50">
         <f>SUM(V15:AC15)</f>
         <v>0</v>
       </c>
-      <c r="AF15" s="9">
+      <c r="AF15" s="50">
         <f>SUM(H15:U15)+AE15</f>
         <v>0</v>
       </c>
-      <c r="AG15" s="9" t="s">
+      <c r="AG15" s="50" t="s">
         <v>137</v>
       </c>
-      <c r="AH15" s="9" t="s">
+      <c r="AH15" s="50" t="s">
         <v>139</v>
       </c>
-      <c r="AI15" s="9" t="s">
+      <c r="AI15" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="AJ15" s="9">
+      <c r="AJ15" s="50">
         <f>SUM(AG15:AI15)</f>
         <v>0</v>
       </c>
-      <c r="AK15" s="19"/>
-      <c r="AL15" s="19"/>
-      <c r="AM15" s="19"/>
-      <c r="AN15" s="19"/>
-      <c r="AO15" s="19"/>
-      <c r="AP15" s="19"/>
-      <c r="AQ15" s="19"/>
-      <c r="AR15" s="19"/>
-      <c r="AS15" s="19"/>
-      <c r="AT15" s="19"/>
-      <c r="AU15" s="19"/>
-      <c r="AV15" s="19"/>
-      <c r="AW15" s="19"/>
-      <c r="AX15" s="19"/>
-      <c r="AY15" s="19"/>
-      <c r="AZ15" s="19"/>
-      <c r="BA15" s="19"/>
-      <c r="BB15" s="19"/>
-      <c r="BC15" s="17"/>
-      <c r="BD15" s="15"/>
-      <c r="BE15" s="15"/>
-      <c r="BF15" s="15"/>
-      <c r="BG15" s="15"/>
-      <c r="BH15" s="15"/>
-      <c r="BI15" s="15"/>
-      <c r="BJ15" s="15"/>
-      <c r="BK15" s="19"/>
-      <c r="BL15" s="19"/>
-      <c r="BM15" s="19"/>
-      <c r="BN15" s="19"/>
-      <c r="BO15" s="19"/>
-      <c r="BP15" s="19"/>
-      <c r="BQ15" s="19"/>
-      <c r="BR15" s="19"/>
-      <c r="BS15" s="19"/>
-      <c r="BT15" s="19"/>
-      <c r="BU15" s="19"/>
-      <c r="BV15" s="19"/>
-      <c r="BW15" s="19"/>
-      <c r="BX15" s="19"/>
-      <c r="BY15" s="19"/>
-      <c r="BZ15" s="19"/>
-      <c r="CA15" s="19"/>
-      <c r="CB15" s="19"/>
-      <c r="CC15" s="19"/>
-      <c r="CD15" s="19"/>
-      <c r="CE15" s="19"/>
-      <c r="CF15" s="19"/>
-      <c r="CG15" s="19"/>
-      <c r="CH15" s="20"/>
-      <c r="CI15" s="19"/>
-      <c r="CJ15" s="19"/>
-      <c r="CK15" s="19"/>
-      <c r="CL15" s="19"/>
-      <c r="CM15" s="19"/>
-      <c r="CN15" s="19"/>
-      <c r="CO15" s="19"/>
-      <c r="CP15" s="10" t="s">
+      <c r="AK15" s="56"/>
+      <c r="AL15" s="56"/>
+      <c r="AM15" s="56"/>
+      <c r="AN15" s="56"/>
+      <c r="AO15" s="56"/>
+      <c r="AP15" s="56"/>
+      <c r="AQ15" s="56"/>
+      <c r="AR15" s="56"/>
+      <c r="AS15" s="56"/>
+      <c r="AT15" s="56"/>
+      <c r="AU15" s="56"/>
+      <c r="AV15" s="56"/>
+      <c r="AW15" s="56"/>
+      <c r="AX15" s="56"/>
+      <c r="AY15" s="56"/>
+      <c r="AZ15" s="56"/>
+      <c r="BA15" s="56"/>
+      <c r="BB15" s="56"/>
+      <c r="BC15" s="57"/>
+      <c r="BD15" s="53"/>
+      <c r="BE15" s="53"/>
+      <c r="BF15" s="53"/>
+      <c r="BG15" s="53"/>
+      <c r="BH15" s="53"/>
+      <c r="BI15" s="53"/>
+      <c r="BJ15" s="53"/>
+      <c r="BK15" s="56"/>
+      <c r="BL15" s="56"/>
+      <c r="BM15" s="56"/>
+      <c r="BN15" s="56"/>
+      <c r="BO15" s="56"/>
+      <c r="BP15" s="56"/>
+      <c r="BQ15" s="56"/>
+      <c r="BR15" s="56"/>
+      <c r="BS15" s="56"/>
+      <c r="BT15" s="56"/>
+      <c r="BU15" s="56"/>
+      <c r="BV15" s="56"/>
+      <c r="BW15" s="56"/>
+      <c r="BX15" s="56"/>
+      <c r="BY15" s="56"/>
+      <c r="BZ15" s="56"/>
+      <c r="CA15" s="56"/>
+      <c r="CB15" s="56"/>
+      <c r="CC15" s="56"/>
+      <c r="CD15" s="56"/>
+      <c r="CE15" s="56"/>
+      <c r="CF15" s="56"/>
+      <c r="CG15" s="56"/>
+      <c r="CH15" s="51"/>
+      <c r="CI15" s="56"/>
+      <c r="CJ15" s="56"/>
+      <c r="CK15" s="56"/>
+      <c r="CL15" s="56"/>
+      <c r="CM15" s="56"/>
+      <c r="CN15" s="56"/>
+      <c r="CO15" s="56"/>
+      <c r="CP15" s="48" t="s">
         <v>184</v>
       </c>
-      <c r="CQ15" s="10" t="s">
+      <c r="CQ15" s="48" t="s">
         <v>185</v>
       </c>
-      <c r="CR15" s="10">
+      <c r="CR15" s="48">
         <f>SUM(CP15:CQ15)</f>
         <v>0</v>
       </c>
-      <c r="CS15" s="10" t="s">
+      <c r="CS15" s="48" t="s">
         <v>188</v>
       </c>
-      <c r="CT15" s="10" t="s">
+      <c r="CT15" s="48" t="s">
         <v>191</v>
       </c>
-      <c r="CU15" s="10" t="s">
+      <c r="CU15" s="48" t="s">
         <v>194</v>
       </c>
-      <c r="CV15" s="10" t="s">
+      <c r="CV15" s="48" t="s">
         <v>196</v>
       </c>
-      <c r="CW15" s="10" t="s">
+      <c r="CW15" s="48" t="s">
         <v>200</v>
       </c>
-      <c r="CX15" s="10" t="s">
+      <c r="CX15" s="48" t="s">
         <v>202</v>
       </c>
-      <c r="CY15" s="10" t="s">
+      <c r="CY15" s="48" t="s">
         <v>205</v>
       </c>
-      <c r="CZ15" s="10" t="s">
+      <c r="CZ15" s="48" t="s">
         <v>208</v>
       </c>
-      <c r="DA15" s="11" t="s">
+      <c r="DA15" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="DB15" s="11" t="s">
+      <c r="DB15" s="49" t="s">
         <v>212</v>
       </c>
-      <c r="DC15" s="11" t="s">
+      <c r="DC15" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="DD15" s="11" t="s">
+      <c r="DD15" s="49" t="s">
         <v>218</v>
       </c>
-      <c r="DE15" s="11" t="s">
+      <c r="DE15" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="DF15" s="11" t="s">
+      <c r="DF15" s="49" t="s">
         <v>224</v>
       </c>
-      <c r="DG15" s="11" t="s">
+      <c r="DG15" s="49" t="s">
         <v>227</v>
       </c>
-      <c r="DH15" s="11" t="s">
+      <c r="DH15" s="49" t="s">
         <v>231</v>
       </c>
-      <c r="DI15" s="11" t="s">
+      <c r="DI15" s="49" t="s">
         <v>234</v>
       </c>
-      <c r="DJ15" s="11" t="s">
+      <c r="DJ15" s="49" t="s">
         <v>237</v>
       </c>
-      <c r="DK15" s="11" t="s">
+      <c r="DK15" s="49" t="s">
         <v>240</v>
       </c>
-      <c r="DL15" s="11" t="s">
+      <c r="DL15" s="49" t="s">
         <v>243</v>
       </c>
-      <c r="DM15" s="11" t="s">
+      <c r="DM15" s="49" t="s">
         <v>246</v>
       </c>
-      <c r="DN15" s="11" t="s">
+      <c r="DN15" s="49" t="s">
         <v>249</v>
       </c>
-      <c r="DO15" s="12"/>
-      <c r="DP15" s="9">
+      <c r="DO15" s="55"/>
+      <c r="DP15" s="50">
         <f>SUM(DG15:DN15)</f>
         <v>0</v>
       </c>
-      <c r="DQ15" s="9">
+      <c r="DQ15" s="50">
         <f>SUM(CS15:DF15)+DP15</f>
         <v>0</v>
       </c>
-      <c r="DR15" s="9" t="s">
+      <c r="DR15" s="50" t="s">
         <v>252</v>
       </c>
-      <c r="DS15" s="9" t="s">
+      <c r="DS15" s="50" t="s">
         <v>255</v>
       </c>
-      <c r="DT15" s="9" t="s">
+      <c r="DT15" s="50" t="s">
         <v>258</v>
       </c>
-      <c r="DU15" s="9">
+      <c r="DU15" s="50">
         <f>SUM(DR15:DT15)</f>
         <v>0</v>
       </c>
-      <c r="DV15" s="19"/>
-      <c r="DW15" s="19"/>
-      <c r="DX15" s="19"/>
-      <c r="DY15" s="19"/>
-      <c r="DZ15" s="19"/>
-      <c r="EA15" s="19"/>
-      <c r="EB15" s="19"/>
-      <c r="EC15" s="19"/>
-      <c r="ED15" s="19"/>
-      <c r="EE15" s="19"/>
-      <c r="EF15" s="19"/>
-      <c r="EG15" s="19"/>
-      <c r="EH15" s="19"/>
-      <c r="EI15" s="19"/>
-      <c r="EJ15" s="19"/>
-      <c r="EK15" s="19"/>
-      <c r="EL15" s="19"/>
-      <c r="EM15" s="19"/>
-      <c r="EN15" s="19"/>
-      <c r="EO15" s="21"/>
-      <c r="EP15" s="19"/>
-      <c r="EQ15" s="19"/>
+      <c r="DV15" s="56"/>
+      <c r="DW15" s="56"/>
+      <c r="DX15" s="56"/>
+      <c r="DY15" s="56"/>
+      <c r="DZ15" s="56"/>
+      <c r="EA15" s="56"/>
+      <c r="EB15" s="56"/>
+      <c r="EC15" s="56"/>
+      <c r="ED15" s="56"/>
+      <c r="EE15" s="56"/>
+      <c r="EF15" s="56"/>
+      <c r="EG15" s="56"/>
+      <c r="EH15" s="56"/>
+      <c r="EI15" s="56"/>
+      <c r="EJ15" s="56"/>
+      <c r="EK15" s="56"/>
+      <c r="EL15" s="56"/>
+      <c r="EM15" s="56"/>
+      <c r="EN15" s="56"/>
+      <c r="EO15" s="54"/>
+      <c r="EP15" s="56"/>
+      <c r="EQ15" s="56"/>
     </row>
     <row r="21" spans="123:123" x14ac:dyDescent="0.2">
       <c r="DS21">
@@ -3674,6 +3693,189 @@
     </row>
   </sheetData>
   <mergeCells count="207">
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="DV13:DV15"/>
+    <mergeCell ref="DW13:DW15"/>
+    <mergeCell ref="DX13:DX15"/>
+    <mergeCell ref="DY13:DY15"/>
+    <mergeCell ref="DZ13:DZ15"/>
+    <mergeCell ref="EA13:EA15"/>
+    <mergeCell ref="BK13:BK15"/>
+    <mergeCell ref="BL13:BL15"/>
+    <mergeCell ref="BM13:BM15"/>
+    <mergeCell ref="BN13:BN15"/>
+    <mergeCell ref="BO13:BO15"/>
+    <mergeCell ref="BP13:BP15"/>
+    <mergeCell ref="BQ13:BQ15"/>
+    <mergeCell ref="BR13:BR15"/>
+    <mergeCell ref="BS13:BS15"/>
+    <mergeCell ref="BT13:BT15"/>
+    <mergeCell ref="BU13:BU15"/>
+    <mergeCell ref="BV13:BV15"/>
+    <mergeCell ref="BW13:BW15"/>
+    <mergeCell ref="BX13:BX15"/>
+    <mergeCell ref="CA13:CA15"/>
+    <mergeCell ref="EB13:EB15"/>
+    <mergeCell ref="EC13:EC15"/>
+    <mergeCell ref="AK13:AK15"/>
+    <mergeCell ref="AL13:AL15"/>
+    <mergeCell ref="AM13:AM15"/>
+    <mergeCell ref="AN13:AN15"/>
+    <mergeCell ref="AO13:AO15"/>
+    <mergeCell ref="ED13:ED15"/>
+    <mergeCell ref="EE13:EE15"/>
+    <mergeCell ref="AP13:AP15"/>
+    <mergeCell ref="AQ13:AQ15"/>
+    <mergeCell ref="AR13:AR15"/>
+    <mergeCell ref="AS13:AS15"/>
+    <mergeCell ref="AT13:AT15"/>
+    <mergeCell ref="AU13:AU15"/>
+    <mergeCell ref="AV13:AV15"/>
+    <mergeCell ref="AW13:AW15"/>
+    <mergeCell ref="AX13:AX15"/>
+    <mergeCell ref="AY13:AY15"/>
+    <mergeCell ref="AZ13:AZ15"/>
+    <mergeCell ref="BA13:BA15"/>
+    <mergeCell ref="BB13:BB15"/>
+    <mergeCell ref="BY13:BY15"/>
+    <mergeCell ref="BZ13:BZ15"/>
+    <mergeCell ref="EF13:EF15"/>
+    <mergeCell ref="EG13:EG15"/>
+    <mergeCell ref="EO13:EO15"/>
+    <mergeCell ref="EP13:EP15"/>
+    <mergeCell ref="EQ13:EQ15"/>
+    <mergeCell ref="EH13:EH15"/>
+    <mergeCell ref="EI13:EI15"/>
+    <mergeCell ref="EJ13:EJ15"/>
+    <mergeCell ref="EK13:EK15"/>
+    <mergeCell ref="EL13:EL15"/>
+    <mergeCell ref="EM13:EM15"/>
+    <mergeCell ref="EN13:EN15"/>
+    <mergeCell ref="CB13:CB15"/>
+    <mergeCell ref="CC13:CC15"/>
+    <mergeCell ref="CK13:CK15"/>
+    <mergeCell ref="DJ11:DL11"/>
+    <mergeCell ref="CL13:CL15"/>
+    <mergeCell ref="CM13:CM15"/>
+    <mergeCell ref="CN13:CN15"/>
+    <mergeCell ref="CO13:CO15"/>
+    <mergeCell ref="CD13:CD15"/>
+    <mergeCell ref="CE13:CE15"/>
+    <mergeCell ref="CF13:CF15"/>
+    <mergeCell ref="CG13:CG15"/>
+    <mergeCell ref="CH13:CH15"/>
+    <mergeCell ref="CI13:CI15"/>
+    <mergeCell ref="CJ13:CJ15"/>
+    <mergeCell ref="CZ11:CZ12"/>
+    <mergeCell ref="DA11:DC11"/>
+    <mergeCell ref="DD11:DF11"/>
+    <mergeCell ref="DG11:DI11"/>
+    <mergeCell ref="BY10:CA12"/>
+    <mergeCell ref="CD11:CD12"/>
+    <mergeCell ref="CE11:CE12"/>
+    <mergeCell ref="CF11:CF12"/>
+    <mergeCell ref="CG11:CG12"/>
+    <mergeCell ref="CH11:CH12"/>
+    <mergeCell ref="EN10:EP10"/>
+    <mergeCell ref="EN11:EN12"/>
+    <mergeCell ref="EO11:EO12"/>
+    <mergeCell ref="EP11:EP12"/>
+    <mergeCell ref="EF11:EF12"/>
+    <mergeCell ref="DR11:DR12"/>
+    <mergeCell ref="DS11:DS12"/>
+    <mergeCell ref="DT11:DT12"/>
+    <mergeCell ref="DU11:DU12"/>
+    <mergeCell ref="DV10:DV12"/>
+    <mergeCell ref="EA11:EA12"/>
+    <mergeCell ref="EB11:EB12"/>
+    <mergeCell ref="ED11:ED12"/>
+    <mergeCell ref="EE11:EE12"/>
+    <mergeCell ref="DR10:DU10"/>
+    <mergeCell ref="CP11:CP12"/>
+    <mergeCell ref="CQ11:CQ12"/>
+    <mergeCell ref="CY11:CY12"/>
+    <mergeCell ref="EQ11:EQ12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="AH11:AH12"/>
+    <mergeCell ref="AI11:AI12"/>
+    <mergeCell ref="AJ11:AJ12"/>
+    <mergeCell ref="AX11:AX12"/>
+    <mergeCell ref="AY11:AY12"/>
+    <mergeCell ref="BM11:BN11"/>
+    <mergeCell ref="BO11:BP11"/>
+    <mergeCell ref="CB11:CB12"/>
+    <mergeCell ref="CC11:CC12"/>
+    <mergeCell ref="CT11:CT12"/>
+    <mergeCell ref="CU11:CU12"/>
+    <mergeCell ref="CV11:CV12"/>
+    <mergeCell ref="CW11:CW12"/>
+    <mergeCell ref="CX11:CX12"/>
+    <mergeCell ref="DY11:DY12"/>
+    <mergeCell ref="DZ11:DZ12"/>
+    <mergeCell ref="AF11:AF12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="BJ10:BJ12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:AF10"/>
+    <mergeCell ref="AG10:AJ10"/>
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="V11:X11"/>
+    <mergeCell ref="Y11:AA11"/>
+    <mergeCell ref="AB11:AD11"/>
+    <mergeCell ref="AE11:AE12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="AP11:AP12"/>
+    <mergeCell ref="AQ11:AQ12"/>
+    <mergeCell ref="AS11:AS12"/>
+    <mergeCell ref="AT11:AT12"/>
+    <mergeCell ref="AU11:AU12"/>
+    <mergeCell ref="AV11:AV12"/>
+    <mergeCell ref="AK10:AK12"/>
+    <mergeCell ref="AL10:AL12"/>
+    <mergeCell ref="AM10:AM12"/>
+    <mergeCell ref="AN10:AQ10"/>
+    <mergeCell ref="AR10:AR12"/>
+    <mergeCell ref="AS10:AV10"/>
+    <mergeCell ref="AO11:AO12"/>
+    <mergeCell ref="BQ11:BR11"/>
+    <mergeCell ref="BS11:BT11"/>
+    <mergeCell ref="BU11:BV11"/>
+    <mergeCell ref="BW11:BX11"/>
+    <mergeCell ref="BK10:BK12"/>
+    <mergeCell ref="BL10:BL12"/>
+    <mergeCell ref="BM10:BR10"/>
+    <mergeCell ref="BS10:BX10"/>
+    <mergeCell ref="DQ11:DQ12"/>
+    <mergeCell ref="CR11:CR12"/>
+    <mergeCell ref="CS11:CS12"/>
+    <mergeCell ref="CB10:CD10"/>
+    <mergeCell ref="CE10:CM10"/>
+    <mergeCell ref="CN10:CO10"/>
+    <mergeCell ref="CP10:CR10"/>
+    <mergeCell ref="CS10:DQ10"/>
+    <mergeCell ref="DP11:DP12"/>
+    <mergeCell ref="CI11:CI12"/>
+    <mergeCell ref="CJ11:CJ12"/>
+    <mergeCell ref="CK11:CK12"/>
+    <mergeCell ref="CL11:CL12"/>
+    <mergeCell ref="CM11:CM12"/>
+    <mergeCell ref="CN11:CN12"/>
+    <mergeCell ref="CO11:CO12"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="EM10:EM12"/>
@@ -3698,191 +3900,8 @@
     <mergeCell ref="ED10:EG10"/>
     <mergeCell ref="EH10:EH12"/>
     <mergeCell ref="DM11:DO11"/>
-    <mergeCell ref="BQ11:BR11"/>
-    <mergeCell ref="BS11:BT11"/>
-    <mergeCell ref="BU11:BV11"/>
-    <mergeCell ref="BW11:BX11"/>
-    <mergeCell ref="BK10:BK12"/>
-    <mergeCell ref="BL10:BL12"/>
-    <mergeCell ref="BM10:BR10"/>
-    <mergeCell ref="BS10:BX10"/>
-    <mergeCell ref="DQ11:DQ12"/>
-    <mergeCell ref="CR11:CR12"/>
-    <mergeCell ref="CS11:CS12"/>
-    <mergeCell ref="CB10:CD10"/>
-    <mergeCell ref="CE10:CM10"/>
-    <mergeCell ref="CN10:CO10"/>
-    <mergeCell ref="CP10:CR10"/>
-    <mergeCell ref="CS10:DQ10"/>
-    <mergeCell ref="DP11:DP12"/>
-    <mergeCell ref="CI11:CI12"/>
-    <mergeCell ref="CJ11:CJ12"/>
-    <mergeCell ref="CK11:CK12"/>
-    <mergeCell ref="CL11:CL12"/>
-    <mergeCell ref="CM11:CM12"/>
-    <mergeCell ref="CN11:CN12"/>
-    <mergeCell ref="CO11:CO12"/>
-    <mergeCell ref="AP11:AP12"/>
-    <mergeCell ref="AQ11:AQ12"/>
-    <mergeCell ref="AS11:AS12"/>
-    <mergeCell ref="AT11:AT12"/>
-    <mergeCell ref="AU11:AU12"/>
-    <mergeCell ref="AV11:AV12"/>
-    <mergeCell ref="AK10:AK12"/>
-    <mergeCell ref="AL10:AL12"/>
-    <mergeCell ref="AM10:AM12"/>
-    <mergeCell ref="AN10:AQ10"/>
-    <mergeCell ref="AR10:AR12"/>
-    <mergeCell ref="AS10:AV10"/>
-    <mergeCell ref="AO11:AO12"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:AF10"/>
-    <mergeCell ref="AG10:AJ10"/>
-    <mergeCell ref="AN11:AN12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="S11:U11"/>
-    <mergeCell ref="V11:X11"/>
-    <mergeCell ref="Y11:AA11"/>
-    <mergeCell ref="AB11:AD11"/>
-    <mergeCell ref="AE11:AE12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="EQ11:EQ12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="AG11:AG12"/>
-    <mergeCell ref="AH11:AH12"/>
-    <mergeCell ref="AI11:AI12"/>
-    <mergeCell ref="AJ11:AJ12"/>
-    <mergeCell ref="AX11:AX12"/>
-    <mergeCell ref="AY11:AY12"/>
-    <mergeCell ref="BM11:BN11"/>
-    <mergeCell ref="BO11:BP11"/>
-    <mergeCell ref="CB11:CB12"/>
-    <mergeCell ref="CC11:CC12"/>
-    <mergeCell ref="CT11:CT12"/>
-    <mergeCell ref="CU11:CU12"/>
-    <mergeCell ref="CV11:CV12"/>
-    <mergeCell ref="CW11:CW12"/>
-    <mergeCell ref="CX11:CX12"/>
-    <mergeCell ref="DY11:DY12"/>
-    <mergeCell ref="DZ11:DZ12"/>
-    <mergeCell ref="AF11:AF12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="BJ10:BJ12"/>
-    <mergeCell ref="BY10:CA12"/>
-    <mergeCell ref="CD11:CD12"/>
-    <mergeCell ref="CE11:CE12"/>
-    <mergeCell ref="CF11:CF12"/>
-    <mergeCell ref="CG11:CG12"/>
-    <mergeCell ref="CH11:CH12"/>
-    <mergeCell ref="EN10:EP10"/>
-    <mergeCell ref="EN11:EN12"/>
-    <mergeCell ref="EO11:EO12"/>
-    <mergeCell ref="EP11:EP12"/>
-    <mergeCell ref="EF11:EF12"/>
-    <mergeCell ref="DR11:DR12"/>
-    <mergeCell ref="DS11:DS12"/>
-    <mergeCell ref="DT11:DT12"/>
-    <mergeCell ref="DU11:DU12"/>
-    <mergeCell ref="DV10:DV12"/>
-    <mergeCell ref="EA11:EA12"/>
-    <mergeCell ref="EB11:EB12"/>
-    <mergeCell ref="ED11:ED12"/>
-    <mergeCell ref="EE11:EE12"/>
-    <mergeCell ref="DR10:DU10"/>
-    <mergeCell ref="CP11:CP12"/>
-    <mergeCell ref="CQ11:CQ12"/>
-    <mergeCell ref="CY11:CY12"/>
-    <mergeCell ref="CB13:CB15"/>
-    <mergeCell ref="CC13:CC15"/>
-    <mergeCell ref="CK13:CK15"/>
-    <mergeCell ref="DJ11:DL11"/>
-    <mergeCell ref="CL13:CL15"/>
-    <mergeCell ref="CM13:CM15"/>
-    <mergeCell ref="CN13:CN15"/>
-    <mergeCell ref="CO13:CO15"/>
-    <mergeCell ref="CD13:CD15"/>
-    <mergeCell ref="CE13:CE15"/>
-    <mergeCell ref="CF13:CF15"/>
-    <mergeCell ref="CG13:CG15"/>
-    <mergeCell ref="CH13:CH15"/>
-    <mergeCell ref="CI13:CI15"/>
-    <mergeCell ref="CJ13:CJ15"/>
-    <mergeCell ref="CZ11:CZ12"/>
-    <mergeCell ref="DA11:DC11"/>
-    <mergeCell ref="DD11:DF11"/>
-    <mergeCell ref="DG11:DI11"/>
-    <mergeCell ref="EF13:EF15"/>
-    <mergeCell ref="EG13:EG15"/>
-    <mergeCell ref="EO13:EO15"/>
-    <mergeCell ref="EP13:EP15"/>
-    <mergeCell ref="EQ13:EQ15"/>
-    <mergeCell ref="EH13:EH15"/>
-    <mergeCell ref="EI13:EI15"/>
-    <mergeCell ref="EJ13:EJ15"/>
-    <mergeCell ref="EK13:EK15"/>
-    <mergeCell ref="EL13:EL15"/>
-    <mergeCell ref="EM13:EM15"/>
-    <mergeCell ref="EN13:EN15"/>
-    <mergeCell ref="EB13:EB15"/>
-    <mergeCell ref="EC13:EC15"/>
-    <mergeCell ref="AK13:AK15"/>
-    <mergeCell ref="AL13:AL15"/>
-    <mergeCell ref="AM13:AM15"/>
-    <mergeCell ref="AN13:AN15"/>
-    <mergeCell ref="AO13:AO15"/>
-    <mergeCell ref="ED13:ED15"/>
-    <mergeCell ref="EE13:EE15"/>
-    <mergeCell ref="AP13:AP15"/>
-    <mergeCell ref="AQ13:AQ15"/>
-    <mergeCell ref="AR13:AR15"/>
-    <mergeCell ref="AS13:AS15"/>
-    <mergeCell ref="AT13:AT15"/>
-    <mergeCell ref="AU13:AU15"/>
-    <mergeCell ref="AV13:AV15"/>
-    <mergeCell ref="AW13:AW15"/>
-    <mergeCell ref="AX13:AX15"/>
-    <mergeCell ref="AY13:AY15"/>
-    <mergeCell ref="AZ13:AZ15"/>
-    <mergeCell ref="BA13:BA15"/>
-    <mergeCell ref="BB13:BB15"/>
-    <mergeCell ref="BY13:BY15"/>
-    <mergeCell ref="BZ13:BZ15"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="DV13:DV15"/>
-    <mergeCell ref="DW13:DW15"/>
-    <mergeCell ref="DX13:DX15"/>
-    <mergeCell ref="DY13:DY15"/>
-    <mergeCell ref="DZ13:DZ15"/>
-    <mergeCell ref="EA13:EA15"/>
-    <mergeCell ref="BK13:BK15"/>
-    <mergeCell ref="BL13:BL15"/>
-    <mergeCell ref="BM13:BM15"/>
-    <mergeCell ref="BN13:BN15"/>
-    <mergeCell ref="BO13:BO15"/>
-    <mergeCell ref="BP13:BP15"/>
-    <mergeCell ref="BQ13:BQ15"/>
-    <mergeCell ref="BR13:BR15"/>
-    <mergeCell ref="BS13:BS15"/>
-    <mergeCell ref="BT13:BT15"/>
-    <mergeCell ref="BU13:BU15"/>
-    <mergeCell ref="BV13:BV15"/>
-    <mergeCell ref="BW13:BW15"/>
-    <mergeCell ref="BX13:BX15"/>
-    <mergeCell ref="CA13:CA15"/>
   </mergeCells>
-  <phoneticPr fontId="14" type="noConversion"/>
+  <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>